<commit_message>
Set A1b tables to A4 portrait layout
</commit_message>
<xml_diff>
--- a/assignments/assA1.xlsx
+++ b/assignments/assA1.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Desktop\Design-of-Enterprise-IoT-design\assignments\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B983879B-596C-44C0-971C-95E5D066BEF3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{355F1CFF-082A-47A6-AED5-C914DDC393CD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="760" yWindow="760" windowWidth="19200" windowHeight="9970" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="380" yWindow="380" windowWidth="19200" windowHeight="9970" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Value Proposition" sheetId="1" r:id="rId1"/>
@@ -47,7 +47,6 @@
         <color rgb="FF202020"/>
         <rFont val="宋体-简"/>
         <family val="1"/>
-        <charset val="134"/>
       </rPr>
       <t xml:space="preserve">People: </t>
     </r>
@@ -57,7 +56,6 @@
         <sz val="11"/>
         <rFont val="宋体-简"/>
         <family val="1"/>
-        <charset val="134"/>
       </rPr>
       <t>养殖管理人员，设备维护人员</t>
     </r>
@@ -1693,7 +1691,6 @@
       <color rgb="FF202020"/>
       <name val="宋体-简"/>
       <family val="1"/>
-      <charset val="134"/>
     </font>
     <font>
       <sz val="10"/>
@@ -1856,7 +1853,6 @@
       <sz val="11"/>
       <name val="宋体-简"/>
       <family val="1"/>
-      <charset val="134"/>
     </font>
     <font>
       <b/>
@@ -2055,13 +2051,13 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.79995117038483843"/>
+        <fgColor theme="4" tint="0.79989013336588644"/>
         <bgColor indexed="65"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.59996337778862885"/>
+        <fgColor theme="4" tint="0.59990234076967686"/>
         <bgColor indexed="65"/>
       </patternFill>
     </fill>
@@ -2078,13 +2074,13 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.79995117038483843"/>
+        <fgColor theme="5" tint="0.79989013336588644"/>
         <bgColor indexed="65"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.59996337778862885"/>
+        <fgColor theme="5" tint="0.59990234076967686"/>
         <bgColor indexed="65"/>
       </patternFill>
     </fill>
@@ -2101,13 +2097,13 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.79995117038483843"/>
+        <fgColor theme="6" tint="0.79989013336588644"/>
         <bgColor indexed="65"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.59996337778862885"/>
+        <fgColor theme="6" tint="0.59990234076967686"/>
         <bgColor indexed="65"/>
       </patternFill>
     </fill>
@@ -2124,13 +2120,13 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.79995117038483843"/>
+        <fgColor theme="7" tint="0.79989013336588644"/>
         <bgColor indexed="65"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.59996337778862885"/>
+        <fgColor theme="7" tint="0.59990234076967686"/>
         <bgColor indexed="65"/>
       </patternFill>
     </fill>
@@ -2147,13 +2143,13 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.79995117038483843"/>
+        <fgColor theme="8" tint="0.79989013336588644"/>
         <bgColor indexed="65"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.59996337778862885"/>
+        <fgColor theme="8" tint="0.59990234076967686"/>
         <bgColor indexed="65"/>
       </patternFill>
     </fill>
@@ -2170,13 +2166,13 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.79995117038483843"/>
+        <fgColor theme="9" tint="0.79989013336588644"/>
         <bgColor indexed="65"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.59996337778862885"/>
+        <fgColor theme="9" tint="0.59990234076967686"/>
         <bgColor indexed="65"/>
       </patternFill>
     </fill>
@@ -2229,7 +2225,7 @@
       <right/>
       <top/>
       <bottom style="medium">
-        <color theme="4" tint="0.49995422223578601"/>
+        <color theme="4" tint="0.49989318521683401"/>
       </bottom>
       <diagonal/>
     </border>
@@ -2763,55 +2759,55 @@
     </xf>
   </cellXfs>
   <cellStyles count="49">
-    <cellStyle name="20% - 强调文字颜色 1" xfId="26" xr:uid="{00000000-0005-0000-0000-00001A000000}"/>
-    <cellStyle name="20% - 强调文字颜色 2" xfId="30" xr:uid="{00000000-0005-0000-0000-00001E000000}"/>
-    <cellStyle name="20% - 强调文字颜色 3" xfId="34" xr:uid="{00000000-0005-0000-0000-000022000000}"/>
-    <cellStyle name="20% - 强调文字颜色 4" xfId="38" xr:uid="{00000000-0005-0000-0000-000026000000}"/>
-    <cellStyle name="20% - 强调文字颜色 5" xfId="42" xr:uid="{00000000-0005-0000-0000-00002A000000}"/>
-    <cellStyle name="20% - 强调文字颜色 6" xfId="46" xr:uid="{00000000-0005-0000-0000-00002E000000}"/>
-    <cellStyle name="40% - 强调文字颜色 1" xfId="27" xr:uid="{00000000-0005-0000-0000-00001B000000}"/>
-    <cellStyle name="40% - 强调文字颜色 2" xfId="31" xr:uid="{00000000-0005-0000-0000-00001F000000}"/>
-    <cellStyle name="40% - 强调文字颜色 3" xfId="35" xr:uid="{00000000-0005-0000-0000-000023000000}"/>
-    <cellStyle name="40% - 强调文字颜色 4" xfId="39" xr:uid="{00000000-0005-0000-0000-000027000000}"/>
-    <cellStyle name="40% - 强调文字颜色 5" xfId="43" xr:uid="{00000000-0005-0000-0000-00002B000000}"/>
-    <cellStyle name="40% - 强调文字颜色 6" xfId="47" xr:uid="{00000000-0005-0000-0000-00002F000000}"/>
-    <cellStyle name="60% - 强调文字颜色 1" xfId="28" xr:uid="{00000000-0005-0000-0000-00001C000000}"/>
-    <cellStyle name="60% - 强调文字颜色 2" xfId="32" xr:uid="{00000000-0005-0000-0000-000020000000}"/>
-    <cellStyle name="60% - 强调文字颜色 3" xfId="36" xr:uid="{00000000-0005-0000-0000-000024000000}"/>
-    <cellStyle name="60% - 强调文字颜色 4" xfId="40" xr:uid="{00000000-0005-0000-0000-000028000000}"/>
-    <cellStyle name="60% - 强调文字颜色 5" xfId="44" xr:uid="{00000000-0005-0000-0000-00002C000000}"/>
-    <cellStyle name="60% - 强调文字颜色 6" xfId="48" xr:uid="{00000000-0005-0000-0000-000030000000}"/>
-    <cellStyle name="千位分隔" xfId="1" xr:uid="{00000000-0005-0000-0000-000001000000}"/>
-    <cellStyle name="千位分隔[0]" xfId="4" xr:uid="{00000000-0005-0000-0000-000004000000}"/>
-    <cellStyle name="好" xfId="22" xr:uid="{00000000-0005-0000-0000-000016000000}"/>
-    <cellStyle name="差" xfId="23" xr:uid="{00000000-0005-0000-0000-000017000000}"/>
-    <cellStyle name="已访问的超链接" xfId="7" xr:uid="{00000000-0005-0000-0000-000007000000}"/>
+    <cellStyle name="20% - 强调文字颜色 1" xfId="26" xr:uid="{00000000-0005-0000-0000-000000000000}"/>
+    <cellStyle name="20% - 强调文字颜色 2" xfId="30" xr:uid="{00000000-0005-0000-0000-000001000000}"/>
+    <cellStyle name="20% - 强调文字颜色 3" xfId="34" xr:uid="{00000000-0005-0000-0000-000002000000}"/>
+    <cellStyle name="20% - 强调文字颜色 4" xfId="38" xr:uid="{00000000-0005-0000-0000-000003000000}"/>
+    <cellStyle name="20% - 强调文字颜色 5" xfId="42" xr:uid="{00000000-0005-0000-0000-000004000000}"/>
+    <cellStyle name="20% - 强调文字颜色 6" xfId="46" xr:uid="{00000000-0005-0000-0000-000005000000}"/>
+    <cellStyle name="40% - 强调文字颜色 1" xfId="27" xr:uid="{00000000-0005-0000-0000-000006000000}"/>
+    <cellStyle name="40% - 强调文字颜色 2" xfId="31" xr:uid="{00000000-0005-0000-0000-000007000000}"/>
+    <cellStyle name="40% - 强调文字颜色 3" xfId="35" xr:uid="{00000000-0005-0000-0000-000008000000}"/>
+    <cellStyle name="40% - 强调文字颜色 4" xfId="39" xr:uid="{00000000-0005-0000-0000-000009000000}"/>
+    <cellStyle name="40% - 强调文字颜色 5" xfId="43" xr:uid="{00000000-0005-0000-0000-00000A000000}"/>
+    <cellStyle name="40% - 强调文字颜色 6" xfId="47" xr:uid="{00000000-0005-0000-0000-00000B000000}"/>
+    <cellStyle name="60% - 强调文字颜色 1" xfId="28" xr:uid="{00000000-0005-0000-0000-00000C000000}"/>
+    <cellStyle name="60% - 强调文字颜色 2" xfId="32" xr:uid="{00000000-0005-0000-0000-00000D000000}"/>
+    <cellStyle name="60% - 强调文字颜色 3" xfId="36" xr:uid="{00000000-0005-0000-0000-00000E000000}"/>
+    <cellStyle name="60% - 强调文字颜色 4" xfId="40" xr:uid="{00000000-0005-0000-0000-00000F000000}"/>
+    <cellStyle name="60% - 强调文字颜色 5" xfId="44" xr:uid="{00000000-0005-0000-0000-000010000000}"/>
+    <cellStyle name="60% - 强调文字颜色 6" xfId="48" xr:uid="{00000000-0005-0000-0000-000011000000}"/>
+    <cellStyle name="千位分隔" xfId="1" xr:uid="{00000000-0005-0000-0000-000012000000}"/>
+    <cellStyle name="千位分隔[0]" xfId="4" xr:uid="{00000000-0005-0000-0000-000013000000}"/>
+    <cellStyle name="好" xfId="22" xr:uid="{00000000-0005-0000-0000-000014000000}"/>
+    <cellStyle name="差" xfId="23" xr:uid="{00000000-0005-0000-0000-000015000000}"/>
+    <cellStyle name="已访问的超链接" xfId="7" xr:uid="{00000000-0005-0000-0000-000016000000}"/>
     <cellStyle name="常规" xfId="0" builtinId="0"/>
-    <cellStyle name="强调文字颜色 1" xfId="25" xr:uid="{00000000-0005-0000-0000-000019000000}"/>
-    <cellStyle name="强调文字颜色 2" xfId="29" xr:uid="{00000000-0005-0000-0000-00001D000000}"/>
-    <cellStyle name="强调文字颜色 3" xfId="33" xr:uid="{00000000-0005-0000-0000-000021000000}"/>
-    <cellStyle name="强调文字颜色 4" xfId="37" xr:uid="{00000000-0005-0000-0000-000025000000}"/>
-    <cellStyle name="强调文字颜色 5" xfId="41" xr:uid="{00000000-0005-0000-0000-000029000000}"/>
-    <cellStyle name="强调文字颜色 6" xfId="45" xr:uid="{00000000-0005-0000-0000-00002D000000}"/>
-    <cellStyle name="标题" xfId="10" xr:uid="{00000000-0005-0000-0000-00000A000000}"/>
-    <cellStyle name="标题 1" xfId="12" xr:uid="{00000000-0005-0000-0000-00000C000000}"/>
-    <cellStyle name="标题 2" xfId="13" xr:uid="{00000000-0005-0000-0000-00000D000000}"/>
-    <cellStyle name="标题 3" xfId="14" xr:uid="{00000000-0005-0000-0000-00000E000000}"/>
-    <cellStyle name="标题 4" xfId="15" xr:uid="{00000000-0005-0000-0000-00000F000000}"/>
-    <cellStyle name="检查单元格" xfId="19" xr:uid="{00000000-0005-0000-0000-000013000000}"/>
-    <cellStyle name="汇总" xfId="21" xr:uid="{00000000-0005-0000-0000-000015000000}"/>
-    <cellStyle name="注释" xfId="8" xr:uid="{00000000-0005-0000-0000-000008000000}"/>
-    <cellStyle name="百分比" xfId="3" xr:uid="{00000000-0005-0000-0000-000003000000}"/>
-    <cellStyle name="解释性文本" xfId="11" xr:uid="{00000000-0005-0000-0000-00000B000000}"/>
-    <cellStyle name="警告文本" xfId="9" xr:uid="{00000000-0005-0000-0000-000009000000}"/>
-    <cellStyle name="计算" xfId="18" xr:uid="{00000000-0005-0000-0000-000012000000}"/>
-    <cellStyle name="货币" xfId="2" xr:uid="{00000000-0005-0000-0000-000002000000}"/>
-    <cellStyle name="货币[0]" xfId="5" xr:uid="{00000000-0005-0000-0000-000005000000}"/>
-    <cellStyle name="超链接" xfId="6" xr:uid="{00000000-0005-0000-0000-000006000000}"/>
-    <cellStyle name="输入" xfId="16" xr:uid="{00000000-0005-0000-0000-000010000000}"/>
-    <cellStyle name="输出" xfId="17" xr:uid="{00000000-0005-0000-0000-000011000000}"/>
-    <cellStyle name="适中" xfId="24" xr:uid="{00000000-0005-0000-0000-000018000000}"/>
-    <cellStyle name="链接单元格" xfId="20" xr:uid="{00000000-0005-0000-0000-000014000000}"/>
+    <cellStyle name="强调文字颜色 1" xfId="25" xr:uid="{00000000-0005-0000-0000-000018000000}"/>
+    <cellStyle name="强调文字颜色 2" xfId="29" xr:uid="{00000000-0005-0000-0000-000019000000}"/>
+    <cellStyle name="强调文字颜色 3" xfId="33" xr:uid="{00000000-0005-0000-0000-00001A000000}"/>
+    <cellStyle name="强调文字颜色 4" xfId="37" xr:uid="{00000000-0005-0000-0000-00001B000000}"/>
+    <cellStyle name="强调文字颜色 5" xfId="41" xr:uid="{00000000-0005-0000-0000-00001C000000}"/>
+    <cellStyle name="强调文字颜色 6" xfId="45" xr:uid="{00000000-0005-0000-0000-00001D000000}"/>
+    <cellStyle name="标题" xfId="10" xr:uid="{00000000-0005-0000-0000-00001E000000}"/>
+    <cellStyle name="标题 1" xfId="12" xr:uid="{00000000-0005-0000-0000-00001F000000}"/>
+    <cellStyle name="标题 2" xfId="13" xr:uid="{00000000-0005-0000-0000-000020000000}"/>
+    <cellStyle name="标题 3" xfId="14" xr:uid="{00000000-0005-0000-0000-000021000000}"/>
+    <cellStyle name="标题 4" xfId="15" xr:uid="{00000000-0005-0000-0000-000022000000}"/>
+    <cellStyle name="检查单元格" xfId="19" xr:uid="{00000000-0005-0000-0000-000023000000}"/>
+    <cellStyle name="汇总" xfId="21" xr:uid="{00000000-0005-0000-0000-000024000000}"/>
+    <cellStyle name="注释" xfId="8" xr:uid="{00000000-0005-0000-0000-000025000000}"/>
+    <cellStyle name="百分比" xfId="3" xr:uid="{00000000-0005-0000-0000-000026000000}"/>
+    <cellStyle name="解释性文本" xfId="11" xr:uid="{00000000-0005-0000-0000-000027000000}"/>
+    <cellStyle name="警告文本" xfId="9" xr:uid="{00000000-0005-0000-0000-000028000000}"/>
+    <cellStyle name="计算" xfId="18" xr:uid="{00000000-0005-0000-0000-000029000000}"/>
+    <cellStyle name="货币" xfId="2" xr:uid="{00000000-0005-0000-0000-00002A000000}"/>
+    <cellStyle name="货币[0]" xfId="5" xr:uid="{00000000-0005-0000-0000-00002B000000}"/>
+    <cellStyle name="超链接" xfId="6" xr:uid="{00000000-0005-0000-0000-00002C000000}"/>
+    <cellStyle name="输入" xfId="16" xr:uid="{00000000-0005-0000-0000-00002D000000}"/>
+    <cellStyle name="输出" xfId="17" xr:uid="{00000000-0005-0000-0000-00002E000000}"/>
+    <cellStyle name="适中" xfId="24" xr:uid="{00000000-0005-0000-0000-00002F000000}"/>
+    <cellStyle name="链接单元格" xfId="20" xr:uid="{00000000-0005-0000-0000-000030000000}"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -3051,7 +3047,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="4" spans="1:2" s="1" customFormat="1" ht="14.5">
+    <row r="4" spans="1:2" s="1" customFormat="1">
       <c r="A4" s="4" t="s">
         <v>4</v>
       </c>
@@ -3059,7 +3055,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="5" spans="1:2" s="1" customFormat="1" ht="14.5">
+    <row r="5" spans="1:2" s="1" customFormat="1">
       <c r="A5" s="4" t="s">
         <v>6</v>
       </c>
@@ -3067,7 +3063,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="6" spans="1:2" s="1" customFormat="1" ht="14.5">
+    <row r="6" spans="1:2" s="1" customFormat="1">
       <c r="A6" s="5" t="s">
         <v>8</v>
       </c>
@@ -3075,7 +3071,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="7" spans="1:2" s="1" customFormat="1" ht="29">
+    <row r="7" spans="1:2" s="1" customFormat="1" ht="28">
       <c r="A7" s="5" t="s">
         <v>10</v>
       </c>
@@ -3099,7 +3095,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="10" spans="1:2" s="1" customFormat="1" ht="29">
+    <row r="10" spans="1:2" s="1" customFormat="1" ht="28">
       <c r="A10" s="8" t="s">
         <v>16</v>
       </c>
@@ -3107,7 +3103,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="11" spans="1:2" s="1" customFormat="1" ht="29">
+    <row r="11" spans="1:2" s="1" customFormat="1" ht="28">
       <c r="A11" s="8" t="s">
         <v>18</v>
       </c>
@@ -3115,7 +3111,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="12" spans="1:2" s="1" customFormat="1" ht="43.5">
+    <row r="12" spans="1:2" s="1" customFormat="1" ht="42">
       <c r="A12" s="8" t="s">
         <v>20</v>
       </c>
@@ -3123,7 +3119,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="13" spans="1:2" s="1" customFormat="1" ht="29">
+    <row r="13" spans="1:2" s="1" customFormat="1" ht="28">
       <c r="A13" s="8" t="s">
         <v>22</v>
       </c>
@@ -3145,7 +3141,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="16" spans="1:2" s="1" customFormat="1" ht="29">
+    <row r="16" spans="1:2" s="1" customFormat="1" ht="28">
       <c r="A16" s="8" t="s">
         <v>27</v>
       </c>
@@ -3153,7 +3149,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="17" spans="1:2" s="1" customFormat="1" ht="29">
+    <row r="17" spans="1:2" s="1" customFormat="1" ht="28">
       <c r="A17" s="8" t="s">
         <v>29</v>
       </c>
@@ -3161,7 +3157,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="18" spans="1:2" s="1" customFormat="1" ht="29">
+    <row r="18" spans="1:2" s="1" customFormat="1" ht="28">
       <c r="A18" s="8" t="s">
         <v>31</v>
       </c>
@@ -3169,7 +3165,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="19" spans="1:2" s="1" customFormat="1" ht="29">
+    <row r="19" spans="1:2" s="1" customFormat="1" ht="28">
       <c r="A19" s="8" t="s">
         <v>33</v>
       </c>
@@ -3388,12 +3384,12 @@
   <dimension ref="A1:G15"/>
   <sheetFormatPr defaultColWidth="9.1640625" defaultRowHeight="14"/>
   <cols>
-    <col min="1" max="1" width="24" customWidth="1"/>
-    <col min="2" max="2" width="11" customWidth="1"/>
-    <col min="3" max="4" width="21" customWidth="1"/>
-    <col min="5" max="5" width="47" customWidth="1"/>
-    <col min="6" max="6" width="36" customWidth="1"/>
-    <col min="7" max="7" width="42" customWidth="1"/>
+    <col min="1" max="1" width="18" customWidth="1"/>
+    <col min="2" max="2" width="9" customWidth="1"/>
+    <col min="3" max="4" width="16" customWidth="1"/>
+    <col min="5" max="5" width="30" customWidth="1"/>
+    <col min="6" max="6" width="24" customWidth="1"/>
+    <col min="7" max="7" width="27" customWidth="1"/>
     <col min="8" max="16384" width="9.1640625" style="1"/>
   </cols>
   <sheetData>
@@ -3420,7 +3416,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="2" spans="1:7" ht="62" customHeight="1">
+    <row r="2" spans="1:7" ht="80" customHeight="1">
       <c r="A2" s="26" t="s">
         <v>80</v>
       </c>
@@ -3443,7 +3439,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="3" spans="1:7" ht="96" customHeight="1">
+    <row r="3" spans="1:7" ht="150" customHeight="1">
       <c r="A3" s="24" t="s">
         <v>117</v>
       </c>
@@ -3466,7 +3462,7 @@
         <v>123</v>
       </c>
     </row>
-    <row r="4" spans="1:7" ht="96" customHeight="1">
+    <row r="4" spans="1:7" ht="150" customHeight="1">
       <c r="A4" s="24" t="s">
         <v>124</v>
       </c>
@@ -3489,7 +3485,7 @@
         <v>128</v>
       </c>
     </row>
-    <row r="5" spans="1:7" ht="96" customHeight="1">
+    <row r="5" spans="1:7" ht="150" customHeight="1">
       <c r="A5" s="24" t="s">
         <v>129</v>
       </c>
@@ -3512,7 +3508,7 @@
         <v>133</v>
       </c>
     </row>
-    <row r="6" spans="1:7" ht="96" customHeight="1">
+    <row r="6" spans="1:7" ht="150" customHeight="1">
       <c r="A6" s="24" t="s">
         <v>134</v>
       </c>
@@ -3535,7 +3531,7 @@
         <v>138</v>
       </c>
     </row>
-    <row r="7" spans="1:7" ht="96" customHeight="1">
+    <row r="7" spans="1:7" ht="150" customHeight="1">
       <c r="A7" s="24" t="s">
         <v>139</v>
       </c>
@@ -3558,7 +3554,7 @@
         <v>143</v>
       </c>
     </row>
-    <row r="8" spans="1:7" ht="96" customHeight="1">
+    <row r="8" spans="1:7" ht="150" customHeight="1">
       <c r="A8" s="24" t="s">
         <v>144</v>
       </c>
@@ -3581,7 +3577,7 @@
         <v>149</v>
       </c>
     </row>
-    <row r="9" spans="1:7" ht="96" customHeight="1">
+    <row r="9" spans="1:7" ht="150" customHeight="1">
       <c r="A9" s="24" t="s">
         <v>150</v>
       </c>
@@ -3604,7 +3600,7 @@
         <v>155</v>
       </c>
     </row>
-    <row r="10" spans="1:7" ht="96" customHeight="1">
+    <row r="10" spans="1:7" ht="150" customHeight="1">
       <c r="A10" s="24" t="s">
         <v>156</v>
       </c>
@@ -3627,7 +3623,7 @@
         <v>161</v>
       </c>
     </row>
-    <row r="11" spans="1:7" ht="96" customHeight="1">
+    <row r="11" spans="1:7" ht="150" customHeight="1">
       <c r="A11" s="24" t="s">
         <v>162</v>
       </c>
@@ -3650,7 +3646,7 @@
         <v>167</v>
       </c>
     </row>
-    <row r="12" spans="1:7" ht="96" customHeight="1">
+    <row r="12" spans="1:7" ht="150" customHeight="1">
       <c r="A12" s="24" t="s">
         <v>168</v>
       </c>
@@ -3673,7 +3669,7 @@
         <v>173</v>
       </c>
     </row>
-    <row r="13" spans="1:7" ht="96" customHeight="1">
+    <row r="13" spans="1:7" ht="150" customHeight="1">
       <c r="A13" s="24" t="s">
         <v>174</v>
       </c>
@@ -3696,7 +3692,7 @@
         <v>179</v>
       </c>
     </row>
-    <row r="14" spans="1:7" ht="96" customHeight="1">
+    <row r="14" spans="1:7" ht="150" customHeight="1">
       <c r="A14" s="24" t="s">
         <v>180</v>
       </c>
@@ -3719,7 +3715,7 @@
         <v>186</v>
       </c>
     </row>
-    <row r="15" spans="1:7" ht="96" customHeight="1">
+    <row r="15" spans="1:7" ht="150" customHeight="1">
       <c r="A15" s="24" t="s">
         <v>187</v>
       </c>
@@ -3746,7 +3742,7 @@
   <phoneticPr fontId="68" type="noConversion"/>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.22" right="0.22" top="0.25" bottom="0.25" header="0" footer="0"/>
-  <pageSetup paperSize="9" scale="65" fitToHeight="2" orientation="landscape" horizontalDpi="1200" verticalDpi="1200" r:id="rId1"/>
+  <pageSetup paperSize="9" scale="66" fitToHeight="4" orientation="portrait" horizontalDpi="1200" verticalDpi="1200" r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -3758,13 +3754,13 @@
   <dimension ref="A1:D15"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="14"/>
   <cols>
-    <col min="1" max="1" width="28" style="1" customWidth="1"/>
-    <col min="2" max="2" width="32" customWidth="1"/>
-    <col min="3" max="3" width="50" customWidth="1"/>
-    <col min="4" max="4" width="78" customWidth="1"/>
+    <col min="1" max="1" width="23" style="1" customWidth="1"/>
+    <col min="2" max="2" width="25" customWidth="1"/>
+    <col min="3" max="3" width="37" customWidth="1"/>
+    <col min="4" max="4" width="50" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" ht="26.65" customHeight="1">
+    <row r="1" spans="1:4" ht="40" customHeight="1">
       <c r="A1" s="30" t="s">
         <v>87</v>
       </c>
@@ -3778,7 +3774,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="2" spans="1:4" ht="48" customHeight="1">
+    <row r="2" spans="1:4" ht="70" customHeight="1">
       <c r="A2" s="42" t="s">
         <v>193</v>
       </c>
@@ -3792,7 +3788,7 @@
         <v>194</v>
       </c>
     </row>
-    <row r="3" spans="1:4" ht="48" customHeight="1">
+    <row r="3" spans="1:4" ht="70" customHeight="1">
       <c r="A3" s="42"/>
       <c r="B3" s="43" t="s">
         <v>93</v>
@@ -3804,7 +3800,7 @@
         <v>195</v>
       </c>
     </row>
-    <row r="4" spans="1:4" ht="48" customHeight="1">
+    <row r="4" spans="1:4" ht="70" customHeight="1">
       <c r="A4" s="42"/>
       <c r="B4" s="43"/>
       <c r="C4" s="27" t="s">
@@ -3814,7 +3810,7 @@
         <v>196</v>
       </c>
     </row>
-    <row r="5" spans="1:4" ht="48" customHeight="1">
+    <row r="5" spans="1:4" ht="70" customHeight="1">
       <c r="A5" s="42"/>
       <c r="B5" s="43"/>
       <c r="C5" s="27" t="s">
@@ -3824,7 +3820,7 @@
         <v>197</v>
       </c>
     </row>
-    <row r="6" spans="1:4" ht="48" customHeight="1">
+    <row r="6" spans="1:4" ht="70" customHeight="1">
       <c r="A6" s="42"/>
       <c r="B6" s="43"/>
       <c r="C6" s="27" t="s">
@@ -3834,7 +3830,7 @@
         <v>198</v>
       </c>
     </row>
-    <row r="7" spans="1:4" ht="48" customHeight="1">
+    <row r="7" spans="1:4" ht="70" customHeight="1">
       <c r="A7" s="42"/>
       <c r="B7" s="43"/>
       <c r="C7" s="27" t="s">
@@ -3844,7 +3840,7 @@
         <v>199</v>
       </c>
     </row>
-    <row r="8" spans="1:4" ht="48" customHeight="1">
+    <row r="8" spans="1:4" ht="70" customHeight="1">
       <c r="A8" s="42"/>
       <c r="B8" s="43"/>
       <c r="C8" s="27" t="s">
@@ -3854,7 +3850,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="9" spans="1:4" ht="48" customHeight="1">
+    <row r="9" spans="1:4" ht="70" customHeight="1">
       <c r="A9" s="42"/>
       <c r="B9" s="43"/>
       <c r="C9" s="27" t="s">
@@ -3890,7 +3886,7 @@
   <phoneticPr fontId="68" type="noConversion"/>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.22" right="0.22" top="0.25" bottom="0.25" header="0" footer="0"/>
-  <pageSetup paperSize="9" scale="70" orientation="landscape" horizontalDpi="1200" verticalDpi="1200" r:id="rId1"/>
+  <pageSetup paperSize="9" scale="67" fitToHeight="2" orientation="portrait" horizontalDpi="1200" verticalDpi="1200" r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -3902,13 +3898,13 @@
   <dimension ref="A1:D30"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="14"/>
   <cols>
-    <col min="1" max="1" width="28" style="1" customWidth="1"/>
-    <col min="2" max="2" width="32" style="1" customWidth="1"/>
-    <col min="3" max="3" width="50" customWidth="1"/>
-    <col min="4" max="4" width="78" customWidth="1"/>
+    <col min="1" max="1" width="23" style="1" customWidth="1"/>
+    <col min="2" max="2" width="25" style="1" customWidth="1"/>
+    <col min="3" max="3" width="37" customWidth="1"/>
+    <col min="4" max="4" width="50" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" ht="26.65" customHeight="1">
+    <row r="1" spans="1:4" ht="40" customHeight="1">
       <c r="A1" s="35" t="s">
         <v>101</v>
       </c>
@@ -3922,7 +3918,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="2" spans="1:4" ht="48" customHeight="1">
+    <row r="2" spans="1:4" ht="70" customHeight="1">
       <c r="A2" s="44" t="s">
         <v>193</v>
       </c>
@@ -3936,7 +3932,7 @@
         <v>194</v>
       </c>
     </row>
-    <row r="3" spans="1:4" ht="48" customHeight="1">
+    <row r="3" spans="1:4" ht="70" customHeight="1">
       <c r="A3" s="45"/>
       <c r="B3" s="46" t="s">
         <v>93</v>
@@ -3948,7 +3944,7 @@
         <v>195</v>
       </c>
     </row>
-    <row r="4" spans="1:4" ht="48" customHeight="1">
+    <row r="4" spans="1:4" ht="70" customHeight="1">
       <c r="A4" s="45"/>
       <c r="B4" s="47"/>
       <c r="C4" s="31" t="s">
@@ -3958,7 +3954,7 @@
         <v>196</v>
       </c>
     </row>
-    <row r="5" spans="1:4" ht="48" customHeight="1">
+    <row r="5" spans="1:4" ht="70" customHeight="1">
       <c r="A5" s="45"/>
       <c r="B5" s="47"/>
       <c r="C5" s="31" t="s">
@@ -3968,7 +3964,7 @@
         <v>197</v>
       </c>
     </row>
-    <row r="6" spans="1:4" ht="48" customHeight="1">
+    <row r="6" spans="1:4" ht="70" customHeight="1">
       <c r="A6" s="45"/>
       <c r="B6" s="47"/>
       <c r="C6" s="31" t="s">
@@ -3978,7 +3974,7 @@
         <v>198</v>
       </c>
     </row>
-    <row r="7" spans="1:4" ht="48" customHeight="1">
+    <row r="7" spans="1:4" ht="70" customHeight="1">
       <c r="A7" s="45"/>
       <c r="B7" s="47"/>
       <c r="C7" s="31" t="s">
@@ -3988,7 +3984,7 @@
         <v>199</v>
       </c>
     </row>
-    <row r="8" spans="1:4" ht="48" customHeight="1">
+    <row r="8" spans="1:4" ht="70" customHeight="1">
       <c r="A8" s="45"/>
       <c r="B8" s="47"/>
       <c r="C8" s="31" t="s">
@@ -3998,7 +3994,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="9" spans="1:4" ht="48" customHeight="1">
+    <row r="9" spans="1:4" ht="70" customHeight="1">
       <c r="A9" s="45"/>
       <c r="B9" s="47"/>
       <c r="C9" s="31" t="s">
@@ -4008,7 +4004,7 @@
         <v>201</v>
       </c>
     </row>
-    <row r="10" spans="1:4" ht="48" customHeight="1">
+    <row r="10" spans="1:4" ht="70" customHeight="1">
       <c r="A10" s="48" t="s">
         <v>202</v>
       </c>
@@ -4022,7 +4018,7 @@
         <v>203</v>
       </c>
     </row>
-    <row r="11" spans="1:4" ht="48" customHeight="1">
+    <row r="11" spans="1:4" ht="70" customHeight="1">
       <c r="A11" s="49"/>
       <c r="B11" s="47"/>
       <c r="C11" s="31" t="s">
@@ -4032,7 +4028,7 @@
         <v>204</v>
       </c>
     </row>
-    <row r="12" spans="1:4" ht="48" customHeight="1">
+    <row r="12" spans="1:4" ht="70" customHeight="1">
       <c r="A12" s="49"/>
       <c r="B12" s="47"/>
       <c r="C12" s="31" t="s">
@@ -4042,7 +4038,7 @@
         <v>205</v>
       </c>
     </row>
-    <row r="13" spans="1:4" ht="48" customHeight="1">
+    <row r="13" spans="1:4" ht="70" customHeight="1">
       <c r="A13" s="49"/>
       <c r="B13" s="47"/>
       <c r="C13" s="31" t="s">
@@ -4052,7 +4048,7 @@
         <v>206</v>
       </c>
     </row>
-    <row r="14" spans="1:4" ht="48" customHeight="1">
+    <row r="14" spans="1:4" ht="70" customHeight="1">
       <c r="A14" s="49"/>
       <c r="B14" s="47"/>
       <c r="C14" s="31" t="s">
@@ -4062,7 +4058,7 @@
         <v>207</v>
       </c>
     </row>
-    <row r="15" spans="1:4" ht="48" customHeight="1">
+    <row r="15" spans="1:4" ht="70" customHeight="1">
       <c r="A15" s="49"/>
       <c r="B15" s="47"/>
       <c r="C15" s="31" t="s">
@@ -4072,7 +4068,7 @@
         <v>208</v>
       </c>
     </row>
-    <row r="16" spans="1:4" ht="48" customHeight="1">
+    <row r="16" spans="1:4" ht="70" customHeight="1">
       <c r="A16" s="50" t="s">
         <v>209</v>
       </c>
@@ -4086,7 +4082,7 @@
         <v>210</v>
       </c>
     </row>
-    <row r="17" spans="1:4" ht="48" customHeight="1">
+    <row r="17" spans="1:4" ht="70" customHeight="1">
       <c r="A17" s="51"/>
       <c r="B17" s="54"/>
       <c r="C17" s="31" t="s">
@@ -4096,7 +4092,7 @@
         <v>211</v>
       </c>
     </row>
-    <row r="18" spans="1:4" ht="48" customHeight="1">
+    <row r="18" spans="1:4" ht="70" customHeight="1">
       <c r="A18" s="51"/>
       <c r="B18" s="54"/>
       <c r="C18" s="31" t="s">
@@ -4106,7 +4102,7 @@
         <v>212</v>
       </c>
     </row>
-    <row r="19" spans="1:4" ht="48" customHeight="1">
+    <row r="19" spans="1:4" ht="70" customHeight="1">
       <c r="A19" s="51"/>
       <c r="B19" s="54"/>
       <c r="C19" s="31" t="s">
@@ -4116,7 +4112,7 @@
         <v>213</v>
       </c>
     </row>
-    <row r="20" spans="1:4" ht="48" customHeight="1">
+    <row r="20" spans="1:4" ht="70" customHeight="1">
       <c r="A20" s="52"/>
       <c r="B20" s="55"/>
       <c r="C20" s="34" t="s">
@@ -4158,6 +4154,6 @@
   <phoneticPr fontId="68" type="noConversion"/>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.22" right="0.22" top="0.25" bottom="0.25" header="0" footer="0"/>
-  <pageSetup paperSize="9" scale="70" fitToHeight="3" orientation="landscape" horizontalDpi="1200" verticalDpi="1200" r:id="rId1"/>
+  <pageSetup paperSize="9" scale="67" fitToHeight="4" orientation="portrait" horizontalDpi="1200" verticalDpi="1200" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Set task 4 Excel print area to one portrait page
</commit_message>
<xml_diff>
--- a/assignments/assA1.xlsx
+++ b/assignments/assA1.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Desktop\Design-of-Enterprise-IoT-design\assignments\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{355F1CFF-082A-47A6-AED5-C914DDC393CD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{93256251-3167-46DD-AE03-E6D9F7109D4E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="380" yWindow="380" windowWidth="19200" windowHeight="9970" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -4154,6 +4154,6 @@
   <phoneticPr fontId="68" type="noConversion"/>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.22" right="0.22" top="0.25" bottom="0.25" header="0" footer="0"/>
-  <pageSetup paperSize="9" scale="67" fitToHeight="4" orientation="portrait" horizontalDpi="1200" verticalDpi="1200" r:id="rId1"/>
+  <pageSetup paperSize="9" scale="67" orientation="portrait" horizontalDpi="1200" verticalDpi="1200" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto-fit A1b table row heights
</commit_message>
<xml_diff>
--- a/assignments/assA1.xlsx
+++ b/assignments/assA1.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Desktop\Design-of-Enterprise-IoT-design\assignments\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{93256251-3167-46DD-AE03-E6D9F7109D4E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B2774055-D53F-4FA9-BAAA-8BBC66693DF9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="380" yWindow="380" windowWidth="19200" windowHeight="9970" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -3393,7 +3393,7 @@
     <col min="8" max="16384" width="9.1640625" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" ht="28" customHeight="1">
+    <row r="1" spans="1:7">
       <c r="A1" s="25" t="s">
         <v>73</v>
       </c>
@@ -3416,7 +3416,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="2" spans="1:7" ht="80" customHeight="1">
+    <row r="2" spans="1:7" ht="48">
       <c r="A2" s="26" t="s">
         <v>80</v>
       </c>
@@ -3439,7 +3439,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="3" spans="1:7" ht="150" customHeight="1">
+    <row r="3" spans="1:7" ht="99" customHeight="1">
       <c r="A3" s="24" t="s">
         <v>117</v>
       </c>
@@ -3462,7 +3462,7 @@
         <v>123</v>
       </c>
     </row>
-    <row r="4" spans="1:7" ht="150" customHeight="1">
+    <row r="4" spans="1:7" ht="80" customHeight="1">
       <c r="A4" s="24" t="s">
         <v>124</v>
       </c>
@@ -3485,7 +3485,7 @@
         <v>128</v>
       </c>
     </row>
-    <row r="5" spans="1:7" ht="150" customHeight="1">
+    <row r="5" spans="1:7" ht="80" customHeight="1">
       <c r="A5" s="24" t="s">
         <v>129</v>
       </c>
@@ -3508,7 +3508,7 @@
         <v>133</v>
       </c>
     </row>
-    <row r="6" spans="1:7" ht="150" customHeight="1">
+    <row r="6" spans="1:7" ht="80" customHeight="1">
       <c r="A6" s="24" t="s">
         <v>134</v>
       </c>
@@ -3531,7 +3531,7 @@
         <v>138</v>
       </c>
     </row>
-    <row r="7" spans="1:7" ht="150" customHeight="1">
+    <row r="7" spans="1:7" ht="60" customHeight="1">
       <c r="A7" s="24" t="s">
         <v>139</v>
       </c>
@@ -3554,7 +3554,7 @@
         <v>143</v>
       </c>
     </row>
-    <row r="8" spans="1:7" ht="150" customHeight="1">
+    <row r="8" spans="1:7" ht="60" customHeight="1">
       <c r="A8" s="24" t="s">
         <v>144</v>
       </c>
@@ -3577,7 +3577,7 @@
         <v>149</v>
       </c>
     </row>
-    <row r="9" spans="1:7" ht="150" customHeight="1">
+    <row r="9" spans="1:7" ht="80" customHeight="1">
       <c r="A9" s="24" t="s">
         <v>150</v>
       </c>
@@ -3600,7 +3600,7 @@
         <v>155</v>
       </c>
     </row>
-    <row r="10" spans="1:7" ht="150" customHeight="1">
+    <row r="10" spans="1:7" ht="80" customHeight="1">
       <c r="A10" s="24" t="s">
         <v>156</v>
       </c>
@@ -3623,7 +3623,7 @@
         <v>161</v>
       </c>
     </row>
-    <row r="11" spans="1:7" ht="150" customHeight="1">
+    <row r="11" spans="1:7" ht="80" customHeight="1">
       <c r="A11" s="24" t="s">
         <v>162</v>
       </c>
@@ -3646,7 +3646,7 @@
         <v>167</v>
       </c>
     </row>
-    <row r="12" spans="1:7" ht="150" customHeight="1">
+    <row r="12" spans="1:7" ht="80" customHeight="1">
       <c r="A12" s="24" t="s">
         <v>168</v>
       </c>
@@ -3669,7 +3669,7 @@
         <v>173</v>
       </c>
     </row>
-    <row r="13" spans="1:7" ht="150" customHeight="1">
+    <row r="13" spans="1:7" ht="99" customHeight="1">
       <c r="A13" s="24" t="s">
         <v>174</v>
       </c>
@@ -3692,7 +3692,7 @@
         <v>179</v>
       </c>
     </row>
-    <row r="14" spans="1:7" ht="150" customHeight="1">
+    <row r="14" spans="1:7" ht="80" customHeight="1">
       <c r="A14" s="24" t="s">
         <v>180</v>
       </c>
@@ -3715,7 +3715,7 @@
         <v>186</v>
       </c>
     </row>
-    <row r="15" spans="1:7" ht="150" customHeight="1">
+    <row r="15" spans="1:7" ht="80" customHeight="1">
       <c r="A15" s="24" t="s">
         <v>187</v>
       </c>
@@ -3760,7 +3760,7 @@
     <col min="4" max="4" width="50" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" ht="40" customHeight="1">
+    <row r="1" spans="1:4" ht="23">
       <c r="A1" s="30" t="s">
         <v>87</v>
       </c>
@@ -3774,7 +3774,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="2" spans="1:4" ht="70" customHeight="1">
+    <row r="2" spans="1:4" ht="66">
       <c r="A2" s="42" t="s">
         <v>193</v>
       </c>
@@ -3788,7 +3788,7 @@
         <v>194</v>
       </c>
     </row>
-    <row r="3" spans="1:4" ht="70" customHeight="1">
+    <row r="3" spans="1:4" ht="55">
       <c r="A3" s="42"/>
       <c r="B3" s="43" t="s">
         <v>93</v>
@@ -3800,7 +3800,7 @@
         <v>195</v>
       </c>
     </row>
-    <row r="4" spans="1:4" ht="70" customHeight="1">
+    <row r="4" spans="1:4" ht="55">
       <c r="A4" s="42"/>
       <c r="B4" s="43"/>
       <c r="C4" s="27" t="s">
@@ -3810,7 +3810,7 @@
         <v>196</v>
       </c>
     </row>
-    <row r="5" spans="1:4" ht="70" customHeight="1">
+    <row r="5" spans="1:4" ht="44">
       <c r="A5" s="42"/>
       <c r="B5" s="43"/>
       <c r="C5" s="27" t="s">
@@ -3820,7 +3820,7 @@
         <v>197</v>
       </c>
     </row>
-    <row r="6" spans="1:4" ht="70" customHeight="1">
+    <row r="6" spans="1:4" ht="55">
       <c r="A6" s="42"/>
       <c r="B6" s="43"/>
       <c r="C6" s="27" t="s">
@@ -3830,7 +3830,7 @@
         <v>198</v>
       </c>
     </row>
-    <row r="7" spans="1:4" ht="70" customHeight="1">
+    <row r="7" spans="1:4" ht="77">
       <c r="A7" s="42"/>
       <c r="B7" s="43"/>
       <c r="C7" s="27" t="s">
@@ -3840,7 +3840,7 @@
         <v>199</v>
       </c>
     </row>
-    <row r="8" spans="1:4" ht="70" customHeight="1">
+    <row r="8" spans="1:4" ht="55">
       <c r="A8" s="42"/>
       <c r="B8" s="43"/>
       <c r="C8" s="27" t="s">
@@ -3850,7 +3850,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="9" spans="1:4" ht="70" customHeight="1">
+    <row r="9" spans="1:4" ht="66">
       <c r="A9" s="42"/>
       <c r="B9" s="43"/>
       <c r="C9" s="27" t="s">
@@ -3904,7 +3904,7 @@
     <col min="4" max="4" width="50" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" ht="40" customHeight="1">
+    <row r="1" spans="1:4" ht="46">
       <c r="A1" s="35" t="s">
         <v>101</v>
       </c>
@@ -3918,7 +3918,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="2" spans="1:4" ht="70" customHeight="1">
+    <row r="2" spans="1:4" ht="66">
       <c r="A2" s="44" t="s">
         <v>193</v>
       </c>
@@ -3932,7 +3932,7 @@
         <v>194</v>
       </c>
     </row>
-    <row r="3" spans="1:4" ht="70" customHeight="1">
+    <row r="3" spans="1:4" ht="55">
       <c r="A3" s="45"/>
       <c r="B3" s="46" t="s">
         <v>93</v>
@@ -3944,7 +3944,7 @@
         <v>195</v>
       </c>
     </row>
-    <row r="4" spans="1:4" ht="70" customHeight="1">
+    <row r="4" spans="1:4" ht="55">
       <c r="A4" s="45"/>
       <c r="B4" s="47"/>
       <c r="C4" s="31" t="s">
@@ -3954,7 +3954,7 @@
         <v>196</v>
       </c>
     </row>
-    <row r="5" spans="1:4" ht="70" customHeight="1">
+    <row r="5" spans="1:4" ht="44">
       <c r="A5" s="45"/>
       <c r="B5" s="47"/>
       <c r="C5" s="31" t="s">
@@ -3964,7 +3964,7 @@
         <v>197</v>
       </c>
     </row>
-    <row r="6" spans="1:4" ht="70" customHeight="1">
+    <row r="6" spans="1:4" ht="55">
       <c r="A6" s="45"/>
       <c r="B6" s="47"/>
       <c r="C6" s="31" t="s">
@@ -3974,7 +3974,7 @@
         <v>198</v>
       </c>
     </row>
-    <row r="7" spans="1:4" ht="70" customHeight="1">
+    <row r="7" spans="1:4" ht="77">
       <c r="A7" s="45"/>
       <c r="B7" s="47"/>
       <c r="C7" s="31" t="s">
@@ -3984,7 +3984,7 @@
         <v>199</v>
       </c>
     </row>
-    <row r="8" spans="1:4" ht="70" customHeight="1">
+    <row r="8" spans="1:4" ht="55">
       <c r="A8" s="45"/>
       <c r="B8" s="47"/>
       <c r="C8" s="31" t="s">
@@ -3994,7 +3994,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="9" spans="1:4" ht="70" customHeight="1">
+    <row r="9" spans="1:4" ht="66">
       <c r="A9" s="45"/>
       <c r="B9" s="47"/>
       <c r="C9" s="31" t="s">
@@ -4004,7 +4004,7 @@
         <v>201</v>
       </c>
     </row>
-    <row r="10" spans="1:4" ht="70" customHeight="1">
+    <row r="10" spans="1:4" ht="55">
       <c r="A10" s="48" t="s">
         <v>202</v>
       </c>
@@ -4018,7 +4018,7 @@
         <v>203</v>
       </c>
     </row>
-    <row r="11" spans="1:4" ht="70" customHeight="1">
+    <row r="11" spans="1:4" ht="55">
       <c r="A11" s="49"/>
       <c r="B11" s="47"/>
       <c r="C11" s="31" t="s">
@@ -4028,7 +4028,7 @@
         <v>204</v>
       </c>
     </row>
-    <row r="12" spans="1:4" ht="70" customHeight="1">
+    <row r="12" spans="1:4" ht="55">
       <c r="A12" s="49"/>
       <c r="B12" s="47"/>
       <c r="C12" s="31" t="s">
@@ -4038,7 +4038,7 @@
         <v>205</v>
       </c>
     </row>
-    <row r="13" spans="1:4" ht="70" customHeight="1">
+    <row r="13" spans="1:4" ht="55">
       <c r="A13" s="49"/>
       <c r="B13" s="47"/>
       <c r="C13" s="31" t="s">
@@ -4048,7 +4048,7 @@
         <v>206</v>
       </c>
     </row>
-    <row r="14" spans="1:4" ht="70" customHeight="1">
+    <row r="14" spans="1:4" ht="44">
       <c r="A14" s="49"/>
       <c r="B14" s="47"/>
       <c r="C14" s="31" t="s">
@@ -4058,7 +4058,7 @@
         <v>207</v>
       </c>
     </row>
-    <row r="15" spans="1:4" ht="70" customHeight="1">
+    <row r="15" spans="1:4" ht="44">
       <c r="A15" s="49"/>
       <c r="B15" s="47"/>
       <c r="C15" s="31" t="s">
@@ -4068,7 +4068,7 @@
         <v>208</v>
       </c>
     </row>
-    <row r="16" spans="1:4" ht="70" customHeight="1">
+    <row r="16" spans="1:4" ht="55">
       <c r="A16" s="50" t="s">
         <v>209</v>
       </c>
@@ -4082,7 +4082,7 @@
         <v>210</v>
       </c>
     </row>
-    <row r="17" spans="1:4" ht="70" customHeight="1">
+    <row r="17" spans="1:4" ht="55">
       <c r="A17" s="51"/>
       <c r="B17" s="54"/>
       <c r="C17" s="31" t="s">
@@ -4092,7 +4092,7 @@
         <v>211</v>
       </c>
     </row>
-    <row r="18" spans="1:4" ht="70" customHeight="1">
+    <row r="18" spans="1:4" ht="55">
       <c r="A18" s="51"/>
       <c r="B18" s="54"/>
       <c r="C18" s="31" t="s">
@@ -4102,7 +4102,7 @@
         <v>212</v>
       </c>
     </row>
-    <row r="19" spans="1:4" ht="70" customHeight="1">
+    <row r="19" spans="1:4" ht="44">
       <c r="A19" s="51"/>
       <c r="B19" s="54"/>
       <c r="C19" s="31" t="s">
@@ -4112,7 +4112,7 @@
         <v>213</v>
       </c>
     </row>
-    <row r="20" spans="1:4" ht="70" customHeight="1">
+    <row r="20" spans="1:4" ht="55">
       <c r="A20" s="52"/>
       <c r="B20" s="55"/>
       <c r="C20" s="34" t="s">

</xml_diff>

<commit_message>
Update A1b device profile with linked hardware
</commit_message>
<xml_diff>
--- a/assignments/assA1.xlsx
+++ b/assignments/assA1.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Desktop\Design-of-Enterprise-IoT-design\assignments\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B2774055-D53F-4FA9-BAAA-8BBC66693DF9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{60E66001-CA21-45A6-839F-5603F0F1426C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="380" yWindow="380" windowWidth="19200" windowHeight="9970" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -22,7 +22,7 @@
   <definedNames>
     <definedName name="_xlnm.Print_Area" localSheetId="4">'IoT Connectivity'!$A$1:$D$20</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="3">'IoT Connectivity (network only)'!$A$1:$D$9</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="2">'IoT Device  Profile'!$A$1:$G$15</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="2">'IoT Device  Profile'!$A$1:$G$13</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="0">'Value Proposition'!$A$1:$B$20</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="1">'Value Proposition en'!$A$1:$B$20</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="4">'IoT Connectivity'!$1:$1</definedName>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="251" uniqueCount="215">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="237" uniqueCount="207">
   <si>
     <t>IoT solution: Smart Turtle Breeding System (STBS)</t>
   </si>
@@ -1245,9 +1245,6 @@
     <t>If the cloud connects with a system, what is the purpose of the connection?</t>
   </si>
   <si>
-    <t>Atlas Scientific Industrial RTD Temperature Kit (KIT-303)</t>
-  </si>
-  <si>
     <t>Sensor</t>
   </si>
   <si>
@@ -1257,222 +1254,15 @@
     <t>Water temperature</t>
   </si>
   <si>
-    <t>Class-A PT-1000 probe; approx. -55 to 220 °C; transmitter accuracy ±0.1 °C; 4–20 mA; 9–36 VDC. (Atlas Scientific, n.d.) https://atlas-scientific.com/transmitters/rtd-temperature-transmitter/</t>
-  </si>
-  <si>
-    <t>PT-1000 probe, RTD3 transmitter, immersion fitting, 24 VDC supply, Opta analogue input</t>
-  </si>
-  <si>
-    <t>Industrial current loop suits long fixed cable runs in a wet plant. The range exceeds the operating envelope and supports continuous local heater control.</t>
-  </si>
-  <si>
-    <t>Atlas Scientific Industrial pH Kit (KIT-102P)</t>
-  </si>
-  <si>
     <t>pH value</t>
   </si>
   <si>
-    <t>pH 0–14; stated accuracy ±0.002; internal PT1000; about 1 s response; 4–20 mA; 3 m cable. (Atlas Scientific, n.d.) https://atlas-scientific.com/kits/industrial-ph-kit/</t>
-  </si>
-  <si>
-    <t>Industrial pH probe and transmitter, immersion fitting, calibration solutions, 24 VDC supply</t>
-  </si>
-  <si>
-    <t>Provides a calibrated industrial interface for early detection of unsuitable acidity or alkalinity. Scheduled two/three-point calibration manages drift.</t>
-  </si>
-  <si>
-    <t>DFRobot Industrial RS485 Turbidity Sensor (SEN0710)</t>
-  </si>
-  <si>
     <t>Turbidity</t>
   </si>
   <si>
-    <t>0–1000 NTU; 0.1 NTU resolution; ±5% full scale; IP68; 10–30 VDC; RS-485 Modbus RTU. (DFRobot, n.d.) https://www.dfrobot.com/product-3104.html</t>
-  </si>
-  <si>
-    <t>Optical probe, Modbus interface, protective stilling tube, 24 VDC supply, shielded RS-485 trunk</t>
-  </si>
-  <si>
-    <t>A waterproof digital probe supports continuous clarity trends and helps identify filtration problems without noise-prone low-level analogue signals.</t>
-  </si>
-  <si>
-    <t>DFRobot Industrial Ammonia-Nitrogen and pH Sensor (SEN0711)</t>
-  </si>
-  <si>
-    <t>Ammonia nitrogen, with pH and temperature compensation</t>
-  </si>
-  <si>
-    <t>NH3-N 0–100 mg/L; 0.01 mg/L resolution; ±3% full scale; pH 0–14; IP68; RS-485 Modbus RTU; 10–30 VDC. (DFRobot, n.d.) https://www.dfrobot.com/product-3107.html</t>
-  </si>
-  <si>
-    <t>Ammonia/pH/temperature probe, Modbus transmitter, immersion mount, calibration standards, 24 VDC supply</t>
-  </si>
-  <si>
-    <t>Direct ammonia indication addresses a high-risk water-quality condition. Compensation channels and local rate-of-change checks reduce false alarms.</t>
-  </si>
-  <si>
-    <t>DFRobot Submersible Water Level Sensor (KIT0139)</t>
-  </si>
-  <si>
-    <t>Water depth and level</t>
-  </si>
-  <si>
-    <t>0–5 m range; ±0.5% full scale; 4–20 mA; 12–36 VDC; IP68 stainless probe. (DFRobot, n.d.) https://www.dfrobot.com/product-1863.html</t>
-  </si>
-  <si>
-    <t>Pressure probe, vented cable termination, stilling tube, 24 VDC supply, Opta analogue input</t>
-  </si>
-  <si>
-    <t>Independent level feedback prevents overflow, excessive drainage and dry-running, and verifies bounded water-change commands.</t>
-  </si>
-  <si>
-    <t>DFRobot Water Flow Sensor (SEN0217 / YF-S201)</t>
-  </si>
-  <si>
-    <t>Tank inlet and drain pipes</t>
-  </si>
-  <si>
-    <t>Flow rate and transferred volume</t>
-  </si>
-  <si>
-    <t>1–30 L/min; Hall-effect pulse output; ±5% over 2–30 L/min; 3.5–12 VDC; 1/2-inch fitting. (DFRobot, n.d.) https://www.dfrobot.com/product-1517.html</t>
-  </si>
-  <si>
-    <t>Two sensors per tank, service unions, screened low-voltage cable, Opta pulse inputs</t>
-  </si>
-  <si>
-    <t>Inlet and drain totals cross-check level change and expose blocked pipes, pump faults or stuck valves while limiting exchanged volume.</t>
-  </si>
-  <si>
-    <t>DFRobot A02YYUW Waterproof Ultrasonic Sensor (SEN0311)</t>
-  </si>
-  <si>
-    <t>Feed in each zone hopper</t>
-  </si>
-  <si>
-    <t>Remaining feed height</t>
-  </si>
-  <si>
-    <t>3–450 cm range; 3 cm blind zone; ±1 cm; 100 ms response; IP67; 3.3–5 V UART. (DFRobot, n.d.) https://www.dfrobot.com/product-1935.html</t>
-  </si>
-  <si>
-    <t>Top mount, dust shield, isolated UART interface, hopper-specific distance-to-fill calibration</t>
-  </si>
-  <si>
-    <t>One sensor per zone hopper provides a low-feed alert. Calibration accounts for the sloped pellet surface and converts distance to an approximate fill percentage.</t>
-  </si>
-  <si>
-    <t>Atlas Scientific EZO Humidity Probe (EZO-HUM-P-S)</t>
-  </si>
-  <si>
-    <t>Air in each breeding/nesting zone</t>
-  </si>
-  <si>
-    <t>Relative humidity and air temperature</t>
-  </si>
-  <si>
-    <t>0–100% RH; stated ±2% RH from 5–95%; 3.3–5 V; UART/I2C; IP67 stainless probe. (Atlas Scientific, n.d.) https://atlas-scientific.com/probes/humidity-probe/</t>
-  </si>
-  <si>
-    <t>Shielded placement away from spray, isolated interface, mounting bracket, periodic comparison check</t>
-  </si>
-  <si>
-    <t>Zone humidity reveals condensation risk that can affect electronics and camera visibility, and provides context for nesting-area observations.</t>
-  </si>
-  <si>
-    <t>Aqua Medic Titanium Heater 500 W</t>
-  </si>
-  <si>
     <t>Actuator</t>
   </si>
   <si>
-    <t>Heat input and water temperature</t>
-  </si>
-  <si>
-    <t>500 W; 110–240 VAC; intended for about 1000–1500 L; external controller required. (Aqua Medic, n.d.) https://www.aqua-medic.de/de/Produkte/Titanium-Heater~p3831</t>
-  </si>
-  <si>
-    <t>Titanium element, rated contactor, RCD, guarded mount, manual isolation, independent over-temperature cut-out</t>
-  </si>
-  <si>
-    <t>Corrosion-resistant construction suits aquaculture. PLC control uses conservative hysteresis, while the independent cut-out remains the final safety layer.</t>
-  </si>
-  <si>
-    <t>AQUAEL UNI PUMP 1500</t>
-  </si>
-  <si>
-    <t>Tank recirculation and filtration line</t>
-  </si>
-  <si>
-    <t>Water circulation</t>
-  </si>
-  <si>
-    <t>1400 L/h; 19 W; maximum head 1.55 m; 220–240 VAC; IPX8; submerged or inline. (AQUAEL, n.d.) https://www.aquael.com/us/products/aquaristics-us/pumps-circulators-us/unipump/</t>
-  </si>
-  <si>
-    <t>Pump, strainer, check valve, service bypass, RCD, overload protection, rated contactor</t>
-  </si>
-  <si>
-    <t>Low-power continuous circulation supports filtration. Flow feedback detects loss of prime, blockage or pump failure.</t>
-  </si>
-  <si>
-    <t>Bürkert Type 6213 EV Normally Closed Valve, 24 VDC</t>
-  </si>
-  <si>
-    <t>Tank inlet and drain lines</t>
-  </si>
-  <si>
-    <t>Water flow state</t>
-  </si>
-  <si>
-    <t>Two-way servo-assisted diaphragm valve; normally closed; 24 VDC option; water service; IP65 with suitable plug. (Bürkert, n.d.) https://www.burkert.com/en/products/solenoid-valves/general-purpose-2-2-solenoids/270895</t>
-  </si>
-  <si>
-    <t>Two valves per tank, selected DN/pressure variant, coil suppression, manual isolation, upstream strainer</t>
-  </si>
-  <si>
-    <t>Normally closed action fails safe on power loss. Paired with level and flow feedback, it enables bounded partial water exchange.</t>
-  </si>
-  <si>
-    <t>FIAP Electronic Feeder 10 kg with Spreader (1586-1)</t>
-  </si>
-  <si>
-    <t>Actuator / device</t>
-  </si>
-  <si>
-    <t>Feed supplied to turtles in each zone</t>
-  </si>
-  <si>
-    <t>Feeding time and estimated portion</t>
-  </si>
-  <si>
-    <t>10 kg hopper; 12 VDC; non-clogging screw; adjustable 2–12 m spread radius. (FIAP, n.d.) https://www.fiap.com/elektronikfuetterer-10-kg-mit-streuer.html</t>
-  </si>
-  <si>
-    <t>Hopper, screw and spreader, isolated enable relay, guarded chute, feed-level sensor, catch-test calibration</t>
-  </si>
-  <si>
-    <t>Commercial feeder reduces manual dosing. Runtime-to-mass calibration and hopper feedback provide a practical, auditable portion estimate.</t>
-  </si>
-  <si>
-    <t>Reolink RLC-811A</t>
-  </si>
-  <si>
-    <t>Turtle activity, feeding and nesting areas</t>
-  </si>
-  <si>
-    <t>Video and event evidence</t>
-  </si>
-  <si>
-    <t>8 MP at 25 fps; H.264/H.265; 5× optical zoom; RTSP/HTTPS; IEEE 802.3af PoE; &lt;12 W; IP67. (Reolink, n.d.) https://support.reolink.com/c/rlc-811a/</t>
-  </si>
-  <si>
-    <t>Image sensor, lens, processor, Ethernet/PoE interface, mount, privacy mask, local microSD fallback</t>
-  </si>
-  <si>
-    <t>Wired PoE avoids local adapters. Standard streams support local activity and nesting inference without continuous cloud video upload.</t>
-  </si>
-  <si>
     <t>20 tank instrument sets; 4 × Arduino Opta RS485 controllers with A0602/D1608 I/O; 20 Reolink RLC-811A PoE cameras; TP-Link TL-SG3428XMP managed PoE+ switch; AAEON BOXER-8653AI edge computer; Teltonika RUTX11 router.</t>
   </si>
   <si>
@@ -1537,6 +1327,192 @@
   </si>
   <si>
     <t>The cloud exports approved maintenance tickets, calibration schedules, equipment runtime, water/feed consumption and compliance summaries through an API or scheduled CSV. Only necessary identifiers and evidence are included. Return status can close a ticket, but the external system cannot issue raw actuator commands.</t>
+  </si>
+  <si>
+    <t>DFRobot DS18B20 Waterproof Temperature Sensor (BOS0042) / 防水温度传感器</t>
+  </si>
+  <si>
+    <t>Waterproof DS18B20 probe; 3–5 V; PH2.0-3P connector; sensing range −55 to 125 °C; display range −10 to 85 °C with ±0.5 °C stated error; requires a pull-up resistor. Source: DFRobot BOS0042.</t>
+  </si>
+  <si>
+    <t>Waterproof DS18B20 probe, 3-pin cable, pull-up resistor, PH2.0 adapter and controller input.</t>
+  </si>
+  <si>
+    <t>Direct temperature feedback supports heater control and alarm limits in wet tanks. The sealed probe is suitable for remote or humid measurement, while local validation prevents unsafe heating commands.</t>
+  </si>
+  <si>
+    <t>DFRobot SEN0189 Turbidity Sensor / 浑浊度传感器</t>
+  </si>
+  <si>
+    <t>Water clarity in each breeding tank</t>
+  </si>
+  <si>
+    <t>Optical infrared emitter/receiver; 5 VDC; 40 mA maximum; response below 500 ms; selectable analogue 0–4.5 V or thresholded digital output; operating range −30 to 80 °C. The probe top is not waterproof.</t>
+  </si>
+  <si>
+    <t>Optical turbidity probe, interface board, A/D or GPIO input, analogue/digital selector and threshold potentiometer.</t>
+  </si>
+  <si>
+    <t>Provides an early warning of suspended solids, filtration faults and contamination. Digital threshold alarms can be local, while analogue values support trend analysis and water-change decisions.</t>
+  </si>
+  <si>
+    <t>DFRobot SEN0161-V2 Gravity Analog pH Meter / 模拟 pH 计 V2</t>
+  </si>
+  <si>
+    <t>Water chemistry in each breeding tank</t>
+  </si>
+  <si>
+    <t>Signal board supply 3.3–5.5 V; analogue output 0–3.0 V; BNC electrode and PH2.0-3P signal connector; stated accuracy ±0.1 at 25 °C; electrode range pH 0–14, 5–60 °C, response below 2 min; 1 m cable.</t>
+  </si>
+  <si>
+    <t>Laboratory-grade pH electrode, V2 signal-conversion board, BNC cable, PH2.0-3P lead, calibration buffers and analogue input.</t>
+  </si>
+  <si>
+    <t>pH is a key water-quality variable for aquaculture. Two-point calibration and local plausibility/rate checks allow the PLC to alarm and bound corrective actions.</t>
+  </si>
+  <si>
+    <t>Lonhand LH-WQS-AN-485-UI NH3-N Ion Sensor / 氨氮离子传感器</t>
+  </si>
+  <si>
+    <t>Ammonia-nitrogen concentration</t>
+  </si>
+  <si>
+    <t>Measurement range 0.1–18,000 mg/L; temperature range 0–60 °C; 4–20 mA and RS-485 outputs; IP68; 5 m cable; NPT3/4 or M39×1.5 connection; 0–3 bar; pH 4–10; repeatability ±4%; PC/PBT corrosion-resistant housing.</t>
+  </si>
+  <si>
+    <t>Ion-selective ammonia electrode, 4–20 mA/RS-485 transmitter, 5 m cable, immersion fitting, PLC analogue/Modbus input and calibration solution.</t>
+  </si>
+  <si>
+    <t>Ammonia is a high-risk water-quality condition. A wired industrial output supports continuous trend logging, local alarm thresholds and dependable response even when the network is unavailable.</t>
+  </si>
+  <si>
+    <t>AXIS M3086-V Network Camera / 网络摄像机</t>
+  </si>
+  <si>
+    <t>Breeding and nesting-zone activity and evidence</t>
+  </si>
+  <si>
+    <t>Video stream and event evidence</t>
+  </si>
+  <si>
+    <t>4 MP maximum resolution 2688×1512; 2.4 mm F2.1 lens; 130° horizontal and 93° vertical field of view; H.264/H.265/Motion JPEG; 25/30 fps; WDR up to 120 dB; Lightfinder; PoE Class 2; IP42 and IK08 variants.</t>
+  </si>
+  <si>
+    <t>Network camera, lens, PoE RJ45 connector, SD-card slot, control button, mounting dome and managed-switch port.</t>
+  </si>
+  <si>
+    <t>Video provides farm-wide context and event evidence for activity, feeding and nesting. PoE simplifies installation; edge analytics should retain only validated clips rather than upload continuous video.</t>
+  </si>
+  <si>
+    <t>Raspberry Pi 5 (8 GB)</t>
+  </si>
+  <si>
+    <t>Device</t>
+  </si>
+  <si>
+    <t>Edge gateway and local sensor aggregation</t>
+  </si>
+  <si>
+    <t>Local processing, protocol bridging and storage</t>
+  </si>
+  <si>
+    <t>Broadcom BCM2712 2.4 GHz quad-core 64-bit Arm Cortex-A76; 8 GB LPDDR4X-4267; standard 40-pin GPIO header; USB, Ethernet, Wi-Fi and Bluetooth; 5 V USB-C power and active cooling recommended for sustained workloads.</t>
+  </si>
+  <si>
+    <t>Raspberry Pi 5 board, microSD or SSD, 40-pin GPIO interface, USB/Ethernet/Wi-Fi links, power supply, case and active cooler.</t>
+  </si>
+  <si>
+    <t>A low-cost Linux edge node can bridge sensors, MQTT and dashboards, buffer data and pre-process camera events. Safety-critical interlocks remain in the dedicated PLC rather than the general-purpose board.</t>
+  </si>
+  <si>
+    <t>ESP32-WROOM-32</t>
+  </si>
+  <si>
+    <t>Distributed sensor and low-power actuator nodes</t>
+  </si>
+  <si>
+    <t>Wireless telemetry and GPIO control</t>
+  </si>
+  <si>
+    <t>Dual-core Xtensa LX6 up to 240 MHz; 448 KB ROM, 520 KB SRAM and 4 MB SPI flash; 2.4 GHz 802.11 b/g/n up to 150 Mbps; Bluetooth 4.2/BLE; up to 32 GPIO; ADC, DAC, touch, PWM and serial peripherals; 3.0–3.6 V supply.</t>
+  </si>
+  <si>
+    <t>ESP32-WROOM-32 module, PCB antenna, 40 MHz crystal, flash, GPIO/ADC interface, regulated 3.3 V supply and enclosure.</t>
+  </si>
+  <si>
+    <t>Provides an economical wireless interface for non-critical distributed measurements. Wet-area deployments still need isolation, watchdogs and bounded local outputs before any actuator command is accepted.</t>
+  </si>
+  <si>
+    <t>Ubuntu Server 22.04</t>
+  </si>
+  <si>
+    <t>Edge/server software platform</t>
+  </si>
+  <si>
+    <t>Container, storage, MQTT and API runtime</t>
+  </si>
+  <si>
+    <t>Ubuntu Server 22.04 LTS provides a maintainable Linux base for scale-out services, networking, storage, containers and system administration. The workload can run on Raspberry Pi 5 or another supported ARM/x86 host.</t>
+  </si>
+  <si>
+    <t>Ubuntu Server image, host storage, network interface, container runtime, MQTT broker, time-series database, API service and monitoring.</t>
+  </si>
+  <si>
+    <t>A documented LTS platform supports repeatable deployment, security updates and service separation for the edge gateway. It improves maintainability without placing deterministic safety control in the operating system.</t>
+  </si>
+  <si>
+    <t>HC-SR501 PIR Motion Sensor / 人体红外传感器</t>
+  </si>
+  <si>
+    <t>Activity in breeding or nesting areas</t>
+  </si>
+  <si>
+    <t>Motion event</t>
+  </si>
+  <si>
+    <t>Pyroelectric dual-element PIR module; 4.5–20 V supply; below 50 µA stated current; 3.3 V high/0 V low GPIO output; cone below 100°; three pins; selectable repeatable/non-repeatable trigger and adjustable delay/sensitivity.</t>
+  </si>
+  <si>
+    <t>PIR element, Fresnel lens, comparator board, delay and sensitivity potentiometers, VCC/OUT/GND header and GPIO input.</t>
+  </si>
+  <si>
+    <t>A low-cost motion trigger can wake or tag camera recording and reduce continuous processing. It is not a safety sensor because initialization time, wind, lighting and animal movement can cause false or missed events.</t>
+  </si>
+  <si>
+    <t>PondMAX Solar Automatic Fish Feeder</t>
+  </si>
+  <si>
+    <t>Feed hopper and pond feeding schedule</t>
+  </si>
+  <si>
+    <t>Scheduled feed dispensing</t>
+  </si>
+  <si>
+    <t>Solar charging with built-in 2200 mAh lithium battery; 1–6 feedings per day; adjustable S/M/L throw and 0–20 s feed duration; 3–10 mm food size; 12 V/1.66 A adapter specification in the supplied manual.</t>
+  </si>
+  <si>
+    <t>Solar panel, rechargeable battery, hopper, motor and spreader, timer/display controls, protective cover and mounting bracket.</t>
+  </si>
+  <si>
+    <t>Automated feeding improves schedule consistency and reduces manual labour. Feed commands should remain bounded by time, quantity and hopper checks, with an operator override and an audit record.</t>
+  </si>
+  <si>
+    <t>Bluefish MINI-200 Submersible Pump / 潜水泵</t>
+  </si>
+  <si>
+    <t>Tank recirculation and water-change line</t>
+  </si>
+  <si>
+    <t>Water circulation and flow</t>
+  </si>
+  <si>
+    <t>12 VDC; 0.4 A; 4.8 W; 200 L/h open flow; 1.5 m maximum head; brushless motor; IP68 submersible construction; approximately 43×38×30 mm; below 35 dB; dry-run/block protection options.</t>
+  </si>
+  <si>
+    <t>Brushless pump, impeller, inlet/outlet, sealed motor, silicone vibration feet, 12 V supply, relay/MOSFET driver and flow feedback.</t>
+  </si>
+  <si>
+    <t>Low-voltage circulation supports filtration and controlled water changes. A relay, flow confirmation and dry-run protection prevent a blocked line or empty tank from damaging the pump.</t>
   </si>
 </sst>
 </file>
@@ -2590,7 +2566,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="56">
+  <cellXfs count="58">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -2756,6 +2732,12 @@
     </xf>
     <xf numFmtId="0" fontId="43" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="17" xfId="6" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="38" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="49">
@@ -3439,310 +3421,295 @@
         <v>86</v>
       </c>
     </row>
-    <row r="3" spans="1:7" ht="99" customHeight="1">
-      <c r="A3" s="24" t="s">
+    <row r="3" spans="1:7" ht="120" customHeight="1">
+      <c r="A3" s="56" t="s">
+        <v>145</v>
+      </c>
+      <c r="B3" s="57" t="s">
         <v>117</v>
       </c>
-      <c r="B3" s="23" t="s">
+      <c r="C3" s="23" t="s">
         <v>118</v>
       </c>
-      <c r="C3" s="23" t="s">
+      <c r="D3" s="23" t="s">
         <v>119</v>
       </c>
-      <c r="D3" s="23" t="s">
+      <c r="E3" s="23" t="s">
+        <v>146</v>
+      </c>
+      <c r="F3" s="23" t="s">
+        <v>147</v>
+      </c>
+      <c r="G3" s="23" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" ht="99" customHeight="1">
+      <c r="A4" s="56" t="s">
+        <v>149</v>
+      </c>
+      <c r="B4" s="57" t="s">
+        <v>117</v>
+      </c>
+      <c r="C4" s="23" t="s">
+        <v>150</v>
+      </c>
+      <c r="D4" s="23" t="s">
+        <v>121</v>
+      </c>
+      <c r="E4" s="23" t="s">
+        <v>151</v>
+      </c>
+      <c r="F4" s="23" t="s">
+        <v>152</v>
+      </c>
+      <c r="G4" s="23" t="s">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" ht="101" customHeight="1">
+      <c r="A5" s="56" t="s">
+        <v>154</v>
+      </c>
+      <c r="B5" s="57" t="s">
+        <v>117</v>
+      </c>
+      <c r="C5" s="23" t="s">
+        <v>155</v>
+      </c>
+      <c r="D5" s="23" t="s">
         <v>120</v>
       </c>
-      <c r="E3" s="23" t="s">
-        <v>121</v>
-      </c>
-      <c r="F3" s="23" t="s">
+      <c r="E5" s="23" t="s">
+        <v>156</v>
+      </c>
+      <c r="F5" s="23" t="s">
+        <v>157</v>
+      </c>
+      <c r="G5" s="23" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" ht="101" customHeight="1">
+      <c r="A6" s="56" t="s">
+        <v>159</v>
+      </c>
+      <c r="B6" s="57" t="s">
+        <v>117</v>
+      </c>
+      <c r="C6" s="23" t="s">
+        <v>155</v>
+      </c>
+      <c r="D6" s="23" t="s">
+        <v>160</v>
+      </c>
+      <c r="E6" s="23" t="s">
+        <v>161</v>
+      </c>
+      <c r="F6" s="23" t="s">
+        <v>162</v>
+      </c>
+      <c r="G6" s="23" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" ht="99" customHeight="1">
+      <c r="A7" s="56" t="s">
+        <v>164</v>
+      </c>
+      <c r="B7" s="57" t="s">
+        <v>117</v>
+      </c>
+      <c r="C7" s="23" t="s">
+        <v>165</v>
+      </c>
+      <c r="D7" s="23" t="s">
+        <v>166</v>
+      </c>
+      <c r="E7" s="23" t="s">
+        <v>167</v>
+      </c>
+      <c r="F7" s="23" t="s">
+        <v>168</v>
+      </c>
+      <c r="G7" s="23" t="s">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" ht="99" customHeight="1">
+      <c r="A8" s="56" t="s">
+        <v>170</v>
+      </c>
+      <c r="B8" s="57" t="s">
+        <v>171</v>
+      </c>
+      <c r="C8" s="23" t="s">
+        <v>172</v>
+      </c>
+      <c r="D8" s="23" t="s">
+        <v>173</v>
+      </c>
+      <c r="E8" s="23" t="s">
+        <v>174</v>
+      </c>
+      <c r="F8" s="23" t="s">
+        <v>175</v>
+      </c>
+      <c r="G8" s="23" t="s">
+        <v>176</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" ht="99" customHeight="1">
+      <c r="A9" s="56" t="s">
+        <v>177</v>
+      </c>
+      <c r="B9" s="57" t="s">
+        <v>171</v>
+      </c>
+      <c r="C9" s="23" t="s">
+        <v>178</v>
+      </c>
+      <c r="D9" s="23" t="s">
+        <v>179</v>
+      </c>
+      <c r="E9" s="23" t="s">
+        <v>180</v>
+      </c>
+      <c r="F9" s="23" t="s">
+        <v>181</v>
+      </c>
+      <c r="G9" s="23" t="s">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" ht="119" customHeight="1">
+      <c r="A10" s="56" t="s">
+        <v>183</v>
+      </c>
+      <c r="B10" s="57" t="s">
+        <v>171</v>
+      </c>
+      <c r="C10" s="23" t="s">
+        <v>184</v>
+      </c>
+      <c r="D10" s="23" t="s">
+        <v>185</v>
+      </c>
+      <c r="E10" s="23" t="s">
+        <v>186</v>
+      </c>
+      <c r="F10" s="23" t="s">
+        <v>187</v>
+      </c>
+      <c r="G10" s="23" t="s">
+        <v>188</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" ht="99" customHeight="1">
+      <c r="A11" s="56" t="s">
+        <v>189</v>
+      </c>
+      <c r="B11" s="57" t="s">
+        <v>117</v>
+      </c>
+      <c r="C11" s="23" t="s">
+        <v>190</v>
+      </c>
+      <c r="D11" s="23" t="s">
+        <v>191</v>
+      </c>
+      <c r="E11" s="23" t="s">
+        <v>192</v>
+      </c>
+      <c r="F11" s="23" t="s">
+        <v>193</v>
+      </c>
+      <c r="G11" s="23" t="s">
+        <v>194</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" ht="99" customHeight="1">
+      <c r="A12" s="56" t="s">
+        <v>195</v>
+      </c>
+      <c r="B12" s="57" t="s">
         <v>122</v>
       </c>
-      <c r="G3" s="23" t="s">
-        <v>123</v>
-      </c>
-    </row>
-    <row r="4" spans="1:7" ht="80" customHeight="1">
-      <c r="A4" s="24" t="s">
-        <v>124</v>
-      </c>
-      <c r="B4" s="23" t="s">
-        <v>118</v>
-      </c>
-      <c r="C4" s="23" t="s">
-        <v>119</v>
-      </c>
-      <c r="D4" s="23" t="s">
-        <v>125</v>
-      </c>
-      <c r="E4" s="23" t="s">
-        <v>126</v>
-      </c>
-      <c r="F4" s="23" t="s">
-        <v>127</v>
-      </c>
-      <c r="G4" s="23" t="s">
-        <v>128</v>
-      </c>
-    </row>
-    <row r="5" spans="1:7" ht="80" customHeight="1">
-      <c r="A5" s="24" t="s">
-        <v>129</v>
-      </c>
-      <c r="B5" s="23" t="s">
-        <v>118</v>
-      </c>
-      <c r="C5" s="23" t="s">
-        <v>119</v>
-      </c>
-      <c r="D5" s="23" t="s">
-        <v>130</v>
-      </c>
-      <c r="E5" s="23" t="s">
-        <v>131</v>
-      </c>
-      <c r="F5" s="23" t="s">
-        <v>132</v>
-      </c>
-      <c r="G5" s="23" t="s">
-        <v>133</v>
-      </c>
-    </row>
-    <row r="6" spans="1:7" ht="80" customHeight="1">
-      <c r="A6" s="24" t="s">
-        <v>134</v>
-      </c>
-      <c r="B6" s="23" t="s">
-        <v>118</v>
-      </c>
-      <c r="C6" s="23" t="s">
-        <v>119</v>
-      </c>
-      <c r="D6" s="23" t="s">
-        <v>135</v>
-      </c>
-      <c r="E6" s="23" t="s">
-        <v>136</v>
-      </c>
-      <c r="F6" s="23" t="s">
-        <v>137</v>
-      </c>
-      <c r="G6" s="23" t="s">
-        <v>138</v>
-      </c>
-    </row>
-    <row r="7" spans="1:7" ht="60" customHeight="1">
-      <c r="A7" s="24" t="s">
-        <v>139</v>
-      </c>
-      <c r="B7" s="23" t="s">
-        <v>118</v>
-      </c>
-      <c r="C7" s="23" t="s">
-        <v>119</v>
-      </c>
-      <c r="D7" s="23" t="s">
-        <v>140</v>
-      </c>
-      <c r="E7" s="23" t="s">
-        <v>141</v>
-      </c>
-      <c r="F7" s="23" t="s">
-        <v>142</v>
-      </c>
-      <c r="G7" s="23" t="s">
-        <v>143</v>
-      </c>
-    </row>
-    <row r="8" spans="1:7" ht="60" customHeight="1">
-      <c r="A8" s="24" t="s">
-        <v>144</v>
-      </c>
-      <c r="B8" s="23" t="s">
-        <v>118</v>
-      </c>
-      <c r="C8" s="23" t="s">
-        <v>145</v>
-      </c>
-      <c r="D8" s="23" t="s">
-        <v>146</v>
-      </c>
-      <c r="E8" s="23" t="s">
-        <v>147</v>
-      </c>
-      <c r="F8" s="23" t="s">
-        <v>148</v>
-      </c>
-      <c r="G8" s="23" t="s">
-        <v>149</v>
-      </c>
-    </row>
-    <row r="9" spans="1:7" ht="80" customHeight="1">
-      <c r="A9" s="24" t="s">
-        <v>150</v>
-      </c>
-      <c r="B9" s="23" t="s">
-        <v>118</v>
-      </c>
-      <c r="C9" s="23" t="s">
-        <v>151</v>
-      </c>
-      <c r="D9" s="23" t="s">
-        <v>152</v>
-      </c>
-      <c r="E9" s="23" t="s">
-        <v>153</v>
-      </c>
-      <c r="F9" s="23" t="s">
-        <v>154</v>
-      </c>
-      <c r="G9" s="23" t="s">
-        <v>155</v>
-      </c>
-    </row>
-    <row r="10" spans="1:7" ht="80" customHeight="1">
-      <c r="A10" s="24" t="s">
-        <v>156</v>
-      </c>
-      <c r="B10" s="23" t="s">
-        <v>118</v>
-      </c>
-      <c r="C10" s="23" t="s">
-        <v>157</v>
-      </c>
-      <c r="D10" s="23" t="s">
-        <v>158</v>
-      </c>
-      <c r="E10" s="23" t="s">
-        <v>159</v>
-      </c>
-      <c r="F10" s="23" t="s">
-        <v>160</v>
-      </c>
-      <c r="G10" s="23" t="s">
-        <v>161</v>
-      </c>
-    </row>
-    <row r="11" spans="1:7" ht="80" customHeight="1">
-      <c r="A11" s="24" t="s">
-        <v>162</v>
-      </c>
-      <c r="B11" s="23" t="s">
-        <v>163</v>
-      </c>
-      <c r="C11" s="23" t="s">
-        <v>119</v>
-      </c>
-      <c r="D11" s="23" t="s">
-        <v>164</v>
-      </c>
-      <c r="E11" s="23" t="s">
-        <v>165</v>
-      </c>
-      <c r="F11" s="23" t="s">
-        <v>166</v>
-      </c>
-      <c r="G11" s="23" t="s">
-        <v>167</v>
-      </c>
-    </row>
-    <row r="12" spans="1:7" ht="80" customHeight="1">
-      <c r="A12" s="24" t="s">
-        <v>168</v>
-      </c>
-      <c r="B12" s="23" t="s">
-        <v>163</v>
-      </c>
       <c r="C12" s="23" t="s">
-        <v>169</v>
+        <v>196</v>
       </c>
       <c r="D12" s="23" t="s">
-        <v>170</v>
+        <v>197</v>
       </c>
       <c r="E12" s="23" t="s">
-        <v>171</v>
+        <v>198</v>
       </c>
       <c r="F12" s="23" t="s">
-        <v>172</v>
+        <v>199</v>
       </c>
       <c r="G12" s="23" t="s">
-        <v>173</v>
+        <v>200</v>
       </c>
     </row>
     <row r="13" spans="1:7" ht="99" customHeight="1">
-      <c r="A13" s="24" t="s">
-        <v>174</v>
-      </c>
-      <c r="B13" s="23" t="s">
-        <v>163</v>
+      <c r="A13" s="56" t="s">
+        <v>201</v>
+      </c>
+      <c r="B13" s="57" t="s">
+        <v>122</v>
       </c>
       <c r="C13" s="23" t="s">
-        <v>175</v>
+        <v>202</v>
       </c>
       <c r="D13" s="23" t="s">
-        <v>176</v>
+        <v>203</v>
       </c>
       <c r="E13" s="23" t="s">
-        <v>177</v>
+        <v>204</v>
       </c>
       <c r="F13" s="23" t="s">
-        <v>178</v>
+        <v>205</v>
       </c>
       <c r="G13" s="23" t="s">
-        <v>179</v>
+        <v>206</v>
       </c>
     </row>
     <row r="14" spans="1:7" ht="80" customHeight="1">
-      <c r="A14" s="24" t="s">
-        <v>180</v>
-      </c>
-      <c r="B14" s="23" t="s">
-        <v>181</v>
-      </c>
-      <c r="C14" s="23" t="s">
-        <v>182</v>
-      </c>
-      <c r="D14" s="23" t="s">
-        <v>183</v>
-      </c>
-      <c r="E14" s="23" t="s">
-        <v>184</v>
-      </c>
-      <c r="F14" s="23" t="s">
-        <v>185</v>
-      </c>
-      <c r="G14" s="23" t="s">
-        <v>186</v>
-      </c>
+      <c r="A14" s="24"/>
+      <c r="B14" s="23"/>
+      <c r="C14" s="23"/>
+      <c r="D14" s="23"/>
+      <c r="E14" s="23"/>
+      <c r="F14" s="23"/>
+      <c r="G14" s="23"/>
     </row>
     <row r="15" spans="1:7" ht="80" customHeight="1">
-      <c r="A15" s="24" t="s">
-        <v>187</v>
-      </c>
-      <c r="B15" s="23" t="s">
-        <v>118</v>
-      </c>
-      <c r="C15" s="23" t="s">
-        <v>188</v>
-      </c>
-      <c r="D15" s="23" t="s">
-        <v>189</v>
-      </c>
-      <c r="E15" s="23" t="s">
-        <v>190</v>
-      </c>
-      <c r="F15" s="23" t="s">
-        <v>191</v>
-      </c>
-      <c r="G15" s="23" t="s">
-        <v>192</v>
-      </c>
+      <c r="A15" s="24"/>
+      <c r="B15" s="23"/>
+      <c r="C15" s="23"/>
+      <c r="D15" s="23"/>
+      <c r="E15" s="23"/>
+      <c r="F15" s="23"/>
+      <c r="G15" s="23"/>
     </row>
   </sheetData>
   <phoneticPr fontId="68" type="noConversion"/>
+  <hyperlinks>
+    <hyperlink ref="A3" r:id="rId1" tooltip="Open source page" xr:uid="{42A0E00C-B42D-41EB-B276-EAECFC050B15}"/>
+    <hyperlink ref="A4" r:id="rId2" tooltip="Open source page" xr:uid="{0938D27D-A9A4-4FBF-8D46-D0AA28FCA6A2}"/>
+    <hyperlink ref="A5" r:id="rId3" tooltip="Open source page" xr:uid="{97966CAD-7DF6-44C8-9A6F-4AB23F8E9875}"/>
+    <hyperlink ref="A6" r:id="rId4" tooltip="Open source page" xr:uid="{EB77D51A-1541-4CEC-BA09-17BACE2419A3}"/>
+    <hyperlink ref="A7" r:id="rId5" tooltip="Open source page" xr:uid="{B8F21E40-6BE4-425D-813F-DCB8AB7D9786}"/>
+    <hyperlink ref="A8" r:id="rId6" tooltip="Open source page" xr:uid="{D1B738E5-B5F5-46BF-BFF4-F587A7C72FDB}"/>
+    <hyperlink ref="A9" r:id="rId7" tooltip="Open source page" xr:uid="{C300A4E9-D4C0-449D-9036-D3ED8F1A6E2E}"/>
+    <hyperlink ref="A10" r:id="rId8" tooltip="Open source page" xr:uid="{316C19EA-C254-49C8-8475-B2EEF617A556}"/>
+    <hyperlink ref="A11" r:id="rId9" tooltip="Open source page" xr:uid="{1D171974-6BA1-4FE6-8803-622547C50C52}"/>
+    <hyperlink ref="A12" r:id="rId10" tooltip="Open source page" xr:uid="{A09F48AD-7D03-4E9F-BF47-1F4F9EAB8F3E}"/>
+    <hyperlink ref="A13" r:id="rId11" tooltip="Open source page" xr:uid="{CCA3DFA5-ECB1-4F55-B109-B50ADEE8537B}"/>
+  </hyperlinks>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.22" right="0.22" top="0.25" bottom="0.25" header="0" footer="0"/>
-  <pageSetup paperSize="9" scale="66" fitToHeight="4" orientation="portrait" horizontalDpi="1200" verticalDpi="1200" r:id="rId1"/>
+  <pageSetup paperSize="9" scale="66" fitToHeight="4" orientation="portrait" horizontalDpi="1200" verticalDpi="1200" r:id="rId12"/>
 </worksheet>
 </file>
 
@@ -3776,7 +3743,7 @@
     </row>
     <row r="2" spans="1:4" ht="66">
       <c r="A2" s="42" t="s">
-        <v>193</v>
+        <v>123</v>
       </c>
       <c r="B2" s="27" t="s">
         <v>91</v>
@@ -3785,7 +3752,7 @@
         <v>92</v>
       </c>
       <c r="D2" s="28" t="s">
-        <v>194</v>
+        <v>124</v>
       </c>
     </row>
     <row r="3" spans="1:4" ht="55">
@@ -3797,7 +3764,7 @@
         <v>94</v>
       </c>
       <c r="D3" s="28" t="s">
-        <v>195</v>
+        <v>125</v>
       </c>
     </row>
     <row r="4" spans="1:4" ht="55">
@@ -3807,7 +3774,7 @@
         <v>95</v>
       </c>
       <c r="D4" s="28" t="s">
-        <v>196</v>
+        <v>126</v>
       </c>
     </row>
     <row r="5" spans="1:4" ht="44">
@@ -3817,7 +3784,7 @@
         <v>96</v>
       </c>
       <c r="D5" s="28" t="s">
-        <v>197</v>
+        <v>127</v>
       </c>
     </row>
     <row r="6" spans="1:4" ht="55">
@@ -3827,7 +3794,7 @@
         <v>97</v>
       </c>
       <c r="D6" s="28" t="s">
-        <v>198</v>
+        <v>128</v>
       </c>
     </row>
     <row r="7" spans="1:4" ht="77">
@@ -3837,7 +3804,7 @@
         <v>98</v>
       </c>
       <c r="D7" s="28" t="s">
-        <v>199</v>
+        <v>129</v>
       </c>
     </row>
     <row r="8" spans="1:4" ht="55">
@@ -3847,7 +3814,7 @@
         <v>99</v>
       </c>
       <c r="D8" s="29" t="s">
-        <v>200</v>
+        <v>130</v>
       </c>
     </row>
     <row r="9" spans="1:4" ht="66">
@@ -3857,7 +3824,7 @@
         <v>100</v>
       </c>
       <c r="D9" s="28" t="s">
-        <v>201</v>
+        <v>131</v>
       </c>
     </row>
     <row r="10" spans="1:4">
@@ -3920,7 +3887,7 @@
     </row>
     <row r="2" spans="1:4" ht="66">
       <c r="A2" s="44" t="s">
-        <v>193</v>
+        <v>123</v>
       </c>
       <c r="B2" s="31" t="s">
         <v>102</v>
@@ -3929,7 +3896,7 @@
         <v>103</v>
       </c>
       <c r="D2" s="32" t="s">
-        <v>194</v>
+        <v>124</v>
       </c>
     </row>
     <row r="3" spans="1:4" ht="55">
@@ -3941,7 +3908,7 @@
         <v>94</v>
       </c>
       <c r="D3" s="32" t="s">
-        <v>195</v>
+        <v>125</v>
       </c>
     </row>
     <row r="4" spans="1:4" ht="55">
@@ -3951,7 +3918,7 @@
         <v>95</v>
       </c>
       <c r="D4" s="32" t="s">
-        <v>196</v>
+        <v>126</v>
       </c>
     </row>
     <row r="5" spans="1:4" ht="44">
@@ -3961,7 +3928,7 @@
         <v>96</v>
       </c>
       <c r="D5" s="32" t="s">
-        <v>197</v>
+        <v>127</v>
       </c>
     </row>
     <row r="6" spans="1:4" ht="55">
@@ -3971,7 +3938,7 @@
         <v>97</v>
       </c>
       <c r="D6" s="32" t="s">
-        <v>198</v>
+        <v>128</v>
       </c>
     </row>
     <row r="7" spans="1:4" ht="77">
@@ -3981,7 +3948,7 @@
         <v>98</v>
       </c>
       <c r="D7" s="32" t="s">
-        <v>199</v>
+        <v>129</v>
       </c>
     </row>
     <row r="8" spans="1:4" ht="55">
@@ -3991,7 +3958,7 @@
         <v>99</v>
       </c>
       <c r="D8" s="33" t="s">
-        <v>200</v>
+        <v>130</v>
       </c>
     </row>
     <row r="9" spans="1:4" ht="66">
@@ -4001,12 +3968,12 @@
         <v>100</v>
       </c>
       <c r="D9" s="32" t="s">
-        <v>201</v>
+        <v>131</v>
       </c>
     </row>
     <row r="10" spans="1:4" ht="55">
       <c r="A10" s="48" t="s">
-        <v>202</v>
+        <v>132</v>
       </c>
       <c r="B10" s="46" t="s">
         <v>104</v>
@@ -4015,7 +3982,7 @@
         <v>105</v>
       </c>
       <c r="D10" s="32" t="s">
-        <v>203</v>
+        <v>133</v>
       </c>
     </row>
     <row r="11" spans="1:4" ht="55">
@@ -4025,7 +3992,7 @@
         <v>106</v>
       </c>
       <c r="D11" s="32" t="s">
-        <v>204</v>
+        <v>134</v>
       </c>
     </row>
     <row r="12" spans="1:4" ht="55">
@@ -4035,7 +4002,7 @@
         <v>107</v>
       </c>
       <c r="D12" s="32" t="s">
-        <v>205</v>
+        <v>135</v>
       </c>
     </row>
     <row r="13" spans="1:4" ht="55">
@@ -4045,7 +4012,7 @@
         <v>108</v>
       </c>
       <c r="D13" s="32" t="s">
-        <v>206</v>
+        <v>136</v>
       </c>
     </row>
     <row r="14" spans="1:4" ht="44">
@@ -4055,7 +4022,7 @@
         <v>109</v>
       </c>
       <c r="D14" s="32" t="s">
-        <v>207</v>
+        <v>137</v>
       </c>
     </row>
     <row r="15" spans="1:4" ht="44">
@@ -4065,12 +4032,12 @@
         <v>110</v>
       </c>
       <c r="D15" s="32" t="s">
-        <v>208</v>
+        <v>138</v>
       </c>
     </row>
     <row r="16" spans="1:4" ht="55">
       <c r="A16" s="50" t="s">
-        <v>209</v>
+        <v>139</v>
       </c>
       <c r="B16" s="53" t="s">
         <v>111</v>
@@ -4079,7 +4046,7 @@
         <v>112</v>
       </c>
       <c r="D16" s="32" t="s">
-        <v>210</v>
+        <v>140</v>
       </c>
     </row>
     <row r="17" spans="1:4" ht="55">
@@ -4089,7 +4056,7 @@
         <v>113</v>
       </c>
       <c r="D17" s="32" t="s">
-        <v>211</v>
+        <v>141</v>
       </c>
     </row>
     <row r="18" spans="1:4" ht="55">
@@ -4099,7 +4066,7 @@
         <v>114</v>
       </c>
       <c r="D18" s="32" t="s">
-        <v>212</v>
+        <v>142</v>
       </c>
     </row>
     <row r="19" spans="1:4" ht="44">
@@ -4109,7 +4076,7 @@
         <v>115</v>
       </c>
       <c r="D19" s="32" t="s">
-        <v>213</v>
+        <v>143</v>
       </c>
     </row>
     <row r="20" spans="1:4" ht="55">
@@ -4119,7 +4086,7 @@
         <v>116</v>
       </c>
       <c r="D20" s="28" t="s">
-        <v>214</v>
+        <v>144</v>
       </c>
     </row>
     <row r="22" spans="1:4">

</xml_diff>

<commit_message>
Restore original A1b device profile rows
</commit_message>
<xml_diff>
--- a/assignments/assA1.xlsx
+++ b/assignments/assA1.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Desktop\Design-of-Enterprise-IoT-design\assignments\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{60E66001-CA21-45A6-839F-5603F0F1426C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E73FCDEB-9EEB-4551-8974-53CB18744421}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="380" yWindow="380" windowWidth="19200" windowHeight="9970" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -22,7 +22,7 @@
   <definedNames>
     <definedName name="_xlnm.Print_Area" localSheetId="4">'IoT Connectivity'!$A$1:$D$20</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="3">'IoT Connectivity (network only)'!$A$1:$D$9</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="2">'IoT Device  Profile'!$A$1:$G$13</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="2">'IoT Device  Profile'!$A$1:$G$15</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="0">'Value Proposition'!$A$1:$B$20</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="1">'Value Proposition en'!$A$1:$B$20</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="4">'IoT Connectivity'!$1:$1</definedName>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="237" uniqueCount="207">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="251" uniqueCount="215">
   <si>
     <t>IoT solution: Smart Turtle Breeding System (STBS)</t>
   </si>
@@ -1245,274 +1245,374 @@
     <t>If the cloud connects with a system, what is the purpose of the connection?</t>
   </si>
   <si>
+    <t>20 tank instrument sets; 4 × Arduino Opta RS485 controllers with A0602/D1608 I/O; 20 Reolink RLC-811A PoE cameras; TP-Link TL-SG3428XMP managed PoE+ switch; AAEON BOXER-8653AI edge computer; Teltonika RUTX11 router.</t>
+  </si>
+  <si>
+    <t>Connectivity closes three loops: probes provide feedback to local control; controllers and cameras provide farm-wide context to the edge computer; selected events reach cloud users. It enables unit-specific alarms, verification of actuator outcomes, cross-unit comparison, nesting evidence and maintenance diagnostics. Safety interlocks remain in each Opta, so network loss reduces visibility rather than basic control.</t>
+  </si>
+  <si>
+    <t>Four RS-485 trunks each serve five nearby tanks and are deliberately kept below 100 m in a linear, terminated bus. Modbus guidance supports multidrop RS-485 and up to 32 unit loads per segment (Modbus Organization, 2006). Cat6 links from PLCs, cameras, edge computer and router remain within the 100 m copper-Ethernet channel limit. The control path does not depend on Wi-Fi coverage.</t>
+  </si>
+  <si>
+    <t>Mains is available, so continuity and protection matter more than battery life. A protected 24 VDC supply powers probes, PLCs and valves; PoE+ powers cameras; separate AC circuits feed heaters and pumps. A UPS supports PLCs, switch, edge computer and router for alarm delivery, buffering and orderly shutdown. Contactors, RCDs and manual isolation protect high-current loads.</t>
+  </si>
+  <si>
+    <t>Minute telemetry and state changes remain below 0.1 Mbit/s. Cameras dominate: 20 H.265 streams at about 4–8 Mbit/s each produce 80–160 Mbit/s aggregate. A gigabit backbone provides headroom. The edge analyses lower-rate substreams, keeps main streams local and uploads only selected event clips.</t>
+  </si>
+  <si>
+    <t>PLC interlocks and heater/valve decisions target sub-second local response. Local alarms and dashboard state should update within about 5 s. Cloud reports tolerate seconds to minutes. No safety action waits for a cloud round trip; cloud commands are authenticated requests that the edge and PLC revalidate against local limits.</t>
+  </si>
+  <si>
+    <t>The switch separates control, camera and management VLANs and applies ACLs, 802.1X/MAC controls and QoS. Its 24 PoE+ ports and 384 W budget cover 20 cameras with reserve (TP-Link, n.d.). Devices use unique credentials; unused services and camera P2P/UPnP are disabled; administration uses VPN. MQTT uses TLS and X.509 certificates. UPS power, watchdogs, local buffering, normally closed valves and Ethernet-primary/LTE-failover WAN improve resilience.</t>
+  </si>
+  <si>
+    <t>Wired installation and industrial probes cost more initially than hobby sensors or Wi-Fi, but reduce battery labour, interference and replacement risk in a wet fixed site. One managed PoE switch removes 20 camera power adapters. Four zone PLCs limit I/O cable length. Edge filtering avoids continuous video upload and reduces WAN, cloud-ingest and storage costs.</t>
+  </si>
+  <si>
+    <t>Field level: 4–20 mA for analogue probes; RS-485/Modbus RTU for multidrop sensors; pulse/UART for simple instruments; isolated relay/24 V control for actuators. Plant level: 1000BASE-T Cat6 and IEEE 802.3af/at PoE through a TP-Link TL-SG3428XMP (TP-Link, n.d.). WAN: Ethernet primary plus Teltonika RUTX11 dual-SIM LTE Cat 6 failover (Teltonika Networks, n.d.). Applications use local Modbus TCP/HTTPS/RTSP and outbound MQTT/TLS/HTTPS.</t>
+  </si>
+  <si>
+    <t>4 × Arduino Opta RS485 zone controllers; AAEON BOXER-8653AI industrial edge computer; TP-Link managed PoE+ switch; local operator web application; maintenance log/API.</t>
+  </si>
+  <si>
+    <t>Yes. Deterministic control must survive Internet loss, and 20 continuous video streams are too bandwidth-intensive and privacy-sensitive for routine cloud upload. Opta PLCs form the device edge; the BOXER is the farm fog node for protocol normalisation, quality checks, video inference, event correlation, short-term storage and store-and-forward delivery.</t>
+  </si>
+  <si>
+    <t>Each Opta executes five-tank control rules and exposes states over the isolated control VLAN. The AAEON BOXER-8653AI runs containerised acquisition, message brokering, rules, local dashboards and vision models. The managed switch and router forward and secure traffic but do not make animal-control decisions.</t>
+  </si>
+  <si>
+    <t>Probes send temperature, pH, turbidity, ammonia, level, flow, feed distance and humidity with timestamps and diagnostics. PLCs add set-points, relay states, accumulated flow, manual/automatic mode, watchdog and alarm codes. Cameras send H.265 RTSP substreams and event windows. The edge adds device identity, tank/zone context and quality flags.</t>
+  </si>
+  <si>
+    <t>PLCs scale signals, debounce pulses, check plausible ranges/rates, enforce hysteresis and time/volume bounds, and execute fail-safe control. The BOXER synchronises timestamps, detects stale or contradictory readings, aggregates summaries, correlates flow with level/valve state, infers activity/feeding/nesting candidates, queues messages during outages and retains rolling evidence locally.</t>
+  </si>
+  <si>
+    <t>On the farm LAN, authorised users see current tank status, local alarms, event video, acknowledgement state and bounded manual controls even during WAN loss. The fog node labels unsynchronised data and preserves operational visibility and intervention capability.</t>
+  </si>
+  <si>
+    <t>The fog service writes an append-only operations log and exports alarms, acknowledgements, maintenance flags, calibration due dates and actuator runtime through signed CSV/API. The maintenance system can create or close work orders but cannot issue raw heater, pump or valve commands.</t>
+  </si>
+  <si>
+    <t>AAEON BOXER-8653AI edge computer; Teltonika RUTX11 firewall/router; AWS IoT Core, time-series/object storage and rules; role-based web application; maintenance/work-order system.</t>
+  </si>
+  <si>
+    <t>Yes, but not for immediate safety. AWS provides durable off-site history, multi-user access, fleet identity, long-term comparison, reporting and notification integration. AWS IoT Core authenticates the edge through X.509 certificates, routes MQTT messages and maintains desired/reported state through device shadows (Amazon Web Services, n.d.).</t>
+  </si>
+  <si>
+    <t>The BOXER publishes validated minute summaries, state changes, alarms, acknowledgements, health/calibration metadata and daily aggregates by MQTT/TLS. Selected event thumbnails/clips and diagnostic bundles use HTTPS object upload. Raw continuous camera streams and high-frequency samples remain on site unless an authorised investigation requests them.</t>
+  </si>
+  <si>
+    <t>IoT rules route telemetry to time-series storage and alarms to notification workflows; object storage retains approved evidence clips. Cloud jobs calculate cross-unit baselines, growth-stage comparisons, sensor-drift indicators and feed/energy/water summaries. Device shadows retain configuration state, while audit records capture user changes and acknowledgements.</t>
+  </si>
+  <si>
+    <t>A role-based web application provides historical charts, unit comparison, alarm notifications, evidence links, weekly reports and audit history. Users may request bounded set-point changes; the cloud records the request, but the edge/PLC rejects stale, unauthorised or out-of-range values.</t>
+  </si>
+  <si>
+    <t>The cloud exports approved maintenance tickets, calibration schedules, equipment runtime, water/feed consumption and compliance summaries through an API or scheduled CSV. Only necessary identifiers and evidence are included. Return status can close a ticket, but the external system cannot issue raw actuator commands.</t>
+  </si>
+  <si>
     <t>Sensor</t>
+    <phoneticPr fontId="68" type="noConversion"/>
   </si>
   <si>
     <t>Water in each breeding tank</t>
+    <phoneticPr fontId="68" type="noConversion"/>
   </si>
   <si>
     <t>Water temperature</t>
+    <phoneticPr fontId="68" type="noConversion"/>
   </si>
   <si>
     <t>pH value</t>
+    <phoneticPr fontId="68" type="noConversion"/>
   </si>
   <si>
     <t>Turbidity</t>
+    <phoneticPr fontId="68" type="noConversion"/>
+  </si>
+  <si>
+    <t>DFRobot Submersible Water Level Sensor (KIT0139)</t>
+    <phoneticPr fontId="68" type="noConversion"/>
+  </si>
+  <si>
+    <t>Water depth and level</t>
+    <phoneticPr fontId="68" type="noConversion"/>
+  </si>
+  <si>
+    <t>0–5 m range; ±0.5% full scale; 4–20 mA; 12–36 VDC; IP68 stainless probe. (DFRobot, n.d.)</t>
+    <phoneticPr fontId="68" type="noConversion"/>
+  </si>
+  <si>
+    <t>Pressure probe, vented cable termination, stilling tube, 24 VDC supply, Opta analogue input</t>
+    <phoneticPr fontId="68" type="noConversion"/>
+  </si>
+  <si>
+    <t>Independent level feedback prevents overflow, excessive drainage and dry-running, and verifies bounded water-change commands.</t>
+    <phoneticPr fontId="68" type="noConversion"/>
+  </si>
+  <si>
+    <t>DFRobot Water Flow Sensor (SEN0217 / YF-S201)</t>
+    <phoneticPr fontId="68" type="noConversion"/>
+  </si>
+  <si>
+    <t>Tank inlet and drain pipes</t>
+    <phoneticPr fontId="68" type="noConversion"/>
+  </si>
+  <si>
+    <t>Flow rate and transferred volume</t>
+    <phoneticPr fontId="68" type="noConversion"/>
+  </si>
+  <si>
+    <t>1–30 L/min; Hall-effect pulse output; ±5% over 2–30 L/min; 3.5–12 VDC; 1/2-inch fitting. (DFRobot, n.d.)</t>
+    <phoneticPr fontId="68" type="noConversion"/>
+  </si>
+  <si>
+    <t>Two sensors per tank, service unions, screened low-voltage cable, Opta pulse inputs</t>
+    <phoneticPr fontId="68" type="noConversion"/>
+  </si>
+  <si>
+    <t>Inlet and drain totals cross-check level change and expose blocked pipes, pump faults or stuck valves while limiting exchanged volume.</t>
+    <phoneticPr fontId="68" type="noConversion"/>
+  </si>
+  <si>
+    <t>DFRobot A02YYUW Waterproof Ultrasonic Sensor (SEN0311)</t>
+    <phoneticPr fontId="68" type="noConversion"/>
+  </si>
+  <si>
+    <t>Feed in each zone hopper</t>
+    <phoneticPr fontId="68" type="noConversion"/>
+  </si>
+  <si>
+    <t>Remaining feed height</t>
+    <phoneticPr fontId="68" type="noConversion"/>
+  </si>
+  <si>
+    <t>3–450 cm range; 3 cm blind zone; ±1 cm; 100 ms response; IP67; 3.3–5 V UART. (DFRobot, n.d.)</t>
+    <phoneticPr fontId="68" type="noConversion"/>
+  </si>
+  <si>
+    <t>Top mount, dust shield, isolated UART interface, hopper-specific distance-to-fill calibration</t>
+    <phoneticPr fontId="68" type="noConversion"/>
+  </si>
+  <si>
+    <t>One sensor per zone hopper provides a low-feed alert. Calibration accounts for the sloped pellet surface and converts distance to an approximate fill percentage.</t>
+    <phoneticPr fontId="68" type="noConversion"/>
+  </si>
+  <si>
+    <t>Atlas Scientific EZO Humidity Probe (EZO-HUM-P-S)</t>
+    <phoneticPr fontId="68" type="noConversion"/>
+  </si>
+  <si>
+    <t>Air in each breeding/nesting zone</t>
+    <phoneticPr fontId="68" type="noConversion"/>
+  </si>
+  <si>
+    <t>Relative humidity and air temperature</t>
+    <phoneticPr fontId="68" type="noConversion"/>
+  </si>
+  <si>
+    <t>0–100% RH; stated ±2% RH from 5–95%; 3.3–5 V; UART/I2C; IP67 stainless probe. (Atlas Scientific, n.d.)</t>
+    <phoneticPr fontId="68" type="noConversion"/>
+  </si>
+  <si>
+    <t>Shielded placement away from spray, isolated interface, mounting bracket, periodic comparison check</t>
+    <phoneticPr fontId="68" type="noConversion"/>
+  </si>
+  <si>
+    <t>Zone humidity reveals condensation risk that can affect electronics and camera visibility, and provides context for nesting-area observations.</t>
+    <phoneticPr fontId="68" type="noConversion"/>
+  </si>
+  <si>
+    <t>Aqua Medic Titanium Heater 500 W</t>
+    <phoneticPr fontId="68" type="noConversion"/>
   </si>
   <si>
     <t>Actuator</t>
-  </si>
-  <si>
-    <t>20 tank instrument sets; 4 × Arduino Opta RS485 controllers with A0602/D1608 I/O; 20 Reolink RLC-811A PoE cameras; TP-Link TL-SG3428XMP managed PoE+ switch; AAEON BOXER-8653AI edge computer; Teltonika RUTX11 router.</t>
-  </si>
-  <si>
-    <t>Connectivity closes three loops: probes provide feedback to local control; controllers and cameras provide farm-wide context to the edge computer; selected events reach cloud users. It enables unit-specific alarms, verification of actuator outcomes, cross-unit comparison, nesting evidence and maintenance diagnostics. Safety interlocks remain in each Opta, so network loss reduces visibility rather than basic control.</t>
-  </si>
-  <si>
-    <t>Four RS-485 trunks each serve five nearby tanks and are deliberately kept below 100 m in a linear, terminated bus. Modbus guidance supports multidrop RS-485 and up to 32 unit loads per segment (Modbus Organization, 2006). Cat6 links from PLCs, cameras, edge computer and router remain within the 100 m copper-Ethernet channel limit. The control path does not depend on Wi-Fi coverage.</t>
-  </si>
-  <si>
-    <t>Mains is available, so continuity and protection matter more than battery life. A protected 24 VDC supply powers probes, PLCs and valves; PoE+ powers cameras; separate AC circuits feed heaters and pumps. A UPS supports PLCs, switch, edge computer and router for alarm delivery, buffering and orderly shutdown. Contactors, RCDs and manual isolation protect high-current loads.</t>
-  </si>
-  <si>
-    <t>Minute telemetry and state changes remain below 0.1 Mbit/s. Cameras dominate: 20 H.265 streams at about 4–8 Mbit/s each produce 80–160 Mbit/s aggregate. A gigabit backbone provides headroom. The edge analyses lower-rate substreams, keeps main streams local and uploads only selected event clips.</t>
-  </si>
-  <si>
-    <t>PLC interlocks and heater/valve decisions target sub-second local response. Local alarms and dashboard state should update within about 5 s. Cloud reports tolerate seconds to minutes. No safety action waits for a cloud round trip; cloud commands are authenticated requests that the edge and PLC revalidate against local limits.</t>
-  </si>
-  <si>
-    <t>The switch separates control, camera and management VLANs and applies ACLs, 802.1X/MAC controls and QoS. Its 24 PoE+ ports and 384 W budget cover 20 cameras with reserve (TP-Link, n.d.). Devices use unique credentials; unused services and camera P2P/UPnP are disabled; administration uses VPN. MQTT uses TLS and X.509 certificates. UPS power, watchdogs, local buffering, normally closed valves and Ethernet-primary/LTE-failover WAN improve resilience.</t>
-  </si>
-  <si>
-    <t>Wired installation and industrial probes cost more initially than hobby sensors or Wi-Fi, but reduce battery labour, interference and replacement risk in a wet fixed site. One managed PoE switch removes 20 camera power adapters. Four zone PLCs limit I/O cable length. Edge filtering avoids continuous video upload and reduces WAN, cloud-ingest and storage costs.</t>
-  </si>
-  <si>
-    <t>Field level: 4–20 mA for analogue probes; RS-485/Modbus RTU for multidrop sensors; pulse/UART for simple instruments; isolated relay/24 V control for actuators. Plant level: 1000BASE-T Cat6 and IEEE 802.3af/at PoE through a TP-Link TL-SG3428XMP (TP-Link, n.d.). WAN: Ethernet primary plus Teltonika RUTX11 dual-SIM LTE Cat 6 failover (Teltonika Networks, n.d.). Applications use local Modbus TCP/HTTPS/RTSP and outbound MQTT/TLS/HTTPS.</t>
-  </si>
-  <si>
-    <t>4 × Arduino Opta RS485 zone controllers; AAEON BOXER-8653AI industrial edge computer; TP-Link managed PoE+ switch; local operator web application; maintenance log/API.</t>
-  </si>
-  <si>
-    <t>Yes. Deterministic control must survive Internet loss, and 20 continuous video streams are too bandwidth-intensive and privacy-sensitive for routine cloud upload. Opta PLCs form the device edge; the BOXER is the farm fog node for protocol normalisation, quality checks, video inference, event correlation, short-term storage and store-and-forward delivery.</t>
-  </si>
-  <si>
-    <t>Each Opta executes five-tank control rules and exposes states over the isolated control VLAN. The AAEON BOXER-8653AI runs containerised acquisition, message brokering, rules, local dashboards and vision models. The managed switch and router forward and secure traffic but do not make animal-control decisions.</t>
-  </si>
-  <si>
-    <t>Probes send temperature, pH, turbidity, ammonia, level, flow, feed distance and humidity with timestamps and diagnostics. PLCs add set-points, relay states, accumulated flow, manual/automatic mode, watchdog and alarm codes. Cameras send H.265 RTSP substreams and event windows. The edge adds device identity, tank/zone context and quality flags.</t>
-  </si>
-  <si>
-    <t>PLCs scale signals, debounce pulses, check plausible ranges/rates, enforce hysteresis and time/volume bounds, and execute fail-safe control. The BOXER synchronises timestamps, detects stale or contradictory readings, aggregates summaries, correlates flow with level/valve state, infers activity/feeding/nesting candidates, queues messages during outages and retains rolling evidence locally.</t>
-  </si>
-  <si>
-    <t>On the farm LAN, authorised users see current tank status, local alarms, event video, acknowledgement state and bounded manual controls even during WAN loss. The fog node labels unsynchronised data and preserves operational visibility and intervention capability.</t>
-  </si>
-  <si>
-    <t>The fog service writes an append-only operations log and exports alarms, acknowledgements, maintenance flags, calibration due dates and actuator runtime through signed CSV/API. The maintenance system can create or close work orders but cannot issue raw heater, pump or valve commands.</t>
-  </si>
-  <si>
-    <t>AAEON BOXER-8653AI edge computer; Teltonika RUTX11 firewall/router; AWS IoT Core, time-series/object storage and rules; role-based web application; maintenance/work-order system.</t>
-  </si>
-  <si>
-    <t>Yes, but not for immediate safety. AWS provides durable off-site history, multi-user access, fleet identity, long-term comparison, reporting and notification integration. AWS IoT Core authenticates the edge through X.509 certificates, routes MQTT messages and maintains desired/reported state through device shadows (Amazon Web Services, n.d.).</t>
-  </si>
-  <si>
-    <t>The BOXER publishes validated minute summaries, state changes, alarms, acknowledgements, health/calibration metadata and daily aggregates by MQTT/TLS. Selected event thumbnails/clips and diagnostic bundles use HTTPS object upload. Raw continuous camera streams and high-frequency samples remain on site unless an authorised investigation requests them.</t>
-  </si>
-  <si>
-    <t>IoT rules route telemetry to time-series storage and alarms to notification workflows; object storage retains approved evidence clips. Cloud jobs calculate cross-unit baselines, growth-stage comparisons, sensor-drift indicators and feed/energy/water summaries. Device shadows retain configuration state, while audit records capture user changes and acknowledgements.</t>
-  </si>
-  <si>
-    <t>A role-based web application provides historical charts, unit comparison, alarm notifications, evidence links, weekly reports and audit history. Users may request bounded set-point changes; the cloud records the request, but the edge/PLC rejects stale, unauthorised or out-of-range values.</t>
-  </si>
-  <si>
-    <t>The cloud exports approved maintenance tickets, calibration schedules, equipment runtime, water/feed consumption and compliance summaries through an API or scheduled CSV. Only necessary identifiers and evidence are included. Return status can close a ticket, but the external system cannot issue raw actuator commands.</t>
-  </si>
-  <si>
-    <t>DFRobot DS18B20 Waterproof Temperature Sensor (BOS0042) / 防水温度传感器</t>
-  </si>
-  <si>
-    <t>Waterproof DS18B20 probe; 3–5 V; PH2.0-3P connector; sensing range −55 to 125 °C; display range −10 to 85 °C with ±0.5 °C stated error; requires a pull-up resistor. Source: DFRobot BOS0042.</t>
+    <phoneticPr fontId="68" type="noConversion"/>
+  </si>
+  <si>
+    <t>Heat input and water temperature</t>
+    <phoneticPr fontId="68" type="noConversion"/>
+  </si>
+  <si>
+    <t>500 W; 110–240 VAC; intended for about 1000–1500 L; external controller required. (Aqua Medic, n.d.)</t>
+    <phoneticPr fontId="68" type="noConversion"/>
+  </si>
+  <si>
+    <t>Titanium element, rated contactor, RCD, guarded mount, manual isolation, independent over-temperature cut-out</t>
+    <phoneticPr fontId="68" type="noConversion"/>
+  </si>
+  <si>
+    <t>Corrosion-resistant construction suits aquaculture. PLC control uses conservative hysteresis, while the independent cut-out remains the final safety layer.</t>
+    <phoneticPr fontId="68" type="noConversion"/>
+  </si>
+  <si>
+    <t>Bürkert Type 6213 EV Normally Closed Valve, 24 VDC</t>
+    <phoneticPr fontId="68" type="noConversion"/>
+  </si>
+  <si>
+    <t>Tank inlet and drain lines</t>
+    <phoneticPr fontId="68" type="noConversion"/>
+  </si>
+  <si>
+    <t>Water flow state</t>
+    <phoneticPr fontId="68" type="noConversion"/>
+  </si>
+  <si>
+    <t>Two-way servo-assisted diaphragm valve; normally closed; 24 VDC option; water service; IP65 with suitable plug. (Bürkert, n.d.)</t>
+    <phoneticPr fontId="68" type="noConversion"/>
+  </si>
+  <si>
+    <t>Two valves per tank, selected DN/pressure variant, coil suppression, manual isolation, upstream strainer</t>
+    <phoneticPr fontId="68" type="noConversion"/>
+  </si>
+  <si>
+    <t>Normally closed action fails safe on power loss. Paired with level and flow feedback, it enables bounded partial water exchange.</t>
+    <phoneticPr fontId="68" type="noConversion"/>
+  </si>
+  <si>
+    <t>Actuator / device</t>
+    <phoneticPr fontId="68" type="noConversion"/>
+  </si>
+  <si>
+    <t>Feed supplied to turtles in each zone</t>
+    <phoneticPr fontId="68" type="noConversion"/>
+  </si>
+  <si>
+    <t>Feeding time and estimated portion</t>
+    <phoneticPr fontId="68" type="noConversion"/>
+  </si>
+  <si>
+    <t>Turtle activity, feeding and nesting areas</t>
+    <phoneticPr fontId="68" type="noConversion"/>
+  </si>
+  <si>
+    <t>Video and event evidence</t>
+    <phoneticPr fontId="68" type="noConversion"/>
+  </si>
+  <si>
+    <t>AXIS M3086-V Network Camera</t>
+    <phoneticPr fontId="68" type="noConversion"/>
+  </si>
+  <si>
+    <t>4 MP maximum resolution 2688x1512; 2.4 mm F2.1 lens; 130 deg horizontal and 93 deg vertical field of view; H.264/H.265/Motion JPEG; 25/30 fps; WDR up to 120 dB; Lightfinder; PoE Class 2; IP42 and IK08.</t>
+    <phoneticPr fontId="68" type="noConversion"/>
+  </si>
+  <si>
+    <t>Network camera, lens, PoE RJ45 connector, SD-card slot, control button, mounting dome and managed-switch port.</t>
+    <phoneticPr fontId="68" type="noConversion"/>
+  </si>
+  <si>
+    <t>Video provides farm-wide context and event evidence for activity, feeding and nesting. PoE simplifies installation; edge analytics retain only validated clips rather than upload continuous video.</t>
+    <phoneticPr fontId="68" type="noConversion"/>
+  </si>
+  <si>
+    <t>PondMAX Solar Automatic Fish Feeder</t>
+    <phoneticPr fontId="68" type="noConversion"/>
+  </si>
+  <si>
+    <t>Solar charging with built-in 2200 mAh lithium battery; 1-6 feedings per day; adjustable S/M/L throw and 0-20 s feed duration; 3-10 mm food size; 12 V/1.66 A adapter specification.</t>
+    <phoneticPr fontId="68" type="noConversion"/>
+  </si>
+  <si>
+    <t>Solar panel, rechargeable battery, hopper, motor and spreader, timer/display controls, protective cover and mounting bracket.</t>
+    <phoneticPr fontId="68" type="noConversion"/>
+  </si>
+  <si>
+    <t>Automated feeding improves schedule consistency and reduces manual labour. Feed commands remain bounded by time, quantity and hopper checks, with operator override and audit records.</t>
+    <phoneticPr fontId="68" type="noConversion"/>
+  </si>
+  <si>
+    <t>Lonhand LH-WQS-AN-485-UI NH3-N Sensor</t>
+    <phoneticPr fontId="68" type="noConversion"/>
+  </si>
+  <si>
+    <t>Ammonia-nitrogen concentration</t>
+    <phoneticPr fontId="68" type="noConversion"/>
+  </si>
+  <si>
+    <t>Measurement range 0.1-18,000 mg/L; temperature range 0-60 deg C; 4-20 mA and RS-485 outputs; IP68; 5 m cable; NPT3/4 or M39x1.5 connection; 0-3 bar; pH 4-10; repeatability +/-4%; PC/PBT housing.</t>
+    <phoneticPr fontId="68" type="noConversion"/>
+  </si>
+  <si>
+    <t>Ion-selective ammonia electrode, 4-20 mA/RS-485 transmitter, 5 m cable, immersion fitting, PLC analogue/Modbus input and calibration solution.</t>
+    <phoneticPr fontId="68" type="noConversion"/>
+  </si>
+  <si>
+    <t>Ammonia is a high-risk water-quality condition. A wired industrial output supports continuous trend logging, local alarm thresholds and dependable response when the network is unavailable.</t>
+    <phoneticPr fontId="68" type="noConversion"/>
+  </si>
+  <si>
+    <t>DFRobot SEN0189 Turbidity Sensor</t>
+    <phoneticPr fontId="68" type="noConversion"/>
+  </si>
+  <si>
+    <t>Optical infrared emitter/receiver; 5 VDC; 40 mA maximum; response below 500 ms; selectable analogue 0-4.5 V or thresholded digital output; operating range -30 to 80 deg C; probe top is not waterproof.</t>
+    <phoneticPr fontId="68" type="noConversion"/>
+  </si>
+  <si>
+    <t>Optical turbidity probe, interface board, A/D or GPIO input, analogue/digital selector and threshold potentiometer.</t>
+    <phoneticPr fontId="68" type="noConversion"/>
+  </si>
+  <si>
+    <t>Provides early warning of suspended solids, filtration faults and contamination. Digital threshold alarms can be local, while analogue values support trend analysis and water-change decisions.</t>
+    <phoneticPr fontId="68" type="noConversion"/>
+  </si>
+  <si>
+    <t>DFRobot SEN0161-V2 Gravity Analog pH Meter</t>
+    <phoneticPr fontId="68" type="noConversion"/>
+  </si>
+  <si>
+    <t>Signal-board supply 3.3-5.5 V; analogue output 0-3.0 V; BNC electrode and PH2.0-3P signal connector; stated accuracy +/-0.1 at 25 deg C; electrode range pH 0-14 and 5-60 deg C; response below 2 min; 1 m cable.</t>
+    <phoneticPr fontId="68" type="noConversion"/>
+  </si>
+  <si>
+    <t>Laboratory-grade pH electrode, V2 signal-conversion board, BNC cable, PH2.0-3P lead, calibration buffers and analogue input.</t>
+    <phoneticPr fontId="68" type="noConversion"/>
+  </si>
+  <si>
+    <t>pH is a key water-quality variable for aquaculture. Two-point calibration and local plausibility/rate checks allow the PLC to alarm and bound corrective actions.</t>
+    <phoneticPr fontId="68" type="noConversion"/>
+  </si>
+  <si>
+    <t>DFRobot Waterproof DS18B20 Temperature Sensor (BOS0042)</t>
+    <phoneticPr fontId="68" type="noConversion"/>
+  </si>
+  <si>
+    <t>Waterproof DS18B20 probe; 3-5 V; PH2.0-3P connector; sensing range -55 to 125 deg C; display range -10 to 85 deg C; stated error +/-0.5 deg C; pull-up resistor required.</t>
+    <phoneticPr fontId="68" type="noConversion"/>
   </si>
   <si>
     <t>Waterproof DS18B20 probe, 3-pin cable, pull-up resistor, PH2.0 adapter and controller input.</t>
-  </si>
-  <si>
-    <t>Direct temperature feedback supports heater control and alarm limits in wet tanks. The sealed probe is suitable for remote or humid measurement, while local validation prevents unsafe heating commands.</t>
-  </si>
-  <si>
-    <t>DFRobot SEN0189 Turbidity Sensor / 浑浊度传感器</t>
-  </si>
-  <si>
-    <t>Water clarity in each breeding tank</t>
-  </si>
-  <si>
-    <t>Optical infrared emitter/receiver; 5 VDC; 40 mA maximum; response below 500 ms; selectable analogue 0–4.5 V or thresholded digital output; operating range −30 to 80 °C. The probe top is not waterproof.</t>
-  </si>
-  <si>
-    <t>Optical turbidity probe, interface board, A/D or GPIO input, analogue/digital selector and threshold potentiometer.</t>
-  </si>
-  <si>
-    <t>Provides an early warning of suspended solids, filtration faults and contamination. Digital threshold alarms can be local, while analogue values support trend analysis and water-change decisions.</t>
-  </si>
-  <si>
-    <t>DFRobot SEN0161-V2 Gravity Analog pH Meter / 模拟 pH 计 V2</t>
-  </si>
-  <si>
-    <t>Water chemistry in each breeding tank</t>
-  </si>
-  <si>
-    <t>Signal board supply 3.3–5.5 V; analogue output 0–3.0 V; BNC electrode and PH2.0-3P signal connector; stated accuracy ±0.1 at 25 °C; electrode range pH 0–14, 5–60 °C, response below 2 min; 1 m cable.</t>
-  </si>
-  <si>
-    <t>Laboratory-grade pH electrode, V2 signal-conversion board, BNC cable, PH2.0-3P lead, calibration buffers and analogue input.</t>
-  </si>
-  <si>
-    <t>pH is a key water-quality variable for aquaculture. Two-point calibration and local plausibility/rate checks allow the PLC to alarm and bound corrective actions.</t>
-  </si>
-  <si>
-    <t>Lonhand LH-WQS-AN-485-UI NH3-N Ion Sensor / 氨氮离子传感器</t>
-  </si>
-  <si>
-    <t>Ammonia-nitrogen concentration</t>
-  </si>
-  <si>
-    <t>Measurement range 0.1–18,000 mg/L; temperature range 0–60 °C; 4–20 mA and RS-485 outputs; IP68; 5 m cable; NPT3/4 or M39×1.5 connection; 0–3 bar; pH 4–10; repeatability ±4%; PC/PBT corrosion-resistant housing.</t>
-  </si>
-  <si>
-    <t>Ion-selective ammonia electrode, 4–20 mA/RS-485 transmitter, 5 m cable, immersion fitting, PLC analogue/Modbus input and calibration solution.</t>
-  </si>
-  <si>
-    <t>Ammonia is a high-risk water-quality condition. A wired industrial output supports continuous trend logging, local alarm thresholds and dependable response even when the network is unavailable.</t>
-  </si>
-  <si>
-    <t>AXIS M3086-V Network Camera / 网络摄像机</t>
-  </si>
-  <si>
-    <t>Breeding and nesting-zone activity and evidence</t>
-  </si>
-  <si>
-    <t>Video stream and event evidence</t>
-  </si>
-  <si>
-    <t>4 MP maximum resolution 2688×1512; 2.4 mm F2.1 lens; 130° horizontal and 93° vertical field of view; H.264/H.265/Motion JPEG; 25/30 fps; WDR up to 120 dB; Lightfinder; PoE Class 2; IP42 and IK08 variants.</t>
-  </si>
-  <si>
-    <t>Network camera, lens, PoE RJ45 connector, SD-card slot, control button, mounting dome and managed-switch port.</t>
-  </si>
-  <si>
-    <t>Video provides farm-wide context and event evidence for activity, feeding and nesting. PoE simplifies installation; edge analytics should retain only validated clips rather than upload continuous video.</t>
-  </si>
-  <si>
-    <t>Raspberry Pi 5 (8 GB)</t>
-  </si>
-  <si>
-    <t>Device</t>
-  </si>
-  <si>
-    <t>Edge gateway and local sensor aggregation</t>
-  </si>
-  <si>
-    <t>Local processing, protocol bridging and storage</t>
-  </si>
-  <si>
-    <t>Broadcom BCM2712 2.4 GHz quad-core 64-bit Arm Cortex-A76; 8 GB LPDDR4X-4267; standard 40-pin GPIO header; USB, Ethernet, Wi-Fi and Bluetooth; 5 V USB-C power and active cooling recommended for sustained workloads.</t>
-  </si>
-  <si>
-    <t>Raspberry Pi 5 board, microSD or SSD, 40-pin GPIO interface, USB/Ethernet/Wi-Fi links, power supply, case and active cooler.</t>
-  </si>
-  <si>
-    <t>A low-cost Linux edge node can bridge sensors, MQTT and dashboards, buffer data and pre-process camera events. Safety-critical interlocks remain in the dedicated PLC rather than the general-purpose board.</t>
-  </si>
-  <si>
-    <t>ESP32-WROOM-32</t>
-  </si>
-  <si>
-    <t>Distributed sensor and low-power actuator nodes</t>
-  </si>
-  <si>
-    <t>Wireless telemetry and GPIO control</t>
-  </si>
-  <si>
-    <t>Dual-core Xtensa LX6 up to 240 MHz; 448 KB ROM, 520 KB SRAM and 4 MB SPI flash; 2.4 GHz 802.11 b/g/n up to 150 Mbps; Bluetooth 4.2/BLE; up to 32 GPIO; ADC, DAC, touch, PWM and serial peripherals; 3.0–3.6 V supply.</t>
-  </si>
-  <si>
-    <t>ESP32-WROOM-32 module, PCB antenna, 40 MHz crystal, flash, GPIO/ADC interface, regulated 3.3 V supply and enclosure.</t>
-  </si>
-  <si>
-    <t>Provides an economical wireless interface for non-critical distributed measurements. Wet-area deployments still need isolation, watchdogs and bounded local outputs before any actuator command is accepted.</t>
-  </si>
-  <si>
-    <t>Ubuntu Server 22.04</t>
-  </si>
-  <si>
-    <t>Edge/server software platform</t>
-  </si>
-  <si>
-    <t>Container, storage, MQTT and API runtime</t>
-  </si>
-  <si>
-    <t>Ubuntu Server 22.04 LTS provides a maintainable Linux base for scale-out services, networking, storage, containers and system administration. The workload can run on Raspberry Pi 5 or another supported ARM/x86 host.</t>
-  </si>
-  <si>
-    <t>Ubuntu Server image, host storage, network interface, container runtime, MQTT broker, time-series database, API service and monitoring.</t>
-  </si>
-  <si>
-    <t>A documented LTS platform supports repeatable deployment, security updates and service separation for the edge gateway. It improves maintainability without placing deterministic safety control in the operating system.</t>
-  </si>
-  <si>
-    <t>HC-SR501 PIR Motion Sensor / 人体红外传感器</t>
-  </si>
-  <si>
-    <t>Activity in breeding or nesting areas</t>
-  </si>
-  <si>
-    <t>Motion event</t>
-  </si>
-  <si>
-    <t>Pyroelectric dual-element PIR module; 4.5–20 V supply; below 50 µA stated current; 3.3 V high/0 V low GPIO output; cone below 100°; three pins; selectable repeatable/non-repeatable trigger and adjustable delay/sensitivity.</t>
-  </si>
-  <si>
-    <t>PIR element, Fresnel lens, comparator board, delay and sensitivity potentiometers, VCC/OUT/GND header and GPIO input.</t>
-  </si>
-  <si>
-    <t>A low-cost motion trigger can wake or tag camera recording and reduce continuous processing. It is not a safety sensor because initialization time, wind, lighting and animal movement can cause false or missed events.</t>
-  </si>
-  <si>
-    <t>PondMAX Solar Automatic Fish Feeder</t>
-  </si>
-  <si>
-    <t>Feed hopper and pond feeding schedule</t>
-  </si>
-  <si>
-    <t>Scheduled feed dispensing</t>
-  </si>
-  <si>
-    <t>Solar charging with built-in 2200 mAh lithium battery; 1–6 feedings per day; adjustable S/M/L throw and 0–20 s feed duration; 3–10 mm food size; 12 V/1.66 A adapter specification in the supplied manual.</t>
-  </si>
-  <si>
-    <t>Solar panel, rechargeable battery, hopper, motor and spreader, timer/display controls, protective cover and mounting bracket.</t>
-  </si>
-  <si>
-    <t>Automated feeding improves schedule consistency and reduces manual labour. Feed commands should remain bounded by time, quantity and hopper checks, with an operator override and an audit record.</t>
-  </si>
-  <si>
-    <t>Bluefish MINI-200 Submersible Pump / 潜水泵</t>
+    <phoneticPr fontId="68" type="noConversion"/>
+  </si>
+  <si>
+    <t>Direct temperature feedback supports heater control and alarm limits in wet tanks. The sealed probe suits remote or humid measurement, while local validation prevents unsafe heating commands.</t>
+    <phoneticPr fontId="68" type="noConversion"/>
+  </si>
+  <si>
+    <t>Bluefish MINI-200 Submersible Pump</t>
+    <phoneticPr fontId="68" type="noConversion"/>
   </si>
   <si>
     <t>Tank recirculation and water-change line</t>
+    <phoneticPr fontId="68" type="noConversion"/>
   </si>
   <si>
     <t>Water circulation and flow</t>
-  </si>
-  <si>
-    <t>12 VDC; 0.4 A; 4.8 W; 200 L/h open flow; 1.5 m maximum head; brushless motor; IP68 submersible construction; approximately 43×38×30 mm; below 35 dB; dry-run/block protection options.</t>
+    <phoneticPr fontId="68" type="noConversion"/>
+  </si>
+  <si>
+    <t>12 VDC; 0.4 A; 4.8 W; 200 L/h open flow; 1.5 m maximum head; brushless motor; IP68 submersible construction; approximately 43x38x30 mm; below 35 dB; dry-run/block protection options.</t>
+    <phoneticPr fontId="68" type="noConversion"/>
   </si>
   <si>
     <t>Brushless pump, impeller, inlet/outlet, sealed motor, silicone vibration feet, 12 V supply, relay/MOSFET driver and flow feedback.</t>
+    <phoneticPr fontId="68" type="noConversion"/>
   </si>
   <si>
     <t>Low-voltage circulation supports filtration and controlled water changes. A relay, flow confirmation and dry-run protection prevent a blocked line or empty tank from damaging the pump.</t>
+    <phoneticPr fontId="68" type="noConversion"/>
   </si>
 </sst>
 </file>
@@ -2566,7 +2666,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="58">
+  <cellXfs count="56">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -2732,12 +2832,6 @@
     </xf>
     <xf numFmtId="0" fontId="43" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="17" xfId="6" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="38" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="49">
@@ -3421,295 +3515,310 @@
         <v>86</v>
       </c>
     </row>
-    <row r="3" spans="1:7" ht="120" customHeight="1">
-      <c r="A3" s="56" t="s">
+    <row r="3" spans="1:7" ht="100" customHeight="1">
+      <c r="A3" s="24" t="s">
+        <v>205</v>
+      </c>
+      <c r="B3" s="23" t="s">
+        <v>139</v>
+      </c>
+      <c r="C3" s="23" t="s">
+        <v>140</v>
+      </c>
+      <c r="D3" s="23" t="s">
+        <v>141</v>
+      </c>
+      <c r="E3" s="23" t="s">
+        <v>206</v>
+      </c>
+      <c r="F3" s="23" t="s">
+        <v>207</v>
+      </c>
+      <c r="G3" s="23" t="s">
+        <v>208</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" ht="100" customHeight="1">
+      <c r="A4" s="24" t="s">
+        <v>201</v>
+      </c>
+      <c r="B4" s="23" t="s">
+        <v>139</v>
+      </c>
+      <c r="C4" s="23" t="s">
+        <v>140</v>
+      </c>
+      <c r="D4" s="23" t="s">
+        <v>142</v>
+      </c>
+      <c r="E4" s="23" t="s">
+        <v>202</v>
+      </c>
+      <c r="F4" s="23" t="s">
+        <v>203</v>
+      </c>
+      <c r="G4" s="23" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" ht="100" customHeight="1">
+      <c r="A5" s="24" t="s">
+        <v>197</v>
+      </c>
+      <c r="B5" s="23" t="s">
+        <v>139</v>
+      </c>
+      <c r="C5" s="23" t="s">
+        <v>140</v>
+      </c>
+      <c r="D5" s="23" t="s">
+        <v>143</v>
+      </c>
+      <c r="E5" s="23" t="s">
+        <v>198</v>
+      </c>
+      <c r="F5" s="23" t="s">
+        <v>199</v>
+      </c>
+      <c r="G5" s="23" t="s">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" ht="110" customHeight="1">
+      <c r="A6" s="24" t="s">
+        <v>192</v>
+      </c>
+      <c r="B6" s="23" t="s">
+        <v>139</v>
+      </c>
+      <c r="C6" s="23" t="s">
+        <v>140</v>
+      </c>
+      <c r="D6" s="23" t="s">
+        <v>193</v>
+      </c>
+      <c r="E6" s="23" t="s">
+        <v>194</v>
+      </c>
+      <c r="F6" s="23" t="s">
+        <v>195</v>
+      </c>
+      <c r="G6" s="23" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" ht="75" customHeight="1">
+      <c r="A7" s="24" t="s">
+        <v>144</v>
+      </c>
+      <c r="B7" s="23" t="s">
+        <v>139</v>
+      </c>
+      <c r="C7" s="23" t="s">
+        <v>140</v>
+      </c>
+      <c r="D7" s="23" t="s">
         <v>145</v>
       </c>
-      <c r="B3" s="57" t="s">
-        <v>117</v>
-      </c>
-      <c r="C3" s="23" t="s">
-        <v>118</v>
-      </c>
-      <c r="D3" s="23" t="s">
-        <v>119</v>
-      </c>
-      <c r="E3" s="23" t="s">
+      <c r="E7" s="23" t="s">
         <v>146</v>
       </c>
-      <c r="F3" s="23" t="s">
+      <c r="F7" s="23" t="s">
         <v>147</v>
       </c>
-      <c r="G3" s="23" t="s">
+      <c r="G7" s="23" t="s">
         <v>148</v>
       </c>
     </row>
-    <row r="4" spans="1:7" ht="99" customHeight="1">
-      <c r="A4" s="56" t="s">
+    <row r="8" spans="1:7" ht="75" customHeight="1">
+      <c r="A8" s="24" t="s">
         <v>149</v>
       </c>
-      <c r="B4" s="57" t="s">
-        <v>117</v>
-      </c>
-      <c r="C4" s="23" t="s">
+      <c r="B8" s="23" t="s">
+        <v>139</v>
+      </c>
+      <c r="C8" s="23" t="s">
         <v>150</v>
       </c>
-      <c r="D4" s="23" t="s">
-        <v>121</v>
-      </c>
-      <c r="E4" s="23" t="s">
+      <c r="D8" s="23" t="s">
         <v>151</v>
       </c>
-      <c r="F4" s="23" t="s">
+      <c r="E8" s="23" t="s">
         <v>152</v>
       </c>
-      <c r="G4" s="23" t="s">
+      <c r="F8" s="23" t="s">
         <v>153</v>
       </c>
-    </row>
-    <row r="5" spans="1:7" ht="101" customHeight="1">
-      <c r="A5" s="56" t="s">
+      <c r="G8" s="23" t="s">
         <v>154</v>
       </c>
-      <c r="B5" s="57" t="s">
-        <v>117</v>
-      </c>
-      <c r="C5" s="23" t="s">
+    </row>
+    <row r="9" spans="1:7" ht="85" customHeight="1">
+      <c r="A9" s="24" t="s">
         <v>155</v>
       </c>
-      <c r="D5" s="23" t="s">
-        <v>120</v>
-      </c>
-      <c r="E5" s="23" t="s">
+      <c r="B9" s="23" t="s">
+        <v>139</v>
+      </c>
+      <c r="C9" s="23" t="s">
         <v>156</v>
       </c>
-      <c r="F5" s="23" t="s">
+      <c r="D9" s="23" t="s">
         <v>157</v>
       </c>
-      <c r="G5" s="23" t="s">
+      <c r="E9" s="23" t="s">
         <v>158</v>
       </c>
-    </row>
-    <row r="6" spans="1:7" ht="101" customHeight="1">
-      <c r="A6" s="56" t="s">
+      <c r="F9" s="23" t="s">
         <v>159</v>
       </c>
-      <c r="B6" s="57" t="s">
-        <v>117</v>
-      </c>
-      <c r="C6" s="23" t="s">
-        <v>155</v>
-      </c>
-      <c r="D6" s="23" t="s">
+      <c r="G9" s="23" t="s">
         <v>160</v>
       </c>
-      <c r="E6" s="23" t="s">
+    </row>
+    <row r="10" spans="1:7" ht="85" customHeight="1">
+      <c r="A10" s="24" t="s">
         <v>161</v>
       </c>
-      <c r="F6" s="23" t="s">
+      <c r="B10" s="23" t="s">
+        <v>139</v>
+      </c>
+      <c r="C10" s="23" t="s">
         <v>162</v>
       </c>
-      <c r="G6" s="23" t="s">
+      <c r="D10" s="23" t="s">
         <v>163</v>
       </c>
-    </row>
-    <row r="7" spans="1:7" ht="99" customHeight="1">
-      <c r="A7" s="56" t="s">
+      <c r="E10" s="23" t="s">
         <v>164</v>
       </c>
-      <c r="B7" s="57" t="s">
-        <v>117</v>
-      </c>
-      <c r="C7" s="23" t="s">
+      <c r="F10" s="23" t="s">
         <v>165</v>
       </c>
-      <c r="D7" s="23" t="s">
+      <c r="G10" s="23" t="s">
         <v>166</v>
       </c>
-      <c r="E7" s="23" t="s">
+    </row>
+    <row r="11" spans="1:7" ht="75" customHeight="1">
+      <c r="A11" s="24" t="s">
         <v>167</v>
       </c>
-      <c r="F7" s="23" t="s">
+      <c r="B11" s="23" t="s">
         <v>168</v>
       </c>
-      <c r="G7" s="23" t="s">
+      <c r="C11" s="23" t="s">
+        <v>140</v>
+      </c>
+      <c r="D11" s="23" t="s">
         <v>169</v>
       </c>
-    </row>
-    <row r="8" spans="1:7" ht="99" customHeight="1">
-      <c r="A8" s="56" t="s">
+      <c r="E11" s="23" t="s">
         <v>170</v>
       </c>
-      <c r="B8" s="57" t="s">
+      <c r="F11" s="23" t="s">
         <v>171</v>
       </c>
-      <c r="C8" s="23" t="s">
+      <c r="G11" s="23" t="s">
         <v>172</v>
       </c>
-      <c r="D8" s="23" t="s">
+    </row>
+    <row r="12" spans="1:7" ht="100" customHeight="1">
+      <c r="A12" s="24" t="s">
+        <v>209</v>
+      </c>
+      <c r="B12" s="23" t="s">
+        <v>168</v>
+      </c>
+      <c r="C12" s="23" t="s">
+        <v>210</v>
+      </c>
+      <c r="D12" s="23" t="s">
+        <v>211</v>
+      </c>
+      <c r="E12" s="23" t="s">
+        <v>212</v>
+      </c>
+      <c r="F12" s="23" t="s">
+        <v>213</v>
+      </c>
+      <c r="G12" s="23" t="s">
+        <v>214</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" ht="75" customHeight="1">
+      <c r="A13" s="24" t="s">
         <v>173</v>
       </c>
-      <c r="E8" s="23" t="s">
+      <c r="B13" s="23" t="s">
+        <v>168</v>
+      </c>
+      <c r="C13" s="23" t="s">
         <v>174</v>
       </c>
-      <c r="F8" s="23" t="s">
+      <c r="D13" s="23" t="s">
         <v>175</v>
       </c>
-      <c r="G8" s="23" t="s">
+      <c r="E13" s="23" t="s">
         <v>176</v>
       </c>
-    </row>
-    <row r="9" spans="1:7" ht="99" customHeight="1">
-      <c r="A9" s="56" t="s">
+      <c r="F13" s="23" t="s">
         <v>177</v>
       </c>
-      <c r="B9" s="57" t="s">
-        <v>171</v>
-      </c>
-      <c r="C9" s="23" t="s">
+      <c r="G13" s="23" t="s">
         <v>178</v>
       </c>
-      <c r="D9" s="23" t="s">
+    </row>
+    <row r="14" spans="1:7" ht="100" customHeight="1">
+      <c r="A14" s="24" t="s">
+        <v>188</v>
+      </c>
+      <c r="B14" s="23" t="s">
         <v>179</v>
       </c>
-      <c r="E9" s="23" t="s">
+      <c r="C14" s="23" t="s">
         <v>180</v>
       </c>
-      <c r="F9" s="23" t="s">
+      <c r="D14" s="23" t="s">
         <v>181</v>
       </c>
-      <c r="G9" s="23" t="s">
+      <c r="E14" s="23" t="s">
+        <v>189</v>
+      </c>
+      <c r="F14" s="23" t="s">
+        <v>190</v>
+      </c>
+      <c r="G14" s="23" t="s">
+        <v>191</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7" ht="100" customHeight="1">
+      <c r="A15" s="24" t="s">
+        <v>184</v>
+      </c>
+      <c r="B15" s="23" t="s">
+        <v>139</v>
+      </c>
+      <c r="C15" s="23" t="s">
         <v>182</v>
       </c>
-    </row>
-    <row r="10" spans="1:7" ht="119" customHeight="1">
-      <c r="A10" s="56" t="s">
+      <c r="D15" s="23" t="s">
         <v>183</v>
       </c>
-      <c r="B10" s="57" t="s">
-        <v>171</v>
-      </c>
-      <c r="C10" s="23" t="s">
-        <v>184</v>
-      </c>
-      <c r="D10" s="23" t="s">
+      <c r="E15" s="23" t="s">
         <v>185</v>
       </c>
-      <c r="E10" s="23" t="s">
+      <c r="F15" s="23" t="s">
         <v>186</v>
       </c>
-      <c r="F10" s="23" t="s">
+      <c r="G15" s="23" t="s">
         <v>187</v>
       </c>
-      <c r="G10" s="23" t="s">
-        <v>188</v>
-      </c>
-    </row>
-    <row r="11" spans="1:7" ht="99" customHeight="1">
-      <c r="A11" s="56" t="s">
-        <v>189</v>
-      </c>
-      <c r="B11" s="57" t="s">
-        <v>117</v>
-      </c>
-      <c r="C11" s="23" t="s">
-        <v>190</v>
-      </c>
-      <c r="D11" s="23" t="s">
-        <v>191</v>
-      </c>
-      <c r="E11" s="23" t="s">
-        <v>192</v>
-      </c>
-      <c r="F11" s="23" t="s">
-        <v>193</v>
-      </c>
-      <c r="G11" s="23" t="s">
-        <v>194</v>
-      </c>
-    </row>
-    <row r="12" spans="1:7" ht="99" customHeight="1">
-      <c r="A12" s="56" t="s">
-        <v>195</v>
-      </c>
-      <c r="B12" s="57" t="s">
-        <v>122</v>
-      </c>
-      <c r="C12" s="23" t="s">
-        <v>196</v>
-      </c>
-      <c r="D12" s="23" t="s">
-        <v>197</v>
-      </c>
-      <c r="E12" s="23" t="s">
-        <v>198</v>
-      </c>
-      <c r="F12" s="23" t="s">
-        <v>199</v>
-      </c>
-      <c r="G12" s="23" t="s">
-        <v>200</v>
-      </c>
-    </row>
-    <row r="13" spans="1:7" ht="99" customHeight="1">
-      <c r="A13" s="56" t="s">
-        <v>201</v>
-      </c>
-      <c r="B13" s="57" t="s">
-        <v>122</v>
-      </c>
-      <c r="C13" s="23" t="s">
-        <v>202</v>
-      </c>
-      <c r="D13" s="23" t="s">
-        <v>203</v>
-      </c>
-      <c r="E13" s="23" t="s">
-        <v>204</v>
-      </c>
-      <c r="F13" s="23" t="s">
-        <v>205</v>
-      </c>
-      <c r="G13" s="23" t="s">
-        <v>206</v>
-      </c>
-    </row>
-    <row r="14" spans="1:7" ht="80" customHeight="1">
-      <c r="A14" s="24"/>
-      <c r="B14" s="23"/>
-      <c r="C14" s="23"/>
-      <c r="D14" s="23"/>
-      <c r="E14" s="23"/>
-      <c r="F14" s="23"/>
-      <c r="G14" s="23"/>
-    </row>
-    <row r="15" spans="1:7" ht="80" customHeight="1">
-      <c r="A15" s="24"/>
-      <c r="B15" s="23"/>
-      <c r="C15" s="23"/>
-      <c r="D15" s="23"/>
-      <c r="E15" s="23"/>
-      <c r="F15" s="23"/>
-      <c r="G15" s="23"/>
     </row>
   </sheetData>
   <phoneticPr fontId="68" type="noConversion"/>
-  <hyperlinks>
-    <hyperlink ref="A3" r:id="rId1" tooltip="Open source page" xr:uid="{42A0E00C-B42D-41EB-B276-EAECFC050B15}"/>
-    <hyperlink ref="A4" r:id="rId2" tooltip="Open source page" xr:uid="{0938D27D-A9A4-4FBF-8D46-D0AA28FCA6A2}"/>
-    <hyperlink ref="A5" r:id="rId3" tooltip="Open source page" xr:uid="{97966CAD-7DF6-44C8-9A6F-4AB23F8E9875}"/>
-    <hyperlink ref="A6" r:id="rId4" tooltip="Open source page" xr:uid="{EB77D51A-1541-4CEC-BA09-17BACE2419A3}"/>
-    <hyperlink ref="A7" r:id="rId5" tooltip="Open source page" xr:uid="{B8F21E40-6BE4-425D-813F-DCB8AB7D9786}"/>
-    <hyperlink ref="A8" r:id="rId6" tooltip="Open source page" xr:uid="{D1B738E5-B5F5-46BF-BFF4-F587A7C72FDB}"/>
-    <hyperlink ref="A9" r:id="rId7" tooltip="Open source page" xr:uid="{C300A4E9-D4C0-449D-9036-D3ED8F1A6E2E}"/>
-    <hyperlink ref="A10" r:id="rId8" tooltip="Open source page" xr:uid="{316C19EA-C254-49C8-8475-B2EEF617A556}"/>
-    <hyperlink ref="A11" r:id="rId9" tooltip="Open source page" xr:uid="{1D171974-6BA1-4FE6-8803-622547C50C52}"/>
-    <hyperlink ref="A12" r:id="rId10" tooltip="Open source page" xr:uid="{A09F48AD-7D03-4E9F-BF47-1F4F9EAB8F3E}"/>
-    <hyperlink ref="A13" r:id="rId11" tooltip="Open source page" xr:uid="{CCA3DFA5-ECB1-4F55-B109-B50ADEE8537B}"/>
-  </hyperlinks>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.22" right="0.22" top="0.25" bottom="0.25" header="0" footer="0"/>
-  <pageSetup paperSize="9" scale="66" fitToHeight="4" orientation="portrait" horizontalDpi="1200" verticalDpi="1200" r:id="rId12"/>
+  <pageSetup paperSize="9" scale="66" fitToHeight="4" orientation="portrait" horizontalDpi="1200" verticalDpi="1200" r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -3743,7 +3852,7 @@
     </row>
     <row r="2" spans="1:4" ht="66">
       <c r="A2" s="42" t="s">
-        <v>123</v>
+        <v>117</v>
       </c>
       <c r="B2" s="27" t="s">
         <v>91</v>
@@ -3752,7 +3861,7 @@
         <v>92</v>
       </c>
       <c r="D2" s="28" t="s">
-        <v>124</v>
+        <v>118</v>
       </c>
     </row>
     <row r="3" spans="1:4" ht="55">
@@ -3764,7 +3873,7 @@
         <v>94</v>
       </c>
       <c r="D3" s="28" t="s">
-        <v>125</v>
+        <v>119</v>
       </c>
     </row>
     <row r="4" spans="1:4" ht="55">
@@ -3774,7 +3883,7 @@
         <v>95</v>
       </c>
       <c r="D4" s="28" t="s">
-        <v>126</v>
+        <v>120</v>
       </c>
     </row>
     <row r="5" spans="1:4" ht="44">
@@ -3784,7 +3893,7 @@
         <v>96</v>
       </c>
       <c r="D5" s="28" t="s">
-        <v>127</v>
+        <v>121</v>
       </c>
     </row>
     <row r="6" spans="1:4" ht="55">
@@ -3794,7 +3903,7 @@
         <v>97</v>
       </c>
       <c r="D6" s="28" t="s">
-        <v>128</v>
+        <v>122</v>
       </c>
     </row>
     <row r="7" spans="1:4" ht="77">
@@ -3804,7 +3913,7 @@
         <v>98</v>
       </c>
       <c r="D7" s="28" t="s">
-        <v>129</v>
+        <v>123</v>
       </c>
     </row>
     <row r="8" spans="1:4" ht="55">
@@ -3814,7 +3923,7 @@
         <v>99</v>
       </c>
       <c r="D8" s="29" t="s">
-        <v>130</v>
+        <v>124</v>
       </c>
     </row>
     <row r="9" spans="1:4" ht="66">
@@ -3824,7 +3933,7 @@
         <v>100</v>
       </c>
       <c r="D9" s="28" t="s">
-        <v>131</v>
+        <v>125</v>
       </c>
     </row>
     <row r="10" spans="1:4">
@@ -3887,7 +3996,7 @@
     </row>
     <row r="2" spans="1:4" ht="66">
       <c r="A2" s="44" t="s">
-        <v>123</v>
+        <v>117</v>
       </c>
       <c r="B2" s="31" t="s">
         <v>102</v>
@@ -3896,7 +4005,7 @@
         <v>103</v>
       </c>
       <c r="D2" s="32" t="s">
-        <v>124</v>
+        <v>118</v>
       </c>
     </row>
     <row r="3" spans="1:4" ht="55">
@@ -3908,7 +4017,7 @@
         <v>94</v>
       </c>
       <c r="D3" s="32" t="s">
-        <v>125</v>
+        <v>119</v>
       </c>
     </row>
     <row r="4" spans="1:4" ht="55">
@@ -3918,7 +4027,7 @@
         <v>95</v>
       </c>
       <c r="D4" s="32" t="s">
-        <v>126</v>
+        <v>120</v>
       </c>
     </row>
     <row r="5" spans="1:4" ht="44">
@@ -3928,7 +4037,7 @@
         <v>96</v>
       </c>
       <c r="D5" s="32" t="s">
-        <v>127</v>
+        <v>121</v>
       </c>
     </row>
     <row r="6" spans="1:4" ht="55">
@@ -3938,7 +4047,7 @@
         <v>97</v>
       </c>
       <c r="D6" s="32" t="s">
-        <v>128</v>
+        <v>122</v>
       </c>
     </row>
     <row r="7" spans="1:4" ht="77">
@@ -3948,7 +4057,7 @@
         <v>98</v>
       </c>
       <c r="D7" s="32" t="s">
-        <v>129</v>
+        <v>123</v>
       </c>
     </row>
     <row r="8" spans="1:4" ht="55">
@@ -3958,7 +4067,7 @@
         <v>99</v>
       </c>
       <c r="D8" s="33" t="s">
-        <v>130</v>
+        <v>124</v>
       </c>
     </row>
     <row r="9" spans="1:4" ht="66">
@@ -3968,12 +4077,12 @@
         <v>100</v>
       </c>
       <c r="D9" s="32" t="s">
-        <v>131</v>
+        <v>125</v>
       </c>
     </row>
     <row r="10" spans="1:4" ht="55">
       <c r="A10" s="48" t="s">
-        <v>132</v>
+        <v>126</v>
       </c>
       <c r="B10" s="46" t="s">
         <v>104</v>
@@ -3982,7 +4091,7 @@
         <v>105</v>
       </c>
       <c r="D10" s="32" t="s">
-        <v>133</v>
+        <v>127</v>
       </c>
     </row>
     <row r="11" spans="1:4" ht="55">
@@ -3992,7 +4101,7 @@
         <v>106</v>
       </c>
       <c r="D11" s="32" t="s">
-        <v>134</v>
+        <v>128</v>
       </c>
     </row>
     <row r="12" spans="1:4" ht="55">
@@ -4002,7 +4111,7 @@
         <v>107</v>
       </c>
       <c r="D12" s="32" t="s">
-        <v>135</v>
+        <v>129</v>
       </c>
     </row>
     <row r="13" spans="1:4" ht="55">
@@ -4012,7 +4121,7 @@
         <v>108</v>
       </c>
       <c r="D13" s="32" t="s">
-        <v>136</v>
+        <v>130</v>
       </c>
     </row>
     <row r="14" spans="1:4" ht="44">
@@ -4022,7 +4131,7 @@
         <v>109</v>
       </c>
       <c r="D14" s="32" t="s">
-        <v>137</v>
+        <v>131</v>
       </c>
     </row>
     <row r="15" spans="1:4" ht="44">
@@ -4032,12 +4141,12 @@
         <v>110</v>
       </c>
       <c r="D15" s="32" t="s">
-        <v>138</v>
+        <v>132</v>
       </c>
     </row>
     <row r="16" spans="1:4" ht="55">
       <c r="A16" s="50" t="s">
-        <v>139</v>
+        <v>133</v>
       </c>
       <c r="B16" s="53" t="s">
         <v>111</v>
@@ -4046,7 +4155,7 @@
         <v>112</v>
       </c>
       <c r="D16" s="32" t="s">
-        <v>140</v>
+        <v>134</v>
       </c>
     </row>
     <row r="17" spans="1:4" ht="55">
@@ -4056,7 +4165,7 @@
         <v>113</v>
       </c>
       <c r="D17" s="32" t="s">
-        <v>141</v>
+        <v>135</v>
       </c>
     </row>
     <row r="18" spans="1:4" ht="55">
@@ -4066,7 +4175,7 @@
         <v>114</v>
       </c>
       <c r="D18" s="32" t="s">
-        <v>142</v>
+        <v>136</v>
       </c>
     </row>
     <row r="19" spans="1:4" ht="44">
@@ -4076,7 +4185,7 @@
         <v>115</v>
       </c>
       <c r="D19" s="32" t="s">
-        <v>143</v>
+        <v>137</v>
       </c>
     </row>
     <row r="20" spans="1:4" ht="55">
@@ -4086,7 +4195,7 @@
         <v>116</v>
       </c>
       <c r="D20" s="28" t="s">
-        <v>144</v>
+        <v>138</v>
       </c>
     </row>
     <row r="22" spans="1:4">

</xml_diff>

<commit_message>
Link available IoT device sources
</commit_message>
<xml_diff>
--- a/assignments/assA1.xlsx
+++ b/assignments/assA1.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Desktop\Design-of-Enterprise-IoT-design\assignments\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E73FCDEB-9EEB-4551-8974-53CB18744421}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AA171DAC-D014-4459-8492-467427D420EC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="380" yWindow="380" windowWidth="19200" windowHeight="9970" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1625,7 +1625,7 @@
     <numFmt numFmtId="178" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
     <numFmt numFmtId="179" formatCode="_ &quot;￥&quot;* #,##0_ ;_ &quot;￥&quot;* \-#,##0_ ;_ &quot;￥&quot;* &quot;-&quot;_ ;_ @_ "/>
   </numFmts>
-  <fonts count="69">
+  <fonts count="70">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -2076,6 +2076,14 @@
       <family val="3"/>
       <charset val="134"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <u/>
+      <sz val="8.5"/>
+      <color rgb="FF0000FF"/>
+      <name val="Times New Roman"/>
+      <family val="1"/>
     </font>
   </fonts>
   <fills count="34">
@@ -2666,7 +2674,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="56">
+  <cellXfs count="57">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -2831,6 +2839,9 @@
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="43" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="69" fillId="0" borderId="0" xfId="6" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -3516,7 +3527,7 @@
       </c>
     </row>
     <row r="3" spans="1:7" ht="100" customHeight="1">
-      <c r="A3" s="24" t="s">
+      <c r="A3" s="56" t="s">
         <v>205</v>
       </c>
       <c r="B3" s="23" t="s">
@@ -3539,7 +3550,7 @@
       </c>
     </row>
     <row r="4" spans="1:7" ht="100" customHeight="1">
-      <c r="A4" s="24" t="s">
+      <c r="A4" s="56" t="s">
         <v>201</v>
       </c>
       <c r="B4" s="23" t="s">
@@ -3562,7 +3573,7 @@
       </c>
     </row>
     <row r="5" spans="1:7" ht="100" customHeight="1">
-      <c r="A5" s="24" t="s">
+      <c r="A5" s="56" t="s">
         <v>197</v>
       </c>
       <c r="B5" s="23" t="s">
@@ -3585,7 +3596,7 @@
       </c>
     </row>
     <row r="6" spans="1:7" ht="110" customHeight="1">
-      <c r="A6" s="24" t="s">
+      <c r="A6" s="56" t="s">
         <v>192</v>
       </c>
       <c r="B6" s="23" t="s">
@@ -3723,7 +3734,7 @@
       </c>
     </row>
     <row r="12" spans="1:7" ht="100" customHeight="1">
-      <c r="A12" s="24" t="s">
+      <c r="A12" s="56" t="s">
         <v>209</v>
       </c>
       <c r="B12" s="23" t="s">
@@ -3769,7 +3780,7 @@
       </c>
     </row>
     <row r="14" spans="1:7" ht="100" customHeight="1">
-      <c r="A14" s="24" t="s">
+      <c r="A14" s="56" t="s">
         <v>188</v>
       </c>
       <c r="B14" s="23" t="s">
@@ -3792,7 +3803,7 @@
       </c>
     </row>
     <row r="15" spans="1:7" ht="100" customHeight="1">
-      <c r="A15" s="24" t="s">
+      <c r="A15" s="56" t="s">
         <v>184</v>
       </c>
       <c r="B15" s="23" t="s">
@@ -3816,9 +3827,18 @@
     </row>
   </sheetData>
   <phoneticPr fontId="68" type="noConversion"/>
+  <hyperlinks>
+    <hyperlink ref="A15" r:id="rId1" xr:uid="{84418D51-D871-4C94-9870-6AFA83DD4A91}"/>
+    <hyperlink ref="A14" r:id="rId2" xr:uid="{CF16F0DB-1D45-4CC4-82AA-A0314723E4D3}"/>
+    <hyperlink ref="A6" r:id="rId3" xr:uid="{8AE08D63-61F9-42A8-93C5-819695F5C209}"/>
+    <hyperlink ref="A5" r:id="rId4" xr:uid="{16326222-6903-4AD6-9137-FCF35B50321E}"/>
+    <hyperlink ref="A4" r:id="rId5" xr:uid="{8D8FB6BF-E2BF-4A27-94C8-29086EEDFEE3}"/>
+    <hyperlink ref="A3" r:id="rId6" xr:uid="{ACF395AA-94F5-4329-B3F0-87B291F32422}"/>
+    <hyperlink ref="A12" r:id="rId7" xr:uid="{FC43DED9-01A1-440C-8686-5D96A702EF91}"/>
+  </hyperlinks>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.22" right="0.22" top="0.25" bottom="0.25" header="0" footer="0"/>
-  <pageSetup paperSize="9" scale="66" fitToHeight="4" orientation="portrait" horizontalDpi="1200" verticalDpi="1200" r:id="rId1"/>
+  <pageSetup paperSize="9" scale="66" fitToHeight="4" orientation="portrait" horizontalDpi="1200" verticalDpi="1200" r:id="rId8"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
Link remaining IoT device models
</commit_message>
<xml_diff>
--- a/assignments/assA1.xlsx
+++ b/assignments/assA1.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Desktop\Design-of-Enterprise-IoT-design\assignments\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AA171DAC-D014-4459-8492-467427D420EC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{277C703E-C377-4724-A86E-5288A19C66DE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="380" yWindow="380" windowWidth="19200" windowHeight="9970" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1312,307 +1312,307 @@
   </si>
   <si>
     <t>Sensor</t>
-    <phoneticPr fontId="68" type="noConversion"/>
+    <phoneticPr fontId="67" type="noConversion"/>
   </si>
   <si>
     <t>Water in each breeding tank</t>
-    <phoneticPr fontId="68" type="noConversion"/>
+    <phoneticPr fontId="67" type="noConversion"/>
   </si>
   <si>
     <t>Water temperature</t>
-    <phoneticPr fontId="68" type="noConversion"/>
+    <phoneticPr fontId="67" type="noConversion"/>
   </si>
   <si>
     <t>pH value</t>
-    <phoneticPr fontId="68" type="noConversion"/>
+    <phoneticPr fontId="67" type="noConversion"/>
   </si>
   <si>
     <t>Turbidity</t>
-    <phoneticPr fontId="68" type="noConversion"/>
+    <phoneticPr fontId="67" type="noConversion"/>
   </si>
   <si>
     <t>DFRobot Submersible Water Level Sensor (KIT0139)</t>
-    <phoneticPr fontId="68" type="noConversion"/>
+    <phoneticPr fontId="67" type="noConversion"/>
   </si>
   <si>
     <t>Water depth and level</t>
-    <phoneticPr fontId="68" type="noConversion"/>
+    <phoneticPr fontId="67" type="noConversion"/>
   </si>
   <si>
     <t>0–5 m range; ±0.5% full scale; 4–20 mA; 12–36 VDC; IP68 stainless probe. (DFRobot, n.d.)</t>
-    <phoneticPr fontId="68" type="noConversion"/>
+    <phoneticPr fontId="67" type="noConversion"/>
   </si>
   <si>
     <t>Pressure probe, vented cable termination, stilling tube, 24 VDC supply, Opta analogue input</t>
-    <phoneticPr fontId="68" type="noConversion"/>
+    <phoneticPr fontId="67" type="noConversion"/>
   </si>
   <si>
     <t>Independent level feedback prevents overflow, excessive drainage and dry-running, and verifies bounded water-change commands.</t>
-    <phoneticPr fontId="68" type="noConversion"/>
+    <phoneticPr fontId="67" type="noConversion"/>
   </si>
   <si>
     <t>DFRobot Water Flow Sensor (SEN0217 / YF-S201)</t>
-    <phoneticPr fontId="68" type="noConversion"/>
+    <phoneticPr fontId="67" type="noConversion"/>
   </si>
   <si>
     <t>Tank inlet and drain pipes</t>
-    <phoneticPr fontId="68" type="noConversion"/>
+    <phoneticPr fontId="67" type="noConversion"/>
   </si>
   <si>
     <t>Flow rate and transferred volume</t>
-    <phoneticPr fontId="68" type="noConversion"/>
+    <phoneticPr fontId="67" type="noConversion"/>
   </si>
   <si>
     <t>1–30 L/min; Hall-effect pulse output; ±5% over 2–30 L/min; 3.5–12 VDC; 1/2-inch fitting. (DFRobot, n.d.)</t>
-    <phoneticPr fontId="68" type="noConversion"/>
+    <phoneticPr fontId="67" type="noConversion"/>
   </si>
   <si>
     <t>Two sensors per tank, service unions, screened low-voltage cable, Opta pulse inputs</t>
-    <phoneticPr fontId="68" type="noConversion"/>
+    <phoneticPr fontId="67" type="noConversion"/>
   </si>
   <si>
     <t>Inlet and drain totals cross-check level change and expose blocked pipes, pump faults or stuck valves while limiting exchanged volume.</t>
-    <phoneticPr fontId="68" type="noConversion"/>
+    <phoneticPr fontId="67" type="noConversion"/>
   </si>
   <si>
     <t>DFRobot A02YYUW Waterproof Ultrasonic Sensor (SEN0311)</t>
-    <phoneticPr fontId="68" type="noConversion"/>
+    <phoneticPr fontId="67" type="noConversion"/>
   </si>
   <si>
     <t>Feed in each zone hopper</t>
-    <phoneticPr fontId="68" type="noConversion"/>
+    <phoneticPr fontId="67" type="noConversion"/>
   </si>
   <si>
     <t>Remaining feed height</t>
-    <phoneticPr fontId="68" type="noConversion"/>
+    <phoneticPr fontId="67" type="noConversion"/>
   </si>
   <si>
     <t>3–450 cm range; 3 cm blind zone; ±1 cm; 100 ms response; IP67; 3.3–5 V UART. (DFRobot, n.d.)</t>
-    <phoneticPr fontId="68" type="noConversion"/>
+    <phoneticPr fontId="67" type="noConversion"/>
   </si>
   <si>
     <t>Top mount, dust shield, isolated UART interface, hopper-specific distance-to-fill calibration</t>
-    <phoneticPr fontId="68" type="noConversion"/>
+    <phoneticPr fontId="67" type="noConversion"/>
   </si>
   <si>
     <t>One sensor per zone hopper provides a low-feed alert. Calibration accounts for the sloped pellet surface and converts distance to an approximate fill percentage.</t>
-    <phoneticPr fontId="68" type="noConversion"/>
+    <phoneticPr fontId="67" type="noConversion"/>
   </si>
   <si>
     <t>Atlas Scientific EZO Humidity Probe (EZO-HUM-P-S)</t>
-    <phoneticPr fontId="68" type="noConversion"/>
+    <phoneticPr fontId="67" type="noConversion"/>
   </si>
   <si>
     <t>Air in each breeding/nesting zone</t>
-    <phoneticPr fontId="68" type="noConversion"/>
+    <phoneticPr fontId="67" type="noConversion"/>
   </si>
   <si>
     <t>Relative humidity and air temperature</t>
-    <phoneticPr fontId="68" type="noConversion"/>
+    <phoneticPr fontId="67" type="noConversion"/>
   </si>
   <si>
     <t>0–100% RH; stated ±2% RH from 5–95%; 3.3–5 V; UART/I2C; IP67 stainless probe. (Atlas Scientific, n.d.)</t>
-    <phoneticPr fontId="68" type="noConversion"/>
+    <phoneticPr fontId="67" type="noConversion"/>
   </si>
   <si>
     <t>Shielded placement away from spray, isolated interface, mounting bracket, periodic comparison check</t>
-    <phoneticPr fontId="68" type="noConversion"/>
+    <phoneticPr fontId="67" type="noConversion"/>
   </si>
   <si>
     <t>Zone humidity reveals condensation risk that can affect electronics and camera visibility, and provides context for nesting-area observations.</t>
-    <phoneticPr fontId="68" type="noConversion"/>
+    <phoneticPr fontId="67" type="noConversion"/>
   </si>
   <si>
     <t>Aqua Medic Titanium Heater 500 W</t>
-    <phoneticPr fontId="68" type="noConversion"/>
+    <phoneticPr fontId="67" type="noConversion"/>
   </si>
   <si>
     <t>Actuator</t>
-    <phoneticPr fontId="68" type="noConversion"/>
+    <phoneticPr fontId="67" type="noConversion"/>
   </si>
   <si>
     <t>Heat input and water temperature</t>
-    <phoneticPr fontId="68" type="noConversion"/>
+    <phoneticPr fontId="67" type="noConversion"/>
   </si>
   <si>
     <t>500 W; 110–240 VAC; intended for about 1000–1500 L; external controller required. (Aqua Medic, n.d.)</t>
-    <phoneticPr fontId="68" type="noConversion"/>
+    <phoneticPr fontId="67" type="noConversion"/>
   </si>
   <si>
     <t>Titanium element, rated contactor, RCD, guarded mount, manual isolation, independent over-temperature cut-out</t>
-    <phoneticPr fontId="68" type="noConversion"/>
+    <phoneticPr fontId="67" type="noConversion"/>
   </si>
   <si>
     <t>Corrosion-resistant construction suits aquaculture. PLC control uses conservative hysteresis, while the independent cut-out remains the final safety layer.</t>
-    <phoneticPr fontId="68" type="noConversion"/>
+    <phoneticPr fontId="67" type="noConversion"/>
   </si>
   <si>
     <t>Bürkert Type 6213 EV Normally Closed Valve, 24 VDC</t>
-    <phoneticPr fontId="68" type="noConversion"/>
+    <phoneticPr fontId="67" type="noConversion"/>
   </si>
   <si>
     <t>Tank inlet and drain lines</t>
-    <phoneticPr fontId="68" type="noConversion"/>
+    <phoneticPr fontId="67" type="noConversion"/>
   </si>
   <si>
     <t>Water flow state</t>
-    <phoneticPr fontId="68" type="noConversion"/>
+    <phoneticPr fontId="67" type="noConversion"/>
   </si>
   <si>
     <t>Two-way servo-assisted diaphragm valve; normally closed; 24 VDC option; water service; IP65 with suitable plug. (Bürkert, n.d.)</t>
-    <phoneticPr fontId="68" type="noConversion"/>
+    <phoneticPr fontId="67" type="noConversion"/>
   </si>
   <si>
     <t>Two valves per tank, selected DN/pressure variant, coil suppression, manual isolation, upstream strainer</t>
-    <phoneticPr fontId="68" type="noConversion"/>
+    <phoneticPr fontId="67" type="noConversion"/>
   </si>
   <si>
     <t>Normally closed action fails safe on power loss. Paired with level and flow feedback, it enables bounded partial water exchange.</t>
-    <phoneticPr fontId="68" type="noConversion"/>
+    <phoneticPr fontId="67" type="noConversion"/>
   </si>
   <si>
     <t>Actuator / device</t>
-    <phoneticPr fontId="68" type="noConversion"/>
+    <phoneticPr fontId="67" type="noConversion"/>
   </si>
   <si>
     <t>Feed supplied to turtles in each zone</t>
-    <phoneticPr fontId="68" type="noConversion"/>
+    <phoneticPr fontId="67" type="noConversion"/>
   </si>
   <si>
     <t>Feeding time and estimated portion</t>
-    <phoneticPr fontId="68" type="noConversion"/>
+    <phoneticPr fontId="67" type="noConversion"/>
   </si>
   <si>
     <t>Turtle activity, feeding and nesting areas</t>
-    <phoneticPr fontId="68" type="noConversion"/>
+    <phoneticPr fontId="67" type="noConversion"/>
   </si>
   <si>
     <t>Video and event evidence</t>
-    <phoneticPr fontId="68" type="noConversion"/>
+    <phoneticPr fontId="67" type="noConversion"/>
   </si>
   <si>
     <t>AXIS M3086-V Network Camera</t>
-    <phoneticPr fontId="68" type="noConversion"/>
+    <phoneticPr fontId="67" type="noConversion"/>
   </si>
   <si>
     <t>4 MP maximum resolution 2688x1512; 2.4 mm F2.1 lens; 130 deg horizontal and 93 deg vertical field of view; H.264/H.265/Motion JPEG; 25/30 fps; WDR up to 120 dB; Lightfinder; PoE Class 2; IP42 and IK08.</t>
-    <phoneticPr fontId="68" type="noConversion"/>
+    <phoneticPr fontId="67" type="noConversion"/>
   </si>
   <si>
     <t>Network camera, lens, PoE RJ45 connector, SD-card slot, control button, mounting dome and managed-switch port.</t>
-    <phoneticPr fontId="68" type="noConversion"/>
+    <phoneticPr fontId="67" type="noConversion"/>
   </si>
   <si>
     <t>Video provides farm-wide context and event evidence for activity, feeding and nesting. PoE simplifies installation; edge analytics retain only validated clips rather than upload continuous video.</t>
-    <phoneticPr fontId="68" type="noConversion"/>
+    <phoneticPr fontId="67" type="noConversion"/>
   </si>
   <si>
     <t>PondMAX Solar Automatic Fish Feeder</t>
-    <phoneticPr fontId="68" type="noConversion"/>
+    <phoneticPr fontId="67" type="noConversion"/>
   </si>
   <si>
     <t>Solar charging with built-in 2200 mAh lithium battery; 1-6 feedings per day; adjustable S/M/L throw and 0-20 s feed duration; 3-10 mm food size; 12 V/1.66 A adapter specification.</t>
-    <phoneticPr fontId="68" type="noConversion"/>
+    <phoneticPr fontId="67" type="noConversion"/>
   </si>
   <si>
     <t>Solar panel, rechargeable battery, hopper, motor and spreader, timer/display controls, protective cover and mounting bracket.</t>
-    <phoneticPr fontId="68" type="noConversion"/>
+    <phoneticPr fontId="67" type="noConversion"/>
   </si>
   <si>
     <t>Automated feeding improves schedule consistency and reduces manual labour. Feed commands remain bounded by time, quantity and hopper checks, with operator override and audit records.</t>
-    <phoneticPr fontId="68" type="noConversion"/>
+    <phoneticPr fontId="67" type="noConversion"/>
   </si>
   <si>
     <t>Lonhand LH-WQS-AN-485-UI NH3-N Sensor</t>
-    <phoneticPr fontId="68" type="noConversion"/>
+    <phoneticPr fontId="67" type="noConversion"/>
   </si>
   <si>
     <t>Ammonia-nitrogen concentration</t>
-    <phoneticPr fontId="68" type="noConversion"/>
+    <phoneticPr fontId="67" type="noConversion"/>
   </si>
   <si>
     <t>Measurement range 0.1-18,000 mg/L; temperature range 0-60 deg C; 4-20 mA and RS-485 outputs; IP68; 5 m cable; NPT3/4 or M39x1.5 connection; 0-3 bar; pH 4-10; repeatability +/-4%; PC/PBT housing.</t>
-    <phoneticPr fontId="68" type="noConversion"/>
+    <phoneticPr fontId="67" type="noConversion"/>
   </si>
   <si>
     <t>Ion-selective ammonia electrode, 4-20 mA/RS-485 transmitter, 5 m cable, immersion fitting, PLC analogue/Modbus input and calibration solution.</t>
-    <phoneticPr fontId="68" type="noConversion"/>
+    <phoneticPr fontId="67" type="noConversion"/>
   </si>
   <si>
     <t>Ammonia is a high-risk water-quality condition. A wired industrial output supports continuous trend logging, local alarm thresholds and dependable response when the network is unavailable.</t>
-    <phoneticPr fontId="68" type="noConversion"/>
+    <phoneticPr fontId="67" type="noConversion"/>
   </si>
   <si>
     <t>DFRobot SEN0189 Turbidity Sensor</t>
-    <phoneticPr fontId="68" type="noConversion"/>
+    <phoneticPr fontId="67" type="noConversion"/>
   </si>
   <si>
     <t>Optical infrared emitter/receiver; 5 VDC; 40 mA maximum; response below 500 ms; selectable analogue 0-4.5 V or thresholded digital output; operating range -30 to 80 deg C; probe top is not waterproof.</t>
-    <phoneticPr fontId="68" type="noConversion"/>
+    <phoneticPr fontId="67" type="noConversion"/>
   </si>
   <si>
     <t>Optical turbidity probe, interface board, A/D or GPIO input, analogue/digital selector and threshold potentiometer.</t>
-    <phoneticPr fontId="68" type="noConversion"/>
+    <phoneticPr fontId="67" type="noConversion"/>
   </si>
   <si>
     <t>Provides early warning of suspended solids, filtration faults and contamination. Digital threshold alarms can be local, while analogue values support trend analysis and water-change decisions.</t>
-    <phoneticPr fontId="68" type="noConversion"/>
+    <phoneticPr fontId="67" type="noConversion"/>
   </si>
   <si>
     <t>DFRobot SEN0161-V2 Gravity Analog pH Meter</t>
-    <phoneticPr fontId="68" type="noConversion"/>
+    <phoneticPr fontId="67" type="noConversion"/>
   </si>
   <si>
     <t>Signal-board supply 3.3-5.5 V; analogue output 0-3.0 V; BNC electrode and PH2.0-3P signal connector; stated accuracy +/-0.1 at 25 deg C; electrode range pH 0-14 and 5-60 deg C; response below 2 min; 1 m cable.</t>
-    <phoneticPr fontId="68" type="noConversion"/>
+    <phoneticPr fontId="67" type="noConversion"/>
   </si>
   <si>
     <t>Laboratory-grade pH electrode, V2 signal-conversion board, BNC cable, PH2.0-3P lead, calibration buffers and analogue input.</t>
-    <phoneticPr fontId="68" type="noConversion"/>
+    <phoneticPr fontId="67" type="noConversion"/>
   </si>
   <si>
     <t>pH is a key water-quality variable for aquaculture. Two-point calibration and local plausibility/rate checks allow the PLC to alarm and bound corrective actions.</t>
-    <phoneticPr fontId="68" type="noConversion"/>
+    <phoneticPr fontId="67" type="noConversion"/>
   </si>
   <si>
     <t>DFRobot Waterproof DS18B20 Temperature Sensor (BOS0042)</t>
-    <phoneticPr fontId="68" type="noConversion"/>
+    <phoneticPr fontId="67" type="noConversion"/>
   </si>
   <si>
     <t>Waterproof DS18B20 probe; 3-5 V; PH2.0-3P connector; sensing range -55 to 125 deg C; display range -10 to 85 deg C; stated error +/-0.5 deg C; pull-up resistor required.</t>
-    <phoneticPr fontId="68" type="noConversion"/>
+    <phoneticPr fontId="67" type="noConversion"/>
   </si>
   <si>
     <t>Waterproof DS18B20 probe, 3-pin cable, pull-up resistor, PH2.0 adapter and controller input.</t>
-    <phoneticPr fontId="68" type="noConversion"/>
+    <phoneticPr fontId="67" type="noConversion"/>
   </si>
   <si>
     <t>Direct temperature feedback supports heater control and alarm limits in wet tanks. The sealed probe suits remote or humid measurement, while local validation prevents unsafe heating commands.</t>
-    <phoneticPr fontId="68" type="noConversion"/>
+    <phoneticPr fontId="67" type="noConversion"/>
   </si>
   <si>
     <t>Bluefish MINI-200 Submersible Pump</t>
-    <phoneticPr fontId="68" type="noConversion"/>
+    <phoneticPr fontId="67" type="noConversion"/>
   </si>
   <si>
     <t>Tank recirculation and water-change line</t>
-    <phoneticPr fontId="68" type="noConversion"/>
+    <phoneticPr fontId="67" type="noConversion"/>
   </si>
   <si>
     <t>Water circulation and flow</t>
-    <phoneticPr fontId="68" type="noConversion"/>
+    <phoneticPr fontId="67" type="noConversion"/>
   </si>
   <si>
     <t>12 VDC; 0.4 A; 4.8 W; 200 L/h open flow; 1.5 m maximum head; brushless motor; IP68 submersible construction; approximately 43x38x30 mm; below 35 dB; dry-run/block protection options.</t>
-    <phoneticPr fontId="68" type="noConversion"/>
+    <phoneticPr fontId="67" type="noConversion"/>
   </si>
   <si>
     <t>Brushless pump, impeller, inlet/outlet, sealed motor, silicone vibration feet, 12 V supply, relay/MOSFET driver and flow feedback.</t>
-    <phoneticPr fontId="68" type="noConversion"/>
+    <phoneticPr fontId="67" type="noConversion"/>
   </si>
   <si>
     <t>Low-voltage circulation supports filtration and controlled water changes. A relay, flow confirmation and dry-run protection prevent a blocked line or empty tank from damaging the pump.</t>
-    <phoneticPr fontId="68" type="noConversion"/>
+    <phoneticPr fontId="67" type="noConversion"/>
   </si>
 </sst>
 </file>
@@ -1625,7 +1625,7 @@
     <numFmt numFmtId="178" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
     <numFmt numFmtId="179" formatCode="_ &quot;￥&quot;* #,##0_ ;_ &quot;￥&quot;* \-#,##0_ ;_ &quot;￥&quot;* &quot;-&quot;_ ;_ @_ "/>
   </numFmts>
-  <fonts count="70">
+  <fonts count="69">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1866,13 +1866,6 @@
       <family val="1"/>
     </font>
     <font>
-      <sz val="8.5"/>
-      <color indexed="64"/>
-      <name val="Times New Roman"/>
-      <family val="1"/>
-    </font>
-    <font>
-      <b/>
       <sz val="8.5"/>
       <color indexed="64"/>
       <name val="Times New Roman"/>
@@ -2529,19 +2522,19 @@
   </borders>
   <cellStyleXfs count="49">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="176" fontId="46" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="177" fontId="46" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="46" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="178" fontId="46" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="179" fontId="46" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyProtection="0">
+    <xf numFmtId="176" fontId="45" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="177" fontId="45" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="45" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="178" fontId="45" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="179" fontId="45" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyProtection="0">
@@ -2550,7 +2543,7 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="46" fillId="2" borderId="1" applyNumberFormat="0" applyFont="0" applyProtection="0">
+    <xf numFmtId="0" fontId="45" fillId="2" borderId="1" applyNumberFormat="0" applyFont="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyProtection="0">
@@ -2604,10 +2597,10 @@
     <xf numFmtId="0" fontId="18" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="46" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="46" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyProtection="0">
+    <xf numFmtId="0" fontId="45" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="45" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="18" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyProtection="0">
@@ -2616,10 +2609,10 @@
     <xf numFmtId="0" fontId="18" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="46" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="46" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyProtection="0">
+    <xf numFmtId="0" fontId="45" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="45" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="18" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyProtection="0">
@@ -2628,10 +2621,10 @@
     <xf numFmtId="0" fontId="18" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="46" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="46" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyProtection="0">
+    <xf numFmtId="0" fontId="45" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="45" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="18" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyProtection="0">
@@ -2640,10 +2633,10 @@
     <xf numFmtId="0" fontId="18" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="46" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="46" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyProtection="0">
+    <xf numFmtId="0" fontId="45" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="45" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="18" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyProtection="0">
@@ -2652,10 +2645,10 @@
     <xf numFmtId="0" fontId="18" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="46" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="46" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyProtection="0">
+    <xf numFmtId="0" fontId="45" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="45" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="18" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyProtection="0">
@@ -2664,10 +2657,10 @@
     <xf numFmtId="0" fontId="18" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="46" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="46" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyProtection="0">
+    <xf numFmtId="0" fontId="45" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="45" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="18" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyProtection="0">
@@ -2745,41 +2738,41 @@
     <xf numFmtId="0" fontId="38" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="39" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    <xf numFmtId="0" fontId="39" fillId="33" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="40" fillId="33" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="41" fillId="33" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    <xf numFmtId="0" fontId="42" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="41" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="43" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="44" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="42" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="41" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="43" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="42" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="44" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="44" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="45" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="68" fillId="0" borderId="0" xfId="6" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="43" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="42" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="44" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="43" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="45" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="19" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
@@ -2799,49 +2792,49 @@
     <xf numFmtId="0" fontId="28" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="41" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="42" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="43" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="41" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="41" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="42" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="42" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="41" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="41" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="41" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="42" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="41" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="43" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="41" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="42" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="43" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="42" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="42" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="42" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="42" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="42" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="42" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="43" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="43" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="43" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="69" fillId="0" borderId="0" xfId="6" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="68" fillId="0" borderId="17" xfId="6" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -3273,7 +3266,7 @@
     <mergeCell ref="A1:B1"/>
     <mergeCell ref="A2:B2"/>
   </mergeCells>
-  <phoneticPr fontId="68" type="noConversion"/>
+  <phoneticPr fontId="67" type="noConversion"/>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.22" right="0.22" top="0.25" bottom="0.25" header="0" footer="0"/>
   <pageSetup paperSize="9" scale="77" fitToHeight="2" orientation="portrait" horizontalDpi="1200" verticalDpi="1200" r:id="rId1"/>
@@ -3456,7 +3449,7 @@
     <mergeCell ref="A1:B1"/>
     <mergeCell ref="A2:B2"/>
   </mergeCells>
-  <phoneticPr fontId="68" type="noConversion"/>
+  <phoneticPr fontId="67" type="noConversion"/>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.22" right="0.22" top="0.25" bottom="0.25" header="0" footer="0"/>
   <pageSetup paperSize="9" scale="67" fitToHeight="2" orientation="portrait" horizontalDpi="1200" verticalDpi="1200" r:id="rId1"/>
@@ -3481,53 +3474,53 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7">
-      <c r="A1" s="25" t="s">
+      <c r="A1" s="24" t="s">
         <v>73</v>
       </c>
-      <c r="B1" s="25" t="s">
+      <c r="B1" s="24" t="s">
         <v>74</v>
       </c>
-      <c r="C1" s="25" t="s">
+      <c r="C1" s="24" t="s">
         <v>75</v>
       </c>
-      <c r="D1" s="25" t="s">
+      <c r="D1" s="24" t="s">
         <v>76</v>
       </c>
-      <c r="E1" s="25" t="s">
+      <c r="E1" s="24" t="s">
         <v>77</v>
       </c>
-      <c r="F1" s="25" t="s">
+      <c r="F1" s="24" t="s">
         <v>78</v>
       </c>
-      <c r="G1" s="25" t="s">
+      <c r="G1" s="24" t="s">
         <v>79</v>
       </c>
     </row>
     <row r="2" spans="1:7" ht="48">
-      <c r="A2" s="26" t="s">
+      <c r="A2" s="25" t="s">
         <v>80</v>
       </c>
-      <c r="B2" s="26" t="s">
+      <c r="B2" s="25" t="s">
         <v>81</v>
       </c>
-      <c r="C2" s="26" t="s">
+      <c r="C2" s="25" t="s">
         <v>82</v>
       </c>
-      <c r="D2" s="26" t="s">
+      <c r="D2" s="25" t="s">
         <v>83</v>
       </c>
-      <c r="E2" s="26" t="s">
+      <c r="E2" s="25" t="s">
         <v>84</v>
       </c>
-      <c r="F2" s="26" t="s">
+      <c r="F2" s="25" t="s">
         <v>85</v>
       </c>
-      <c r="G2" s="26" t="s">
+      <c r="G2" s="25" t="s">
         <v>86</v>
       </c>
     </row>
     <row r="3" spans="1:7" ht="100" customHeight="1">
-      <c r="A3" s="56" t="s">
+      <c r="A3" s="35" t="s">
         <v>205</v>
       </c>
       <c r="B3" s="23" t="s">
@@ -3550,7 +3543,7 @@
       </c>
     </row>
     <row r="4" spans="1:7" ht="100" customHeight="1">
-      <c r="A4" s="56" t="s">
+      <c r="A4" s="35" t="s">
         <v>201</v>
       </c>
       <c r="B4" s="23" t="s">
@@ -3573,7 +3566,7 @@
       </c>
     </row>
     <row r="5" spans="1:7" ht="100" customHeight="1">
-      <c r="A5" s="56" t="s">
+      <c r="A5" s="35" t="s">
         <v>197</v>
       </c>
       <c r="B5" s="23" t="s">
@@ -3596,7 +3589,7 @@
       </c>
     </row>
     <row r="6" spans="1:7" ht="110" customHeight="1">
-      <c r="A6" s="56" t="s">
+      <c r="A6" s="35" t="s">
         <v>192</v>
       </c>
       <c r="B6" s="23" t="s">
@@ -3619,7 +3612,7 @@
       </c>
     </row>
     <row r="7" spans="1:7" ht="75" customHeight="1">
-      <c r="A7" s="24" t="s">
+      <c r="A7" s="56" t="s">
         <v>144</v>
       </c>
       <c r="B7" s="23" t="s">
@@ -3642,7 +3635,7 @@
       </c>
     </row>
     <row r="8" spans="1:7" ht="75" customHeight="1">
-      <c r="A8" s="24" t="s">
+      <c r="A8" s="56" t="s">
         <v>149</v>
       </c>
       <c r="B8" s="23" t="s">
@@ -3665,7 +3658,7 @@
       </c>
     </row>
     <row r="9" spans="1:7" ht="85" customHeight="1">
-      <c r="A9" s="24" t="s">
+      <c r="A9" s="56" t="s">
         <v>155</v>
       </c>
       <c r="B9" s="23" t="s">
@@ -3688,7 +3681,7 @@
       </c>
     </row>
     <row r="10" spans="1:7" ht="85" customHeight="1">
-      <c r="A10" s="24" t="s">
+      <c r="A10" s="56" t="s">
         <v>161</v>
       </c>
       <c r="B10" s="23" t="s">
@@ -3711,7 +3704,7 @@
       </c>
     </row>
     <row r="11" spans="1:7" ht="75" customHeight="1">
-      <c r="A11" s="24" t="s">
+      <c r="A11" s="56" t="s">
         <v>167</v>
       </c>
       <c r="B11" s="23" t="s">
@@ -3734,7 +3727,7 @@
       </c>
     </row>
     <row r="12" spans="1:7" ht="100" customHeight="1">
-      <c r="A12" s="56" t="s">
+      <c r="A12" s="35" t="s">
         <v>209</v>
       </c>
       <c r="B12" s="23" t="s">
@@ -3757,7 +3750,7 @@
       </c>
     </row>
     <row r="13" spans="1:7" ht="75" customHeight="1">
-      <c r="A13" s="24" t="s">
+      <c r="A13" s="56" t="s">
         <v>173</v>
       </c>
       <c r="B13" s="23" t="s">
@@ -3780,7 +3773,7 @@
       </c>
     </row>
     <row r="14" spans="1:7" ht="100" customHeight="1">
-      <c r="A14" s="56" t="s">
+      <c r="A14" s="35" t="s">
         <v>188</v>
       </c>
       <c r="B14" s="23" t="s">
@@ -3803,7 +3796,7 @@
       </c>
     </row>
     <row r="15" spans="1:7" ht="100" customHeight="1">
-      <c r="A15" s="56" t="s">
+      <c r="A15" s="35" t="s">
         <v>184</v>
       </c>
       <c r="B15" s="23" t="s">
@@ -3826,19 +3819,25 @@
       </c>
     </row>
   </sheetData>
-  <phoneticPr fontId="68" type="noConversion"/>
+  <phoneticPr fontId="67" type="noConversion"/>
   <hyperlinks>
-    <hyperlink ref="A15" r:id="rId1" xr:uid="{84418D51-D871-4C94-9870-6AFA83DD4A91}"/>
-    <hyperlink ref="A14" r:id="rId2" xr:uid="{CF16F0DB-1D45-4CC4-82AA-A0314723E4D3}"/>
-    <hyperlink ref="A6" r:id="rId3" xr:uid="{8AE08D63-61F9-42A8-93C5-819695F5C209}"/>
-    <hyperlink ref="A5" r:id="rId4" xr:uid="{16326222-6903-4AD6-9137-FCF35B50321E}"/>
-    <hyperlink ref="A4" r:id="rId5" xr:uid="{8D8FB6BF-E2BF-4A27-94C8-29086EEDFEE3}"/>
-    <hyperlink ref="A3" r:id="rId6" xr:uid="{ACF395AA-94F5-4329-B3F0-87B291F32422}"/>
-    <hyperlink ref="A12" r:id="rId7" xr:uid="{FC43DED9-01A1-440C-8686-5D96A702EF91}"/>
+    <hyperlink ref="A15" r:id="rId1" xr:uid="{807C2E75-D0C4-462C-A467-7BC0351D30B2}"/>
+    <hyperlink ref="A14" r:id="rId2" xr:uid="{101AA2DF-FB6B-4EC5-A28B-6F2ECD66DF5F}"/>
+    <hyperlink ref="A13" r:id="rId3" xr:uid="{F6E07958-2FB6-47A7-9E06-CB72C2FC57E5}"/>
+    <hyperlink ref="A12" r:id="rId4" xr:uid="{EFFD57F2-42E5-4B4F-BEBF-3463B134944B}"/>
+    <hyperlink ref="A11" r:id="rId5" xr:uid="{7566F753-951B-4455-910C-C31FCFF28742}"/>
+    <hyperlink ref="A10" r:id="rId6" xr:uid="{E91EF359-6E4E-42D9-BDA8-DCADD28EB08D}"/>
+    <hyperlink ref="A9" r:id="rId7" xr:uid="{237E20BD-1D7A-4B5B-82AC-16B726C535BB}"/>
+    <hyperlink ref="A8" r:id="rId8" xr:uid="{331A737F-11F5-4073-A1C7-E39059390C86}"/>
+    <hyperlink ref="A7" r:id="rId9" xr:uid="{E7300E1D-5483-4665-A98A-A4EAF5D9AF86}"/>
+    <hyperlink ref="A6" r:id="rId10" xr:uid="{AF888DFA-DE59-4D73-B1C8-1DE834E2C45C}"/>
+    <hyperlink ref="A5" r:id="rId11" xr:uid="{93588D19-58EB-4089-BF98-EF66A5001FF7}"/>
+    <hyperlink ref="A4" r:id="rId12" xr:uid="{EC10C21B-AA0A-4D3C-AA81-108B84D0C940}"/>
+    <hyperlink ref="A3" r:id="rId13" xr:uid="{C87C25A7-FADA-42C8-ADC0-91860DB5797A}"/>
   </hyperlinks>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.22" right="0.22" top="0.25" bottom="0.25" header="0" footer="0"/>
-  <pageSetup paperSize="9" scale="66" fitToHeight="4" orientation="portrait" horizontalDpi="1200" verticalDpi="1200" r:id="rId8"/>
+  <pageSetup paperSize="9" scale="66" fitToHeight="4" orientation="portrait" horizontalDpi="1200" verticalDpi="1200" r:id="rId14"/>
 </worksheet>
 </file>
 
@@ -3857,16 +3856,16 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="23">
-      <c r="A1" s="30" t="s">
+      <c r="A1" s="29" t="s">
         <v>87</v>
       </c>
-      <c r="B1" s="30" t="s">
+      <c r="B1" s="29" t="s">
         <v>88</v>
       </c>
-      <c r="C1" s="30" t="s">
+      <c r="C1" s="29" t="s">
         <v>89</v>
       </c>
-      <c r="D1" s="30" t="s">
+      <c r="D1" s="29" t="s">
         <v>90</v>
       </c>
     </row>
@@ -3874,13 +3873,13 @@
       <c r="A2" s="42" t="s">
         <v>117</v>
       </c>
-      <c r="B2" s="27" t="s">
+      <c r="B2" s="26" t="s">
         <v>91</v>
       </c>
-      <c r="C2" s="27" t="s">
+      <c r="C2" s="26" t="s">
         <v>92</v>
       </c>
-      <c r="D2" s="28" t="s">
+      <c r="D2" s="27" t="s">
         <v>118</v>
       </c>
     </row>
@@ -3889,70 +3888,70 @@
       <c r="B3" s="43" t="s">
         <v>93</v>
       </c>
-      <c r="C3" s="27" t="s">
+      <c r="C3" s="26" t="s">
         <v>94</v>
       </c>
-      <c r="D3" s="28" t="s">
+      <c r="D3" s="27" t="s">
         <v>119</v>
       </c>
     </row>
     <row r="4" spans="1:4" ht="55">
       <c r="A4" s="42"/>
       <c r="B4" s="43"/>
-      <c r="C4" s="27" t="s">
+      <c r="C4" s="26" t="s">
         <v>95</v>
       </c>
-      <c r="D4" s="28" t="s">
+      <c r="D4" s="27" t="s">
         <v>120</v>
       </c>
     </row>
     <row r="5" spans="1:4" ht="44">
       <c r="A5" s="42"/>
       <c r="B5" s="43"/>
-      <c r="C5" s="27" t="s">
+      <c r="C5" s="26" t="s">
         <v>96</v>
       </c>
-      <c r="D5" s="28" t="s">
+      <c r="D5" s="27" t="s">
         <v>121</v>
       </c>
     </row>
     <row r="6" spans="1:4" ht="55">
       <c r="A6" s="42"/>
       <c r="B6" s="43"/>
-      <c r="C6" s="27" t="s">
+      <c r="C6" s="26" t="s">
         <v>97</v>
       </c>
-      <c r="D6" s="28" t="s">
+      <c r="D6" s="27" t="s">
         <v>122</v>
       </c>
     </row>
     <row r="7" spans="1:4" ht="77">
       <c r="A7" s="42"/>
       <c r="B7" s="43"/>
-      <c r="C7" s="27" t="s">
+      <c r="C7" s="26" t="s">
         <v>98</v>
       </c>
-      <c r="D7" s="28" t="s">
+      <c r="D7" s="27" t="s">
         <v>123</v>
       </c>
     </row>
     <row r="8" spans="1:4" ht="55">
       <c r="A8" s="42"/>
       <c r="B8" s="43"/>
-      <c r="C8" s="27" t="s">
+      <c r="C8" s="26" t="s">
         <v>99</v>
       </c>
-      <c r="D8" s="29" t="s">
+      <c r="D8" s="28" t="s">
         <v>124</v>
       </c>
     </row>
     <row r="9" spans="1:4" ht="66">
       <c r="A9" s="42"/>
       <c r="B9" s="43"/>
-      <c r="C9" s="27" t="s">
+      <c r="C9" s="26" t="s">
         <v>100</v>
       </c>
-      <c r="D9" s="28" t="s">
+      <c r="D9" s="27" t="s">
         <v>125</v>
       </c>
     </row>
@@ -3979,7 +3978,7 @@
     <mergeCell ref="A2:A9"/>
     <mergeCell ref="B3:B9"/>
   </mergeCells>
-  <phoneticPr fontId="68" type="noConversion"/>
+  <phoneticPr fontId="67" type="noConversion"/>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.22" right="0.22" top="0.25" bottom="0.25" header="0" footer="0"/>
   <pageSetup paperSize="9" scale="67" fitToHeight="2" orientation="portrait" horizontalDpi="1200" verticalDpi="1200" r:id="rId1"/>
@@ -4001,16 +4000,16 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="46">
-      <c r="A1" s="35" t="s">
+      <c r="A1" s="34" t="s">
         <v>101</v>
       </c>
-      <c r="B1" s="35" t="s">
+      <c r="B1" s="34" t="s">
         <v>88</v>
       </c>
-      <c r="C1" s="35" t="s">
+      <c r="C1" s="34" t="s">
         <v>89</v>
       </c>
-      <c r="D1" s="35" t="s">
+      <c r="D1" s="34" t="s">
         <v>90</v>
       </c>
     </row>
@@ -4018,13 +4017,13 @@
       <c r="A2" s="44" t="s">
         <v>117</v>
       </c>
-      <c r="B2" s="31" t="s">
+      <c r="B2" s="30" t="s">
         <v>102</v>
       </c>
-      <c r="C2" s="31" t="s">
+      <c r="C2" s="30" t="s">
         <v>103</v>
       </c>
-      <c r="D2" s="32" t="s">
+      <c r="D2" s="31" t="s">
         <v>118</v>
       </c>
     </row>
@@ -4033,70 +4032,70 @@
       <c r="B3" s="46" t="s">
         <v>93</v>
       </c>
-      <c r="C3" s="31" t="s">
+      <c r="C3" s="30" t="s">
         <v>94</v>
       </c>
-      <c r="D3" s="32" t="s">
+      <c r="D3" s="31" t="s">
         <v>119</v>
       </c>
     </row>
     <row r="4" spans="1:4" ht="55">
       <c r="A4" s="45"/>
       <c r="B4" s="47"/>
-      <c r="C4" s="31" t="s">
+      <c r="C4" s="30" t="s">
         <v>95</v>
       </c>
-      <c r="D4" s="32" t="s">
+      <c r="D4" s="31" t="s">
         <v>120</v>
       </c>
     </row>
     <row r="5" spans="1:4" ht="44">
       <c r="A5" s="45"/>
       <c r="B5" s="47"/>
-      <c r="C5" s="31" t="s">
+      <c r="C5" s="30" t="s">
         <v>96</v>
       </c>
-      <c r="D5" s="32" t="s">
+      <c r="D5" s="31" t="s">
         <v>121</v>
       </c>
     </row>
     <row r="6" spans="1:4" ht="55">
       <c r="A6" s="45"/>
       <c r="B6" s="47"/>
-      <c r="C6" s="31" t="s">
+      <c r="C6" s="30" t="s">
         <v>97</v>
       </c>
-      <c r="D6" s="32" t="s">
+      <c r="D6" s="31" t="s">
         <v>122</v>
       </c>
     </row>
     <row r="7" spans="1:4" ht="77">
       <c r="A7" s="45"/>
       <c r="B7" s="47"/>
-      <c r="C7" s="31" t="s">
+      <c r="C7" s="30" t="s">
         <v>98</v>
       </c>
-      <c r="D7" s="32" t="s">
+      <c r="D7" s="31" t="s">
         <v>123</v>
       </c>
     </row>
     <row r="8" spans="1:4" ht="55">
       <c r="A8" s="45"/>
       <c r="B8" s="47"/>
-      <c r="C8" s="31" t="s">
+      <c r="C8" s="30" t="s">
         <v>99</v>
       </c>
-      <c r="D8" s="33" t="s">
+      <c r="D8" s="32" t="s">
         <v>124</v>
       </c>
     </row>
     <row r="9" spans="1:4" ht="66">
       <c r="A9" s="45"/>
       <c r="B9" s="47"/>
-      <c r="C9" s="31" t="s">
+      <c r="C9" s="30" t="s">
         <v>100</v>
       </c>
-      <c r="D9" s="32" t="s">
+      <c r="D9" s="31" t="s">
         <v>125</v>
       </c>
     </row>
@@ -4107,60 +4106,60 @@
       <c r="B10" s="46" t="s">
         <v>104</v>
       </c>
-      <c r="C10" s="31" t="s">
+      <c r="C10" s="30" t="s">
         <v>105</v>
       </c>
-      <c r="D10" s="32" t="s">
+      <c r="D10" s="31" t="s">
         <v>127</v>
       </c>
     </row>
     <row r="11" spans="1:4" ht="55">
       <c r="A11" s="49"/>
       <c r="B11" s="47"/>
-      <c r="C11" s="31" t="s">
+      <c r="C11" s="30" t="s">
         <v>106</v>
       </c>
-      <c r="D11" s="32" t="s">
+      <c r="D11" s="31" t="s">
         <v>128</v>
       </c>
     </row>
     <row r="12" spans="1:4" ht="55">
       <c r="A12" s="49"/>
       <c r="B12" s="47"/>
-      <c r="C12" s="31" t="s">
+      <c r="C12" s="30" t="s">
         <v>107</v>
       </c>
-      <c r="D12" s="32" t="s">
+      <c r="D12" s="31" t="s">
         <v>129</v>
       </c>
     </row>
     <row r="13" spans="1:4" ht="55">
       <c r="A13" s="49"/>
       <c r="B13" s="47"/>
-      <c r="C13" s="31" t="s">
+      <c r="C13" s="30" t="s">
         <v>108</v>
       </c>
-      <c r="D13" s="32" t="s">
+      <c r="D13" s="31" t="s">
         <v>130</v>
       </c>
     </row>
     <row r="14" spans="1:4" ht="44">
       <c r="A14" s="49"/>
       <c r="B14" s="47"/>
-      <c r="C14" s="31" t="s">
+      <c r="C14" s="30" t="s">
         <v>109</v>
       </c>
-      <c r="D14" s="32" t="s">
+      <c r="D14" s="31" t="s">
         <v>131</v>
       </c>
     </row>
     <row r="15" spans="1:4" ht="44">
       <c r="A15" s="49"/>
       <c r="B15" s="47"/>
-      <c r="C15" s="31" t="s">
+      <c r="C15" s="30" t="s">
         <v>110</v>
       </c>
-      <c r="D15" s="32" t="s">
+      <c r="D15" s="31" t="s">
         <v>132</v>
       </c>
     </row>
@@ -4171,50 +4170,50 @@
       <c r="B16" s="53" t="s">
         <v>111</v>
       </c>
-      <c r="C16" s="31" t="s">
+      <c r="C16" s="30" t="s">
         <v>112</v>
       </c>
-      <c r="D16" s="32" t="s">
+      <c r="D16" s="31" t="s">
         <v>134</v>
       </c>
     </row>
     <row r="17" spans="1:4" ht="55">
       <c r="A17" s="51"/>
       <c r="B17" s="54"/>
-      <c r="C17" s="31" t="s">
+      <c r="C17" s="30" t="s">
         <v>113</v>
       </c>
-      <c r="D17" s="32" t="s">
+      <c r="D17" s="31" t="s">
         <v>135</v>
       </c>
     </row>
     <row r="18" spans="1:4" ht="55">
       <c r="A18" s="51"/>
       <c r="B18" s="54"/>
-      <c r="C18" s="31" t="s">
+      <c r="C18" s="30" t="s">
         <v>114</v>
       </c>
-      <c r="D18" s="32" t="s">
+      <c r="D18" s="31" t="s">
         <v>136</v>
       </c>
     </row>
     <row r="19" spans="1:4" ht="44">
       <c r="A19" s="51"/>
       <c r="B19" s="54"/>
-      <c r="C19" s="31" t="s">
+      <c r="C19" s="30" t="s">
         <v>115</v>
       </c>
-      <c r="D19" s="32" t="s">
+      <c r="D19" s="31" t="s">
         <v>137</v>
       </c>
     </row>
     <row r="20" spans="1:4" ht="55">
       <c r="A20" s="52"/>
       <c r="B20" s="55"/>
-      <c r="C20" s="34" t="s">
+      <c r="C20" s="33" t="s">
         <v>116</v>
       </c>
-      <c r="D20" s="28" t="s">
+      <c r="D20" s="27" t="s">
         <v>138</v>
       </c>
     </row>
@@ -4247,7 +4246,7 @@
     <mergeCell ref="A16:A20"/>
     <mergeCell ref="B16:B20"/>
   </mergeCells>
-  <phoneticPr fontId="68" type="noConversion"/>
+  <phoneticPr fontId="67" type="noConversion"/>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.22" right="0.22" top="0.25" bottom="0.25" header="0" footer="0"/>
   <pageSetup paperSize="9" scale="67" orientation="portrait" horizontalDpi="1200" verticalDpi="1200" r:id="rId1"/>

</xml_diff>